<commit_message>
#4 Client BOM Updated.
</commit_message>
<xml_diff>
--- a/Design Files/LightSPT-Device-v1.0/BOM/Client_BOM_Light_spt_device.xlsx
+++ b/Design Files/LightSPT-Device-v1.0/BOM/Client_BOM_Light_spt_device.xlsx
@@ -5,7 +5,7 @@
   <workbookPr codeName="ThisWorkbook" defaultThemeVersion="153222"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\eSpark-Consultants\chrisbyrd-lightsptdevice\Design Files\Light_spt_device\BOM\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\eSpark-Consultants\chrisbyrd-lightsptdevice\Design Files\LightSPT-Device-v1.0\BOM\"/>
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
@@ -19,7 +19,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="637" uniqueCount="323">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="637" uniqueCount="324">
   <si>
     <t>Component list</t>
   </si>
@@ -66,9 +66,6 @@
     <t>Pogo Connector</t>
   </si>
   <si>
-    <t>SMA</t>
-  </si>
-  <si>
     <t>SIM Card Connectors</t>
   </si>
   <si>
@@ -378,9 +375,6 @@
     <t>Pogo Pad 2.5mm 4 Pin</t>
   </si>
   <si>
-    <t>1 Inner bore SMA Board Edge Bend -55℃~+155℃ 50Ω Plugin RF Connectors / Coaxial Connectors ROHS</t>
-  </si>
-  <si>
     <t>Copper Alloy Self bomb Gold plating 1.25mm Deck -40℃~+85℃ 260℃ NanoSIM SMD SIM Card Connectors ROHS</t>
   </si>
   <si>
@@ -669,9 +663,6 @@
     <t>POGO Connector 4 Pin</t>
   </si>
   <si>
-    <t>HJ-SMA508</t>
-  </si>
-  <si>
     <t>SLF10145T-100M2R5-PF</t>
   </si>
   <si>
@@ -819,9 +810,6 @@
     <t>BOOMELE</t>
   </si>
   <si>
-    <t>HJ Tech</t>
-  </si>
-  <si>
     <t>XKB Connectivity</t>
   </si>
   <si>
@@ -988,6 +976,21 @@
   </si>
   <si>
     <t>Custom Supplier</t>
+  </si>
+  <si>
+    <t>SMA Connector</t>
+  </si>
+  <si>
+    <t>Sma Female Connector, Pcb Edge Mount Rohs Compliant: Yes</t>
+  </si>
+  <si>
+    <t>CON-SMA-EDGE_S</t>
+  </si>
+  <si>
+    <t>CON-SMA-EDGE-S</t>
+  </si>
+  <si>
+    <t>RF Solutions</t>
   </si>
 </sst>
 </file>
@@ -1559,15 +1562,6 @@
     <xf numFmtId="0" fontId="10" fillId="3" borderId="5" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="10" fillId="4" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -1708,6 +1702,15 @@
     </xf>
     <xf numFmtId="0" fontId="21" fillId="0" borderId="16" xfId="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -2081,13 +2084,13 @@
       <c r="G1" s="2"/>
       <c r="H1" s="2"/>
       <c r="I1" s="2"/>
-      <c r="J1" s="46"/>
-      <c r="K1" s="46"/>
-      <c r="L1" s="46"/>
-      <c r="M1" s="46"/>
-      <c r="N1" s="46"/>
-      <c r="O1" s="46"/>
-      <c r="P1" s="46"/>
+      <c r="J1" s="92"/>
+      <c r="K1" s="92"/>
+      <c r="L1" s="92"/>
+      <c r="M1" s="92"/>
+      <c r="N1" s="92"/>
+      <c r="O1" s="92"/>
+      <c r="P1" s="92"/>
     </row>
     <row r="2" spans="1:16" ht="32.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A2" s="1"/>
@@ -2098,7 +2101,7 @@
       </c>
       <c r="E2" s="10"/>
       <c r="F2" s="42" t="s">
-        <v>309</v>
+        <v>305</v>
       </c>
       <c r="G2" s="11"/>
       <c r="H2" s="11"/>
@@ -2106,7 +2109,7 @@
       <c r="J2" s="3"/>
       <c r="K2" s="3"/>
       <c r="L2" s="3"/>
-      <c r="M2" s="86"/>
+      <c r="M2" s="83"/>
       <c r="N2" s="3"/>
       <c r="O2" s="3"/>
       <c r="P2" s="32"/>
@@ -2120,7 +2123,7 @@
       </c>
       <c r="E3" s="12"/>
       <c r="F3" s="43" t="s">
-        <v>310</v>
+        <v>306</v>
       </c>
       <c r="G3" s="12"/>
       <c r="H3" s="12"/>
@@ -2128,10 +2131,10 @@
       <c r="J3" s="4"/>
       <c r="K3" s="4"/>
       <c r="L3" s="4"/>
-      <c r="M3" s="87"/>
+      <c r="M3" s="84"/>
       <c r="N3" s="4"/>
       <c r="O3" s="4"/>
-      <c r="P3" s="47"/>
+      <c r="P3" s="93"/>
     </row>
     <row r="4" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A4" s="1"/>
@@ -2142,7 +2145,7 @@
       </c>
       <c r="E4" s="12"/>
       <c r="F4" s="44" t="s">
-        <v>310</v>
+        <v>306</v>
       </c>
       <c r="G4" s="13"/>
       <c r="H4" s="13"/>
@@ -2150,10 +2153,10 @@
       <c r="J4" s="6"/>
       <c r="K4" s="6"/>
       <c r="L4" s="6"/>
-      <c r="M4" s="88"/>
+      <c r="M4" s="85"/>
       <c r="N4" s="5"/>
       <c r="O4" s="5"/>
-      <c r="P4" s="48"/>
+      <c r="P4" s="94"/>
     </row>
     <row r="5" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A5" s="1"/>
@@ -2172,10 +2175,10 @@
       <c r="J5" s="5"/>
       <c r="K5" s="5"/>
       <c r="L5" s="5"/>
-      <c r="M5" s="88"/>
+      <c r="M5" s="85"/>
       <c r="N5" s="5"/>
       <c r="O5" s="5"/>
-      <c r="P5" s="48"/>
+      <c r="P5" s="94"/>
     </row>
     <row r="6" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A6" s="1"/>
@@ -2190,10 +2193,10 @@
       <c r="J6" s="5"/>
       <c r="K6" s="5"/>
       <c r="L6" s="5"/>
-      <c r="M6" s="88"/>
+      <c r="M6" s="85"/>
       <c r="N6" s="5"/>
       <c r="O6" s="5"/>
-      <c r="P6" s="48"/>
+      <c r="P6" s="94"/>
     </row>
     <row r="7" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A7" s="1"/>
@@ -2208,10 +2211,10 @@
       <c r="J7" s="7"/>
       <c r="K7" s="7"/>
       <c r="L7" s="7"/>
-      <c r="M7" s="89"/>
+      <c r="M7" s="86"/>
       <c r="N7" s="7"/>
       <c r="O7" s="7"/>
-      <c r="P7" s="48"/>
+      <c r="P7" s="94"/>
     </row>
     <row r="8" spans="1:16" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A8" s="1"/>
@@ -2226,10 +2229,10 @@
       <c r="J8" s="7"/>
       <c r="K8" s="7"/>
       <c r="L8" s="7"/>
-      <c r="M8" s="89"/>
+      <c r="M8" s="86"/>
       <c r="N8" s="7"/>
       <c r="O8" s="7"/>
-      <c r="P8" s="48"/>
+      <c r="P8" s="94"/>
     </row>
     <row r="9" spans="1:16" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A9" s="1"/>
@@ -2240,135 +2243,135 @@
         <v>6</v>
       </c>
       <c r="D9" s="29" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="E9" s="29" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="F9" s="29" t="s">
-        <v>152</v>
+        <v>150</v>
       </c>
       <c r="G9" s="29" t="s">
-        <v>189</v>
+        <v>187</v>
       </c>
       <c r="H9" s="29" t="s">
+        <v>309</v>
+      </c>
+      <c r="I9" s="29" t="s">
+        <v>241</v>
+      </c>
+      <c r="J9" s="29" t="s">
+        <v>311</v>
+      </c>
+      <c r="K9" s="29" t="s">
+        <v>304</v>
+      </c>
+      <c r="L9" s="41" t="s">
+        <v>312</v>
+      </c>
+      <c r="M9" s="29" t="s">
+        <v>314</v>
+      </c>
+      <c r="N9" s="82" t="s">
+        <v>315</v>
+      </c>
+      <c r="O9" s="29" t="s">
+        <v>316</v>
+      </c>
+      <c r="P9" s="29" t="s">
         <v>313</v>
-      </c>
-      <c r="I9" s="29" t="s">
-        <v>244</v>
-      </c>
-      <c r="J9" s="29" t="s">
-        <v>315</v>
-      </c>
-      <c r="K9" s="29" t="s">
-        <v>308</v>
-      </c>
-      <c r="L9" s="41" t="s">
-        <v>316</v>
-      </c>
-      <c r="M9" s="29" t="s">
-        <v>318</v>
-      </c>
-      <c r="N9" s="85" t="s">
-        <v>319</v>
-      </c>
-      <c r="O9" s="29" t="s">
-        <v>320</v>
-      </c>
-      <c r="P9" s="29" t="s">
-        <v>317</v>
       </c>
     </row>
     <row r="10" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A10" s="1"/>
-      <c r="B10" s="49">
+      <c r="B10" s="46">
         <f>ROW(B10) - ROW($B$9)</f>
         <v>1</v>
       </c>
-      <c r="C10" s="50" t="s">
+      <c r="C10" s="47" t="s">
         <v>7</v>
       </c>
-      <c r="D10" s="51" t="s">
-        <v>26</v>
-      </c>
-      <c r="E10" s="51"/>
-      <c r="F10" s="51" t="s">
-        <v>311</v>
-      </c>
-      <c r="G10" s="51" t="s">
-        <v>153</v>
-      </c>
-      <c r="H10" s="51" t="s">
-        <v>314</v>
-      </c>
-      <c r="I10" s="51" t="s">
-        <v>314</v>
-      </c>
-      <c r="J10" s="51" t="s">
-        <v>314</v>
-      </c>
-      <c r="K10" s="51">
+      <c r="D10" s="48" t="s">
+        <v>25</v>
+      </c>
+      <c r="E10" s="48"/>
+      <c r="F10" s="48" t="s">
+        <v>307</v>
+      </c>
+      <c r="G10" s="48" t="s">
+        <v>151</v>
+      </c>
+      <c r="H10" s="48" t="s">
+        <v>310</v>
+      </c>
+      <c r="I10" s="48" t="s">
+        <v>310</v>
+      </c>
+      <c r="J10" s="48" t="s">
+        <v>310</v>
+      </c>
+      <c r="K10" s="48">
         <v>1</v>
       </c>
-      <c r="L10" s="79">
+      <c r="L10" s="76">
         <f>K10*5</f>
         <v>5</v>
       </c>
-      <c r="M10" s="51" t="s">
-        <v>314</v>
-      </c>
-      <c r="N10" s="84" t="s">
-        <v>314</v>
-      </c>
-      <c r="O10" s="66" t="s">
-        <v>314</v>
+      <c r="M10" s="48" t="s">
+        <v>310</v>
+      </c>
+      <c r="N10" s="81" t="s">
+        <v>310</v>
+      </c>
+      <c r="O10" s="63" t="s">
+        <v>310</v>
       </c>
       <c r="P10" s="30"/>
     </row>
     <row r="11" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A11" s="1"/>
-      <c r="B11" s="52">
+      <c r="B11" s="49">
         <f t="shared" ref="B11:B71" si="0">ROW(B11) - ROW($B$9)</f>
         <v>2</v>
       </c>
-      <c r="C11" s="50" t="s">
+      <c r="C11" s="47" t="s">
         <v>7</v>
       </c>
       <c r="D11" s="31" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="E11" s="31" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="F11" s="31" t="s">
-        <v>311</v>
+        <v>307</v>
       </c>
       <c r="G11" s="31" t="s">
-        <v>154</v>
+        <v>152</v>
       </c>
       <c r="H11" s="30" t="s">
-        <v>314</v>
+        <v>310</v>
       </c>
       <c r="I11" s="31" t="s">
-        <v>245</v>
+        <v>242</v>
       </c>
       <c r="J11" s="30" t="s">
-        <v>314</v>
+        <v>310</v>
       </c>
       <c r="K11" s="31">
         <v>1</v>
       </c>
-      <c r="L11" s="75">
+      <c r="L11" s="72">
         <f t="shared" ref="L11" si="1">K11*5</f>
         <v>5</v>
       </c>
-      <c r="M11" s="67" t="s">
-        <v>321</v>
-      </c>
-      <c r="N11" s="81">
+      <c r="M11" s="64" t="s">
+        <v>317</v>
+      </c>
+      <c r="N11" s="78">
         <v>1.59</v>
       </c>
-      <c r="O11" s="69">
+      <c r="O11" s="66">
         <f t="shared" ref="O11" si="2">N11*L11</f>
         <v>7.95</v>
       </c>
@@ -2376,48 +2379,48 @@
     </row>
     <row r="12" spans="1:16" ht="36" x14ac:dyDescent="0.25">
       <c r="A12" s="1"/>
-      <c r="B12" s="49">
+      <c r="B12" s="46">
         <f>ROW(B12) - ROW($B$9)</f>
         <v>3</v>
       </c>
-      <c r="C12" s="53" t="s">
+      <c r="C12" s="50" t="s">
         <v>8</v>
       </c>
       <c r="D12" s="30" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="E12" s="30" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="F12" s="30" t="s">
-        <v>155</v>
+        <v>153</v>
       </c>
       <c r="G12" s="30" t="s">
-        <v>190</v>
+        <v>188</v>
       </c>
       <c r="H12" s="30" t="s">
-        <v>314</v>
+        <v>310</v>
       </c>
       <c r="I12" s="30" t="s">
-        <v>246</v>
+        <v>243</v>
       </c>
       <c r="J12" s="30" t="s">
-        <v>282</v>
+        <v>278</v>
       </c>
       <c r="K12" s="30">
         <v>23</v>
       </c>
-      <c r="L12" s="76">
+      <c r="L12" s="73">
         <f>K12*5</f>
         <v>115</v>
       </c>
-      <c r="M12" s="70" t="s">
-        <v>321</v>
-      </c>
-      <c r="N12" s="81">
+      <c r="M12" s="67" t="s">
+        <v>317</v>
+      </c>
+      <c r="N12" s="78">
         <v>1.03E-2</v>
       </c>
-      <c r="O12" s="68">
+      <c r="O12" s="65">
         <f>N12*L12</f>
         <v>1.1845000000000001</v>
       </c>
@@ -2425,48 +2428,48 @@
     </row>
     <row r="13" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A13" s="1"/>
-      <c r="B13" s="52">
+      <c r="B13" s="49">
         <f t="shared" si="0"/>
         <v>4</v>
       </c>
-      <c r="C13" s="50" t="s">
+      <c r="C13" s="47" t="s">
         <v>8</v>
       </c>
       <c r="D13" s="31" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="E13" s="31" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="F13" s="31" t="s">
-        <v>155</v>
+        <v>153</v>
       </c>
       <c r="G13" s="31" t="s">
-        <v>191</v>
+        <v>189</v>
       </c>
       <c r="H13" s="31" t="s">
-        <v>314</v>
+        <v>310</v>
       </c>
       <c r="I13" s="31" t="s">
-        <v>247</v>
+        <v>244</v>
       </c>
       <c r="J13" s="31" t="s">
-        <v>283</v>
+        <v>279</v>
       </c>
       <c r="K13" s="31">
         <v>3</v>
       </c>
-      <c r="L13" s="75">
+      <c r="L13" s="72">
         <f t="shared" ref="L13" si="3">K13*5</f>
         <v>15</v>
       </c>
-      <c r="M13" s="90" t="s">
-        <v>321</v>
-      </c>
-      <c r="N13" s="80">
+      <c r="M13" s="87" t="s">
+        <v>317</v>
+      </c>
+      <c r="N13" s="77">
         <v>0.121</v>
       </c>
-      <c r="O13" s="69">
+      <c r="O13" s="66">
         <f t="shared" ref="O13" si="4">N13*L13</f>
         <v>1.8149999999999999</v>
       </c>
@@ -2474,48 +2477,48 @@
     </row>
     <row r="14" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A14" s="1"/>
-      <c r="B14" s="49">
+      <c r="B14" s="46">
         <f>ROW(B14) - ROW($B$9)</f>
         <v>5</v>
       </c>
-      <c r="C14" s="50" t="s">
+      <c r="C14" s="47" t="s">
         <v>8</v>
       </c>
       <c r="D14" s="30" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="E14" s="30" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="F14" s="30" t="s">
-        <v>155</v>
+        <v>153</v>
       </c>
       <c r="G14" s="30" t="s">
-        <v>192</v>
+        <v>190</v>
       </c>
       <c r="H14" s="30" t="s">
-        <v>314</v>
+        <v>310</v>
       </c>
       <c r="I14" s="30" t="s">
-        <v>246</v>
+        <v>243</v>
       </c>
       <c r="J14" s="30" t="s">
-        <v>284</v>
+        <v>280</v>
       </c>
       <c r="K14" s="30">
         <v>1</v>
       </c>
-      <c r="L14" s="76">
+      <c r="L14" s="73">
         <f>K14*5</f>
         <v>5</v>
       </c>
-      <c r="M14" s="90" t="s">
-        <v>321</v>
-      </c>
-      <c r="N14" s="81">
+      <c r="M14" s="87" t="s">
+        <v>317</v>
+      </c>
+      <c r="N14" s="78">
         <v>0.1</v>
       </c>
-      <c r="O14" s="68">
+      <c r="O14" s="65">
         <f>N14*L14</f>
         <v>0.5</v>
       </c>
@@ -2523,48 +2526,48 @@
     </row>
     <row r="15" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A15" s="1"/>
-      <c r="B15" s="52">
+      <c r="B15" s="49">
         <f t="shared" si="0"/>
         <v>6</v>
       </c>
-      <c r="C15" s="50" t="s">
+      <c r="C15" s="47" t="s">
         <v>8</v>
       </c>
       <c r="D15" s="31" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="E15" s="31" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="F15" s="31" t="s">
-        <v>156</v>
+        <v>154</v>
       </c>
       <c r="G15" s="31" t="s">
-        <v>193</v>
+        <v>191</v>
       </c>
       <c r="H15" s="31" t="s">
-        <v>314</v>
+        <v>310</v>
       </c>
       <c r="I15" s="31" t="s">
-        <v>248</v>
+        <v>245</v>
       </c>
       <c r="J15" s="31" t="s">
-        <v>285</v>
+        <v>281</v>
       </c>
       <c r="K15" s="31">
         <v>4</v>
       </c>
-      <c r="L15" s="75">
+      <c r="L15" s="72">
         <f t="shared" ref="L15" si="5">K15*5</f>
         <v>20</v>
       </c>
-      <c r="M15" s="90" t="s">
-        <v>321</v>
-      </c>
-      <c r="N15" s="80">
+      <c r="M15" s="87" t="s">
+        <v>317</v>
+      </c>
+      <c r="N15" s="77">
         <v>0.78600000000000003</v>
       </c>
-      <c r="O15" s="69">
+      <c r="O15" s="66">
         <f t="shared" ref="O15" si="6">N15*L15</f>
         <v>15.72</v>
       </c>
@@ -2572,48 +2575,48 @@
     </row>
     <row r="16" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A16" s="1"/>
-      <c r="B16" s="49">
+      <c r="B16" s="46">
         <f>ROW(B16) - ROW($B$9)</f>
         <v>7</v>
       </c>
-      <c r="C16" s="53" t="s">
+      <c r="C16" s="50" t="s">
         <v>8</v>
       </c>
       <c r="D16" s="30" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="E16" s="30" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="F16" s="30" t="s">
-        <v>155</v>
-      </c>
-      <c r="G16" s="65" t="s">
-        <v>194</v>
+        <v>153</v>
+      </c>
+      <c r="G16" s="62" t="s">
+        <v>192</v>
       </c>
       <c r="H16" s="30" t="s">
-        <v>314</v>
+        <v>310</v>
       </c>
       <c r="I16" s="30" t="s">
-        <v>249</v>
+        <v>246</v>
       </c>
       <c r="J16" s="30" t="s">
-        <v>286</v>
+        <v>282</v>
       </c>
       <c r="K16" s="30">
         <v>5</v>
       </c>
-      <c r="L16" s="76">
+      <c r="L16" s="73">
         <f>K16*5</f>
         <v>25</v>
       </c>
-      <c r="M16" s="90" t="s">
-        <v>321</v>
-      </c>
-      <c r="N16" s="81">
+      <c r="M16" s="87" t="s">
+        <v>317</v>
+      </c>
+      <c r="N16" s="78">
         <v>0.161</v>
       </c>
-      <c r="O16" s="68">
+      <c r="O16" s="65">
         <f>N16*L16</f>
         <v>4.0250000000000004</v>
       </c>
@@ -2621,48 +2624,48 @@
     </row>
     <row r="17" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A17" s="1"/>
-      <c r="B17" s="52">
+      <c r="B17" s="49">
         <f t="shared" si="0"/>
         <v>8</v>
       </c>
-      <c r="C17" s="50" t="s">
+      <c r="C17" s="47" t="s">
         <v>8</v>
       </c>
       <c r="D17" s="31" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="E17" s="31" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="F17" s="31" t="s">
-        <v>155</v>
+        <v>153</v>
       </c>
       <c r="G17" s="31" t="s">
-        <v>195</v>
+        <v>193</v>
       </c>
       <c r="H17" s="31" t="s">
-        <v>314</v>
+        <v>310</v>
       </c>
       <c r="I17" s="31" t="s">
-        <v>250</v>
+        <v>247</v>
       </c>
       <c r="J17" s="31" t="s">
-        <v>287</v>
+        <v>283</v>
       </c>
       <c r="K17" s="31">
         <v>2</v>
       </c>
-      <c r="L17" s="75">
+      <c r="L17" s="72">
         <f t="shared" ref="L17" si="7">K17*5</f>
         <v>10</v>
       </c>
-      <c r="M17" s="90" t="s">
-        <v>321</v>
-      </c>
-      <c r="N17" s="80">
+      <c r="M17" s="87" t="s">
+        <v>317</v>
+      </c>
+      <c r="N17" s="77">
         <v>1.6E-2</v>
       </c>
-      <c r="O17" s="69">
+      <c r="O17" s="66">
         <f t="shared" ref="O17" si="8">N17*L17</f>
         <v>0.16</v>
       </c>
@@ -2670,48 +2673,48 @@
     </row>
     <row r="18" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A18" s="1"/>
-      <c r="B18" s="49">
+      <c r="B18" s="46">
         <f>ROW(B18) - ROW($B$9)</f>
         <v>9</v>
       </c>
-      <c r="C18" s="53" t="s">
+      <c r="C18" s="50" t="s">
         <v>8</v>
       </c>
       <c r="D18" s="30" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="E18" s="30" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="F18" s="30" t="s">
-        <v>155</v>
+        <v>153</v>
       </c>
       <c r="G18" s="30" t="s">
-        <v>196</v>
+        <v>194</v>
       </c>
       <c r="H18" s="30" t="s">
-        <v>314</v>
+        <v>310</v>
       </c>
       <c r="I18" s="30" t="s">
-        <v>250</v>
+        <v>247</v>
       </c>
       <c r="J18" s="30" t="s">
-        <v>288</v>
+        <v>284</v>
       </c>
       <c r="K18" s="30">
         <v>5</v>
       </c>
-      <c r="L18" s="76">
+      <c r="L18" s="73">
         <f>K18*5</f>
         <v>25</v>
       </c>
-      <c r="M18" s="90" t="s">
-        <v>321</v>
-      </c>
-      <c r="N18" s="81">
+      <c r="M18" s="87" t="s">
+        <v>317</v>
+      </c>
+      <c r="N18" s="78">
         <v>1.9E-2</v>
       </c>
-      <c r="O18" s="68">
+      <c r="O18" s="65">
         <f>N18*L18</f>
         <v>0.47499999999999998</v>
       </c>
@@ -2719,48 +2722,48 @@
     </row>
     <row r="19" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A19" s="1"/>
-      <c r="B19" s="52">
+      <c r="B19" s="49">
         <f t="shared" si="0"/>
         <v>10</v>
       </c>
-      <c r="C19" s="50" t="s">
+      <c r="C19" s="47" t="s">
         <v>8</v>
       </c>
       <c r="D19" s="31" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="E19" s="31" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="F19" s="31" t="s">
-        <v>157</v>
+        <v>155</v>
       </c>
       <c r="G19" s="31" t="s">
-        <v>197</v>
+        <v>195</v>
       </c>
       <c r="H19" s="31" t="s">
-        <v>314</v>
+        <v>310</v>
       </c>
       <c r="I19" s="31" t="s">
-        <v>250</v>
+        <v>247</v>
       </c>
       <c r="J19" s="31" t="s">
-        <v>289</v>
+        <v>285</v>
       </c>
       <c r="K19" s="31">
         <v>1</v>
       </c>
-      <c r="L19" s="75">
+      <c r="L19" s="72">
         <f t="shared" ref="L19" si="9">K19*5</f>
         <v>5</v>
       </c>
-      <c r="M19" s="90" t="s">
-        <v>321</v>
-      </c>
-      <c r="N19" s="80">
+      <c r="M19" s="87" t="s">
+        <v>317</v>
+      </c>
+      <c r="N19" s="77">
         <v>0.1</v>
       </c>
-      <c r="O19" s="69">
+      <c r="O19" s="66">
         <f t="shared" ref="O19" si="10">N19*L19</f>
         <v>0.5</v>
       </c>
@@ -2768,48 +2771,48 @@
     </row>
     <row r="20" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A20" s="1"/>
-      <c r="B20" s="49">
+      <c r="B20" s="46">
         <f>ROW(B20) - ROW($B$9)</f>
         <v>11</v>
       </c>
-      <c r="C20" s="50" t="s">
+      <c r="C20" s="47" t="s">
         <v>8</v>
       </c>
       <c r="D20" s="30" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="E20" s="30" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="F20" s="30" t="s">
-        <v>155</v>
+        <v>153</v>
       </c>
       <c r="G20" s="30" t="s">
-        <v>198</v>
+        <v>196</v>
       </c>
       <c r="H20" s="30" t="s">
-        <v>314</v>
+        <v>310</v>
       </c>
       <c r="I20" s="30" t="s">
-        <v>246</v>
+        <v>243</v>
       </c>
       <c r="J20" s="30" t="s">
-        <v>290</v>
+        <v>286</v>
       </c>
       <c r="K20" s="30">
         <v>1</v>
       </c>
-      <c r="L20" s="76">
+      <c r="L20" s="73">
         <f>K20*5</f>
         <v>5</v>
       </c>
-      <c r="M20" s="90" t="s">
-        <v>321</v>
-      </c>
-      <c r="N20" s="81">
+      <c r="M20" s="87" t="s">
+        <v>317</v>
+      </c>
+      <c r="N20" s="78">
         <v>0.1</v>
       </c>
-      <c r="O20" s="68">
+      <c r="O20" s="65">
         <f>N20*L20</f>
         <v>0.5</v>
       </c>
@@ -2817,48 +2820,48 @@
     </row>
     <row r="21" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A21" s="1"/>
-      <c r="B21" s="52">
+      <c r="B21" s="49">
         <f t="shared" si="0"/>
         <v>12</v>
       </c>
-      <c r="C21" s="50" t="s">
+      <c r="C21" s="47" t="s">
         <v>8</v>
       </c>
       <c r="D21" s="31" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="E21" s="31" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="F21" s="31" t="s">
-        <v>155</v>
+        <v>153</v>
       </c>
       <c r="G21" s="31" t="s">
-        <v>199</v>
+        <v>197</v>
       </c>
       <c r="H21" s="31" t="s">
-        <v>314</v>
+        <v>310</v>
       </c>
       <c r="I21" s="31" t="s">
-        <v>250</v>
+        <v>247</v>
       </c>
       <c r="J21" s="31" t="s">
-        <v>291</v>
+        <v>287</v>
       </c>
       <c r="K21" s="31">
         <v>1</v>
       </c>
-      <c r="L21" s="75">
+      <c r="L21" s="72">
         <f t="shared" ref="L21" si="11">K21*5</f>
         <v>5</v>
       </c>
-      <c r="M21" s="90" t="s">
-        <v>321</v>
-      </c>
-      <c r="N21" s="80">
+      <c r="M21" s="87" t="s">
+        <v>317</v>
+      </c>
+      <c r="N21" s="77">
         <v>0.1</v>
       </c>
-      <c r="O21" s="69">
+      <c r="O21" s="66">
         <f t="shared" ref="O21" si="12">N21*L21</f>
         <v>0.5</v>
       </c>
@@ -2866,48 +2869,48 @@
     </row>
     <row r="22" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A22" s="1"/>
-      <c r="B22" s="49">
+      <c r="B22" s="46">
         <f>ROW(B22) - ROW($B$9)</f>
         <v>13</v>
       </c>
-      <c r="C22" s="53" t="s">
+      <c r="C22" s="50" t="s">
         <v>8</v>
       </c>
       <c r="D22" s="30" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="E22" s="30" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="F22" s="30" t="s">
-        <v>158</v>
+        <v>156</v>
       </c>
       <c r="G22" s="30" t="s">
-        <v>200</v>
+        <v>198</v>
       </c>
       <c r="H22" s="30" t="s">
-        <v>314</v>
+        <v>310</v>
       </c>
       <c r="I22" s="30" t="s">
-        <v>248</v>
+        <v>245</v>
       </c>
       <c r="J22" s="30" t="s">
-        <v>292</v>
+        <v>288</v>
       </c>
       <c r="K22" s="30">
         <v>1</v>
       </c>
-      <c r="L22" s="76">
+      <c r="L22" s="73">
         <f>K22*5</f>
         <v>5</v>
       </c>
-      <c r="M22" s="90" t="s">
-        <v>321</v>
-      </c>
-      <c r="N22" s="81">
+      <c r="M22" s="87" t="s">
+        <v>317</v>
+      </c>
+      <c r="N22" s="78">
         <v>0.99</v>
       </c>
-      <c r="O22" s="68">
+      <c r="O22" s="65">
         <f>N22*L22</f>
         <v>4.95</v>
       </c>
@@ -2915,96 +2918,96 @@
     </row>
     <row r="23" spans="1:16" ht="30" x14ac:dyDescent="0.25">
       <c r="A23" s="1"/>
-      <c r="B23" s="52">
+      <c r="B23" s="49">
         <f t="shared" si="0"/>
         <v>14</v>
       </c>
-      <c r="C23" s="50" t="s">
+      <c r="C23" s="47" t="s">
         <v>9</v>
       </c>
       <c r="D23" s="31" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="E23" s="31" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="F23" s="31" t="s">
-        <v>159</v>
+        <v>157</v>
       </c>
       <c r="G23" s="31" t="s">
-        <v>201</v>
+        <v>199</v>
       </c>
       <c r="H23" s="31" t="s">
-        <v>314</v>
+        <v>310</v>
       </c>
       <c r="I23" s="31" t="s">
-        <v>251</v>
+        <v>248</v>
       </c>
       <c r="J23" s="30" t="s">
-        <v>314</v>
+        <v>310</v>
       </c>
       <c r="K23" s="31">
         <v>1</v>
       </c>
-      <c r="L23" s="75">
+      <c r="L23" s="72">
         <f t="shared" ref="L23" si="13">K23*5</f>
         <v>5</v>
       </c>
-      <c r="M23" s="94" t="s">
-        <v>322</v>
-      </c>
-      <c r="N23" s="80" t="s">
-        <v>314</v>
-      </c>
-      <c r="O23" s="69" t="s">
-        <v>314</v>
+      <c r="M23" s="91" t="s">
+        <v>318</v>
+      </c>
+      <c r="N23" s="77" t="s">
+        <v>310</v>
+      </c>
+      <c r="O23" s="66" t="s">
+        <v>310</v>
       </c>
       <c r="P23" s="31"/>
     </row>
     <row r="24" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A24" s="1"/>
-      <c r="B24" s="49">
+      <c r="B24" s="46">
         <f>ROW(B24) - ROW($B$9)</f>
         <v>15</v>
       </c>
-      <c r="C24" s="53" t="s">
+      <c r="C24" s="50" t="s">
         <v>9</v>
       </c>
       <c r="D24" s="30" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="E24" s="30" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="F24" s="30" t="s">
-        <v>160</v>
+        <v>158</v>
       </c>
       <c r="G24" s="30" t="s">
-        <v>202</v>
+        <v>200</v>
       </c>
       <c r="H24" s="30" t="s">
-        <v>314</v>
+        <v>310</v>
       </c>
       <c r="I24" s="30" t="s">
-        <v>252</v>
+        <v>249</v>
       </c>
       <c r="J24" s="31" t="s">
-        <v>314</v>
+        <v>310</v>
       </c>
       <c r="K24" s="30">
         <v>2</v>
       </c>
-      <c r="L24" s="76">
+      <c r="L24" s="73">
         <f>K24*5</f>
         <v>10</v>
       </c>
-      <c r="M24" s="90" t="s">
-        <v>321</v>
-      </c>
-      <c r="N24" s="81">
+      <c r="M24" s="87" t="s">
+        <v>317</v>
+      </c>
+      <c r="N24" s="78">
         <v>0.159</v>
       </c>
-      <c r="O24" s="68">
+      <c r="O24" s="65">
         <f>N24*L24</f>
         <v>1.59</v>
       </c>
@@ -3012,96 +3015,96 @@
     </row>
     <row r="25" spans="1:16" ht="30" x14ac:dyDescent="0.25">
       <c r="A25" s="1"/>
-      <c r="B25" s="52">
+      <c r="B25" s="49">
         <f t="shared" si="0"/>
         <v>16</v>
       </c>
-      <c r="C25" s="50" t="s">
+      <c r="C25" s="47" t="s">
         <v>10</v>
       </c>
       <c r="D25" s="31" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="E25" s="31" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="F25" s="31" t="s">
-        <v>160</v>
+        <v>158</v>
       </c>
       <c r="G25" s="31" t="s">
-        <v>203</v>
+        <v>201</v>
       </c>
       <c r="H25" s="31" t="s">
-        <v>314</v>
+        <v>310</v>
       </c>
       <c r="I25" s="31" t="s">
-        <v>253</v>
+        <v>250</v>
       </c>
       <c r="J25" s="30" t="s">
-        <v>314</v>
+        <v>310</v>
       </c>
       <c r="K25" s="31">
         <v>1</v>
       </c>
-      <c r="L25" s="75">
+      <c r="L25" s="72">
         <f t="shared" ref="L25" si="14">K25*5</f>
         <v>5</v>
       </c>
-      <c r="M25" s="94" t="s">
-        <v>322</v>
-      </c>
-      <c r="N25" s="80" t="s">
-        <v>314</v>
-      </c>
-      <c r="O25" s="69" t="s">
-        <v>314</v>
+      <c r="M25" s="91" t="s">
+        <v>318</v>
+      </c>
+      <c r="N25" s="77" t="s">
+        <v>310</v>
+      </c>
+      <c r="O25" s="66" t="s">
+        <v>310</v>
       </c>
       <c r="P25" s="31"/>
     </row>
     <row r="26" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A26" s="1"/>
-      <c r="B26" s="49">
+      <c r="B26" s="46">
         <f>ROW(B26) - ROW($B$9)</f>
         <v>17</v>
       </c>
-      <c r="C26" s="53" t="s">
+      <c r="C26" s="50" t="s">
         <v>9</v>
       </c>
       <c r="D26" s="30" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="E26" s="30" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="F26" s="30" t="s">
-        <v>161</v>
+        <v>159</v>
       </c>
       <c r="G26" s="30" t="s">
-        <v>204</v>
+        <v>202</v>
       </c>
       <c r="H26" s="30" t="s">
-        <v>314</v>
+        <v>310</v>
       </c>
       <c r="I26" s="30" t="s">
-        <v>254</v>
+        <v>251</v>
       </c>
       <c r="J26" s="31" t="s">
-        <v>314</v>
+        <v>310</v>
       </c>
       <c r="K26" s="30">
         <v>1</v>
       </c>
-      <c r="L26" s="76">
+      <c r="L26" s="73">
         <f>K26*5</f>
         <v>5</v>
       </c>
-      <c r="M26" s="90" t="s">
-        <v>321</v>
-      </c>
-      <c r="N26" s="81">
+      <c r="M26" s="87" t="s">
+        <v>317</v>
+      </c>
+      <c r="N26" s="78">
         <v>0.23</v>
       </c>
-      <c r="O26" s="68">
+      <c r="O26" s="65">
         <f>N26*L26</f>
         <v>1.1500000000000001</v>
       </c>
@@ -3109,48 +3112,48 @@
     </row>
     <row r="27" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A27" s="1"/>
-      <c r="B27" s="52">
+      <c r="B27" s="49">
         <f t="shared" si="0"/>
         <v>18</v>
       </c>
-      <c r="C27" s="50" t="s">
+      <c r="C27" s="47" t="s">
         <v>9</v>
       </c>
       <c r="D27" s="31" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="E27" s="31" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="F27" s="31" t="s">
-        <v>162</v>
+        <v>160</v>
       </c>
       <c r="G27" s="31" t="s">
-        <v>205</v>
+        <v>203</v>
       </c>
       <c r="H27" s="31" t="s">
-        <v>314</v>
+        <v>310</v>
       </c>
       <c r="I27" s="31" t="s">
-        <v>255</v>
+        <v>252</v>
       </c>
       <c r="J27" s="30" t="s">
-        <v>314</v>
+        <v>310</v>
       </c>
       <c r="K27" s="31">
         <v>1</v>
       </c>
-      <c r="L27" s="75">
+      <c r="L27" s="72">
         <f t="shared" ref="L27" si="15">K27*5</f>
         <v>5</v>
       </c>
-      <c r="M27" s="90" t="s">
-        <v>321</v>
-      </c>
-      <c r="N27" s="80">
+      <c r="M27" s="87" t="s">
+        <v>317</v>
+      </c>
+      <c r="N27" s="77">
         <v>0.44</v>
       </c>
-      <c r="O27" s="69">
+      <c r="O27" s="66">
         <f t="shared" ref="O27" si="16">N27*L27</f>
         <v>2.2000000000000002</v>
       </c>
@@ -3158,142 +3161,142 @@
     </row>
     <row r="28" spans="1:16" ht="30" x14ac:dyDescent="0.25">
       <c r="A28" s="1"/>
-      <c r="B28" s="49">
+      <c r="B28" s="46">
         <f>ROW(B28) - ROW($B$9)</f>
         <v>19</v>
       </c>
-      <c r="C28" s="53" t="s">
+      <c r="C28" s="50" t="s">
         <v>9</v>
       </c>
       <c r="D28" s="30" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="E28" s="30" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="F28" s="30" t="s">
-        <v>163</v>
+        <v>161</v>
       </c>
       <c r="G28" s="30" t="s">
-        <v>206</v>
+        <v>204</v>
       </c>
       <c r="H28" s="30" t="s">
-        <v>314</v>
+        <v>310</v>
       </c>
       <c r="I28" s="30" t="s">
-        <v>256</v>
+        <v>253</v>
       </c>
       <c r="J28" s="30" t="s">
-        <v>314</v>
+        <v>310</v>
       </c>
       <c r="K28" s="30">
         <v>1</v>
       </c>
-      <c r="L28" s="76">
+      <c r="L28" s="73">
         <f>K28*5</f>
         <v>5</v>
       </c>
-      <c r="M28" s="94" t="s">
-        <v>322</v>
-      </c>
-      <c r="N28" s="80" t="s">
-        <v>314</v>
-      </c>
-      <c r="O28" s="69" t="s">
-        <v>314</v>
+      <c r="M28" s="91" t="s">
+        <v>318</v>
+      </c>
+      <c r="N28" s="77" t="s">
+        <v>310</v>
+      </c>
+      <c r="O28" s="66" t="s">
+        <v>310</v>
       </c>
       <c r="P28" s="30"/>
     </row>
     <row r="29" spans="1:16" ht="30" x14ac:dyDescent="0.25">
       <c r="A29" s="1"/>
-      <c r="B29" s="52">
+      <c r="B29" s="49">
         <f t="shared" si="0"/>
         <v>20</v>
       </c>
-      <c r="C29" s="50" t="s">
+      <c r="C29" s="47" t="s">
         <v>9</v>
       </c>
       <c r="D29" s="31" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="E29" s="31" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="F29" s="31" t="s">
-        <v>164</v>
+        <v>162</v>
       </c>
       <c r="G29" s="31" t="s">
-        <v>207</v>
+        <v>205</v>
       </c>
       <c r="H29" s="31" t="s">
-        <v>314</v>
+        <v>310</v>
       </c>
       <c r="I29" s="31" t="s">
-        <v>257</v>
+        <v>254</v>
       </c>
       <c r="J29" s="31" t="s">
-        <v>314</v>
+        <v>310</v>
       </c>
       <c r="K29" s="31">
         <v>2</v>
       </c>
-      <c r="L29" s="75">
+      <c r="L29" s="72">
         <f t="shared" ref="L29" si="17">K29*5</f>
         <v>10</v>
       </c>
-      <c r="M29" s="94" t="s">
-        <v>322</v>
-      </c>
-      <c r="N29" s="80" t="s">
-        <v>314</v>
-      </c>
-      <c r="O29" s="69" t="s">
-        <v>314</v>
+      <c r="M29" s="91" t="s">
+        <v>318</v>
+      </c>
+      <c r="N29" s="77" t="s">
+        <v>310</v>
+      </c>
+      <c r="O29" s="66" t="s">
+        <v>310</v>
       </c>
       <c r="P29" s="31"/>
     </row>
     <row r="30" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A30" s="1"/>
-      <c r="B30" s="49">
+      <c r="B30" s="46">
         <f>ROW(B30) - ROW($B$9)</f>
         <v>21</v>
       </c>
-      <c r="C30" s="53" t="s">
+      <c r="C30" s="50" t="s">
         <v>9</v>
       </c>
       <c r="D30" s="30" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="E30" s="30" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="F30" s="30" t="s">
-        <v>165</v>
+        <v>163</v>
       </c>
       <c r="G30" s="30" t="s">
-        <v>208</v>
+        <v>206</v>
       </c>
       <c r="H30" s="30"/>
       <c r="I30" s="30" t="s">
-        <v>258</v>
+        <v>255</v>
       </c>
       <c r="J30" s="30" t="s">
-        <v>314</v>
+        <v>310</v>
       </c>
       <c r="K30" s="30">
         <v>3</v>
       </c>
-      <c r="L30" s="76">
+      <c r="L30" s="73">
         <f>K30*5</f>
         <v>15</v>
       </c>
-      <c r="M30" s="90" t="s">
-        <v>321</v>
-      </c>
-      <c r="N30" s="81">
+      <c r="M30" s="87" t="s">
+        <v>317</v>
+      </c>
+      <c r="N30" s="78">
         <v>0.32300000000000001</v>
       </c>
-      <c r="O30" s="68">
+      <c r="O30" s="65">
         <f>N30*L30</f>
         <v>4.8449999999999998</v>
       </c>
@@ -3301,336 +3304,336 @@
     </row>
     <row r="31" spans="1:16" ht="30" x14ac:dyDescent="0.25">
       <c r="A31" s="1"/>
-      <c r="B31" s="52">
+      <c r="B31" s="49">
         <f t="shared" si="0"/>
         <v>22</v>
       </c>
-      <c r="C31" s="50" t="s">
+      <c r="C31" s="47" t="s">
         <v>9</v>
       </c>
       <c r="D31" s="31" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="E31" s="31" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="F31" s="31" t="s">
-        <v>159</v>
+        <v>157</v>
       </c>
       <c r="G31" s="31" t="s">
-        <v>209</v>
+        <v>207</v>
       </c>
       <c r="H31" s="31" t="s">
-        <v>314</v>
+        <v>310</v>
       </c>
       <c r="I31" s="31" t="s">
-        <v>259</v>
+        <v>256</v>
       </c>
       <c r="J31" s="31" t="s">
-        <v>314</v>
+        <v>310</v>
       </c>
       <c r="K31" s="31">
         <v>2</v>
       </c>
-      <c r="L31" s="75">
+      <c r="L31" s="72">
         <f t="shared" ref="L31" si="18">K31*5</f>
         <v>10</v>
       </c>
-      <c r="M31" s="94" t="s">
-        <v>322</v>
-      </c>
-      <c r="N31" s="80" t="s">
-        <v>314</v>
-      </c>
-      <c r="O31" s="69" t="s">
-        <v>314</v>
+      <c r="M31" s="91" t="s">
+        <v>318</v>
+      </c>
+      <c r="N31" s="77" t="s">
+        <v>310</v>
+      </c>
+      <c r="O31" s="66" t="s">
+        <v>310</v>
       </c>
       <c r="P31" s="31"/>
     </row>
     <row r="32" spans="1:16" ht="30" x14ac:dyDescent="0.25">
       <c r="A32" s="1"/>
-      <c r="B32" s="49">
+      <c r="B32" s="46">
         <f>ROW(B32) - ROW($B$9)</f>
         <v>23</v>
       </c>
-      <c r="C32" s="53" t="s">
+      <c r="C32" s="50" t="s">
         <v>11</v>
       </c>
       <c r="D32" s="30" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="E32" s="30" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="F32" s="30" t="s">
-        <v>166</v>
+        <v>164</v>
       </c>
       <c r="G32" s="30" t="s">
-        <v>210</v>
+        <v>208</v>
       </c>
       <c r="H32" s="30" t="s">
-        <v>314</v>
+        <v>310</v>
       </c>
       <c r="I32" s="30" t="s">
-        <v>260</v>
+        <v>257</v>
       </c>
       <c r="J32" s="30" t="s">
-        <v>314</v>
+        <v>310</v>
       </c>
       <c r="K32" s="30">
         <v>1</v>
       </c>
-      <c r="L32" s="76">
+      <c r="L32" s="73">
         <f>K32*5</f>
         <v>5</v>
       </c>
-      <c r="M32" s="94" t="s">
-        <v>322</v>
-      </c>
-      <c r="N32" s="80" t="s">
-        <v>314</v>
-      </c>
-      <c r="O32" s="69" t="s">
-        <v>314</v>
+      <c r="M32" s="91" t="s">
+        <v>318</v>
+      </c>
+      <c r="N32" s="77" t="s">
+        <v>310</v>
+      </c>
+      <c r="O32" s="66" t="s">
+        <v>310</v>
       </c>
       <c r="P32" s="30"/>
     </row>
     <row r="33" spans="1:16" ht="30" x14ac:dyDescent="0.25">
       <c r="A33" s="1"/>
-      <c r="B33" s="52">
+      <c r="B33" s="49">
         <f t="shared" si="0"/>
         <v>24</v>
       </c>
-      <c r="C33" s="50" t="s">
+      <c r="C33" s="47" t="s">
         <v>11</v>
       </c>
       <c r="D33" s="31" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="E33" s="31" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="F33" s="31" t="s">
-        <v>167</v>
+        <v>165</v>
       </c>
       <c r="G33" s="31" t="s">
-        <v>211</v>
+        <v>209</v>
       </c>
       <c r="H33" s="31" t="s">
-        <v>314</v>
+        <v>310</v>
       </c>
       <c r="I33" s="31" t="s">
-        <v>261</v>
+        <v>258</v>
       </c>
       <c r="J33" s="30" t="s">
-        <v>314</v>
+        <v>310</v>
       </c>
       <c r="K33" s="31">
         <v>1</v>
       </c>
-      <c r="L33" s="75">
+      <c r="L33" s="72">
         <f t="shared" ref="L33" si="19">K33*5</f>
         <v>5</v>
       </c>
-      <c r="M33" s="94" t="s">
-        <v>322</v>
-      </c>
-      <c r="N33" s="80" t="s">
-        <v>314</v>
-      </c>
-      <c r="O33" s="69" t="s">
-        <v>314</v>
+      <c r="M33" s="91" t="s">
+        <v>318</v>
+      </c>
+      <c r="N33" s="77" t="s">
+        <v>310</v>
+      </c>
+      <c r="O33" s="66" t="s">
+        <v>310</v>
       </c>
       <c r="P33" s="31"/>
     </row>
     <row r="34" spans="1:16" ht="30" x14ac:dyDescent="0.25">
       <c r="A34" s="1"/>
-      <c r="B34" s="49">
+      <c r="B34" s="46">
         <f>ROW(B34) - ROW($B$9)</f>
         <v>25</v>
       </c>
-      <c r="C34" s="53" t="s">
+      <c r="C34" s="50" t="s">
         <v>11</v>
       </c>
       <c r="D34" s="30" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="E34" s="30" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="F34" s="30" t="s">
-        <v>168</v>
+        <v>166</v>
       </c>
       <c r="G34" s="30" t="s">
-        <v>212</v>
+        <v>210</v>
       </c>
       <c r="H34" s="30" t="s">
-        <v>314</v>
+        <v>310</v>
       </c>
       <c r="I34" s="30" t="s">
-        <v>262</v>
+        <v>259</v>
       </c>
       <c r="J34" s="31" t="s">
-        <v>314</v>
+        <v>310</v>
       </c>
       <c r="K34" s="30">
         <v>2</v>
       </c>
-      <c r="L34" s="76">
+      <c r="L34" s="73">
         <f>K34*5</f>
         <v>10</v>
       </c>
-      <c r="M34" s="94" t="s">
-        <v>322</v>
-      </c>
-      <c r="N34" s="80" t="s">
-        <v>314</v>
-      </c>
-      <c r="O34" s="69" t="s">
-        <v>314</v>
+      <c r="M34" s="91" t="s">
+        <v>318</v>
+      </c>
+      <c r="N34" s="77" t="s">
+        <v>310</v>
+      </c>
+      <c r="O34" s="66" t="s">
+        <v>310</v>
       </c>
       <c r="P34" s="30"/>
     </row>
     <row r="35" spans="1:16" ht="48" x14ac:dyDescent="0.25">
       <c r="A35" s="1"/>
-      <c r="B35" s="52">
+      <c r="B35" s="49">
         <f t="shared" si="0"/>
         <v>26</v>
       </c>
-      <c r="C35" s="50" t="s">
+      <c r="C35" s="47" t="s">
         <v>12</v>
       </c>
       <c r="D35" s="31" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="E35" s="31" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="F35" s="31" t="s">
-        <v>311</v>
+        <v>307</v>
       </c>
       <c r="G35" s="31" t="s">
-        <v>169</v>
+        <v>167</v>
       </c>
       <c r="H35" s="31" t="s">
-        <v>314</v>
+        <v>310</v>
       </c>
       <c r="I35" s="31" t="s">
-        <v>263</v>
+        <v>260</v>
       </c>
       <c r="J35" s="30" t="s">
-        <v>314</v>
+        <v>310</v>
       </c>
       <c r="K35" s="31">
         <v>1</v>
       </c>
-      <c r="L35" s="75">
+      <c r="L35" s="72">
         <f t="shared" ref="L35" si="20">K35*5</f>
         <v>5</v>
       </c>
-      <c r="M35" s="94" t="s">
-        <v>322</v>
-      </c>
-      <c r="N35" s="80" t="s">
-        <v>314</v>
-      </c>
-      <c r="O35" s="69" t="s">
-        <v>314</v>
+      <c r="M35" s="91" t="s">
+        <v>318</v>
+      </c>
+      <c r="N35" s="77" t="s">
+        <v>310</v>
+      </c>
+      <c r="O35" s="66" t="s">
+        <v>310</v>
       </c>
       <c r="P35" s="31"/>
     </row>
     <row r="36" spans="1:16" ht="48" x14ac:dyDescent="0.25">
       <c r="A36" s="1"/>
-      <c r="B36" s="49">
+      <c r="B36" s="46">
         <f>ROW(B36) - ROW($B$9)</f>
         <v>27</v>
       </c>
-      <c r="C36" s="53" t="s">
+      <c r="C36" s="50" t="s">
         <v>12</v>
       </c>
       <c r="D36" s="30" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="E36" s="30" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="F36" s="30" t="s">
-        <v>311</v>
+        <v>307</v>
       </c>
       <c r="G36" s="30" t="s">
-        <v>170</v>
+        <v>168</v>
       </c>
       <c r="H36" s="30" t="s">
-        <v>314</v>
+        <v>310</v>
       </c>
       <c r="I36" s="30" t="s">
-        <v>263</v>
+        <v>260</v>
       </c>
       <c r="J36" s="31" t="s">
-        <v>314</v>
+        <v>310</v>
       </c>
       <c r="K36" s="30">
         <v>5</v>
       </c>
-      <c r="L36" s="76">
+      <c r="L36" s="73">
         <f>K36*5</f>
         <v>25</v>
       </c>
-      <c r="M36" s="94" t="s">
-        <v>322</v>
-      </c>
-      <c r="N36" s="80" t="s">
-        <v>314</v>
-      </c>
-      <c r="O36" s="69" t="s">
-        <v>314</v>
+      <c r="M36" s="91" t="s">
+        <v>318</v>
+      </c>
+      <c r="N36" s="77" t="s">
+        <v>310</v>
+      </c>
+      <c r="O36" s="66" t="s">
+        <v>310</v>
       </c>
       <c r="P36" s="30"/>
     </row>
     <row r="37" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A37" s="1"/>
-      <c r="B37" s="52">
+      <c r="B37" s="49">
         <f t="shared" si="0"/>
         <v>28</v>
       </c>
-      <c r="C37" s="53" t="s">
+      <c r="C37" s="50" t="s">
         <v>13</v>
       </c>
       <c r="D37" s="31" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="E37" s="31" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="F37" s="31" t="s">
-        <v>311</v>
+        <v>307</v>
       </c>
       <c r="G37" s="31" t="s">
-        <v>213</v>
+        <v>211</v>
       </c>
       <c r="H37" s="31" t="s">
-        <v>314</v>
+        <v>310</v>
       </c>
       <c r="I37" s="31" t="s">
-        <v>264</v>
+        <v>261</v>
       </c>
       <c r="J37" s="30" t="s">
-        <v>314</v>
+        <v>310</v>
       </c>
       <c r="K37" s="31">
         <v>1</v>
       </c>
-      <c r="L37" s="75">
+      <c r="L37" s="72">
         <f t="shared" ref="L37" si="21">K37*5</f>
         <v>5</v>
       </c>
-      <c r="M37" s="90" t="s">
-        <v>321</v>
-      </c>
-      <c r="N37" s="80">
+      <c r="M37" s="87" t="s">
+        <v>317</v>
+      </c>
+      <c r="N37" s="77">
         <v>1.46</v>
       </c>
-      <c r="O37" s="69">
+      <c r="O37" s="66">
         <f t="shared" ref="O37" si="22">N37*L37</f>
         <v>7.3</v>
       </c>
@@ -3638,240 +3641,240 @@
     </row>
     <row r="38" spans="1:16" ht="36" x14ac:dyDescent="0.25">
       <c r="A38" s="1"/>
-      <c r="B38" s="49">
+      <c r="B38" s="46">
         <f>ROW(B38) - ROW($B$9)</f>
         <v>29</v>
       </c>
-      <c r="C38" s="53" t="s">
+      <c r="C38" s="50" t="s">
         <v>13</v>
       </c>
       <c r="D38" s="30" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="E38" s="30" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="F38" s="30" t="s">
-        <v>311</v>
+        <v>307</v>
       </c>
       <c r="G38" s="30" t="s">
-        <v>214</v>
+        <v>212</v>
       </c>
       <c r="H38" s="30" t="s">
-        <v>314</v>
+        <v>310</v>
       </c>
       <c r="I38" s="30" t="s">
-        <v>265</v>
+        <v>262</v>
       </c>
       <c r="J38" s="30" t="s">
-        <v>314</v>
+        <v>310</v>
       </c>
       <c r="K38" s="30">
         <v>1</v>
       </c>
-      <c r="L38" s="76">
+      <c r="L38" s="73">
         <f>K38*5</f>
         <v>5</v>
       </c>
-      <c r="M38" s="94" t="s">
-        <v>322</v>
-      </c>
-      <c r="N38" s="80" t="s">
-        <v>314</v>
-      </c>
-      <c r="O38" s="69" t="s">
-        <v>314</v>
+      <c r="M38" s="91" t="s">
+        <v>318</v>
+      </c>
+      <c r="N38" s="77" t="s">
+        <v>310</v>
+      </c>
+      <c r="O38" s="66" t="s">
+        <v>310</v>
       </c>
       <c r="P38" s="30"/>
     </row>
     <row r="39" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A39" s="1"/>
-      <c r="B39" s="52">
+      <c r="B39" s="49">
         <f t="shared" si="0"/>
         <v>30</v>
       </c>
-      <c r="C39" s="50" t="s">
+      <c r="C39" s="47" t="s">
         <v>14</v>
       </c>
-      <c r="D39" s="54" t="s">
-        <v>55</v>
-      </c>
-      <c r="E39" s="54" t="s">
-        <v>118</v>
-      </c>
-      <c r="F39" s="51" t="s">
-        <v>311</v>
-      </c>
-      <c r="G39" s="54" t="s">
-        <v>215</v>
-      </c>
-      <c r="H39" s="51" t="s">
-        <v>314</v>
-      </c>
-      <c r="I39" s="51" t="s">
-        <v>314</v>
-      </c>
-      <c r="J39" s="54" t="s">
-        <v>314</v>
-      </c>
-      <c r="K39" s="54">
+      <c r="D39" s="51" t="s">
+        <v>54</v>
+      </c>
+      <c r="E39" s="51" t="s">
+        <v>117</v>
+      </c>
+      <c r="F39" s="48" t="s">
+        <v>307</v>
+      </c>
+      <c r="G39" s="51" t="s">
+        <v>213</v>
+      </c>
+      <c r="H39" s="48" t="s">
+        <v>310</v>
+      </c>
+      <c r="I39" s="48" t="s">
+        <v>310</v>
+      </c>
+      <c r="J39" s="51" t="s">
+        <v>310</v>
+      </c>
+      <c r="K39" s="51">
         <v>2</v>
       </c>
-      <c r="L39" s="77">
+      <c r="L39" s="74">
         <f t="shared" ref="L39" si="23">K39*5</f>
         <v>10</v>
       </c>
-      <c r="M39" s="91" t="s">
-        <v>314</v>
-      </c>
-      <c r="N39" s="82" t="s">
-        <v>314</v>
-      </c>
-      <c r="O39" s="71" t="s">
-        <v>314</v>
+      <c r="M39" s="88" t="s">
+        <v>310</v>
+      </c>
+      <c r="N39" s="79" t="s">
+        <v>310</v>
+      </c>
+      <c r="O39" s="68" t="s">
+        <v>310</v>
       </c>
       <c r="P39" s="31"/>
     </row>
-    <row r="40" spans="1:16" ht="48" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:16" ht="30" x14ac:dyDescent="0.25">
       <c r="A40" s="1"/>
-      <c r="B40" s="49">
+      <c r="B40" s="46">
         <f>ROW(B40) - ROW($B$9)</f>
         <v>31</v>
       </c>
-      <c r="C40" s="53" t="s">
-        <v>15</v>
+      <c r="C40" s="50" t="s">
+        <v>319</v>
       </c>
       <c r="D40" s="30" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="E40" s="30" t="s">
-        <v>119</v>
+        <v>320</v>
       </c>
       <c r="F40" s="30" t="s">
-        <v>311</v>
+        <v>321</v>
       </c>
       <c r="G40" s="30" t="s">
-        <v>216</v>
+        <v>322</v>
       </c>
       <c r="H40" s="30" t="s">
-        <v>314</v>
+        <v>310</v>
       </c>
       <c r="I40" s="30" t="s">
-        <v>266</v>
+        <v>323</v>
       </c>
       <c r="J40" s="30" t="s">
-        <v>314</v>
+        <v>310</v>
       </c>
       <c r="K40" s="30">
         <v>1</v>
       </c>
-      <c r="L40" s="76">
+      <c r="L40" s="73">
         <f>K40*5</f>
         <v>5</v>
       </c>
-      <c r="M40" s="94" t="s">
-        <v>322</v>
-      </c>
-      <c r="N40" s="80" t="s">
-        <v>314</v>
-      </c>
-      <c r="O40" s="69" t="s">
-        <v>314</v>
+      <c r="M40" s="91" t="s">
+        <v>318</v>
+      </c>
+      <c r="N40" s="77" t="s">
+        <v>310</v>
+      </c>
+      <c r="O40" s="66" t="s">
+        <v>310</v>
       </c>
       <c r="P40" s="30"/>
     </row>
     <row r="41" spans="1:16" ht="48" x14ac:dyDescent="0.25">
       <c r="A41" s="1"/>
-      <c r="B41" s="52">
+      <c r="B41" s="49">
         <f t="shared" si="0"/>
         <v>32</v>
       </c>
-      <c r="C41" s="50" t="s">
-        <v>16</v>
+      <c r="C41" s="47" t="s">
+        <v>15</v>
       </c>
       <c r="D41" s="31" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="E41" s="31" t="s">
-        <v>120</v>
+        <v>118</v>
       </c>
       <c r="F41" s="30" t="s">
-        <v>311</v>
+        <v>307</v>
       </c>
       <c r="G41" s="31" t="s">
-        <v>171</v>
+        <v>169</v>
       </c>
       <c r="H41" s="31" t="s">
-        <v>314</v>
+        <v>310</v>
       </c>
       <c r="I41" s="31" t="s">
-        <v>267</v>
+        <v>263</v>
       </c>
       <c r="J41" s="31" t="s">
-        <v>314</v>
+        <v>310</v>
       </c>
       <c r="K41" s="31">
         <v>1</v>
       </c>
-      <c r="L41" s="75">
+      <c r="L41" s="72">
         <f t="shared" ref="L41" si="24">K41*5</f>
         <v>5</v>
       </c>
-      <c r="M41" s="94" t="s">
-        <v>322</v>
-      </c>
-      <c r="N41" s="80" t="s">
-        <v>314</v>
-      </c>
-      <c r="O41" s="69" t="s">
-        <v>314</v>
+      <c r="M41" s="91" t="s">
+        <v>318</v>
+      </c>
+      <c r="N41" s="77" t="s">
+        <v>310</v>
+      </c>
+      <c r="O41" s="66" t="s">
+        <v>310</v>
       </c>
       <c r="P41" s="31"/>
     </row>
     <row r="42" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A42" s="1"/>
-      <c r="B42" s="55">
+      <c r="B42" s="52">
         <f>ROW(B42) - ROW($B$9)</f>
         <v>33</v>
       </c>
-      <c r="C42" s="56" t="s">
-        <v>17</v>
-      </c>
-      <c r="D42" s="57" t="s">
-        <v>58</v>
-      </c>
-      <c r="E42" s="57" t="s">
-        <v>121</v>
-      </c>
-      <c r="F42" s="57" t="s">
-        <v>311</v>
-      </c>
-      <c r="G42" s="57" t="s">
-        <v>172</v>
-      </c>
-      <c r="H42" s="64" t="s">
-        <v>314</v>
-      </c>
-      <c r="I42" s="57" t="s">
-        <v>268</v>
-      </c>
-      <c r="J42" s="64" t="s">
-        <v>314</v>
-      </c>
-      <c r="K42" s="57">
+      <c r="C42" s="53" t="s">
+        <v>16</v>
+      </c>
+      <c r="D42" s="54" t="s">
+        <v>57</v>
+      </c>
+      <c r="E42" s="54" t="s">
+        <v>119</v>
+      </c>
+      <c r="F42" s="54" t="s">
+        <v>307</v>
+      </c>
+      <c r="G42" s="54" t="s">
+        <v>170</v>
+      </c>
+      <c r="H42" s="61" t="s">
+        <v>310</v>
+      </c>
+      <c r="I42" s="54" t="s">
+        <v>264</v>
+      </c>
+      <c r="J42" s="61" t="s">
+        <v>310</v>
+      </c>
+      <c r="K42" s="54">
         <v>1</v>
       </c>
-      <c r="L42" s="78">
+      <c r="L42" s="75">
         <f>K42*5</f>
         <v>5</v>
       </c>
-      <c r="M42" s="90" t="s">
-        <v>321</v>
-      </c>
-      <c r="N42" s="83">
+      <c r="M42" s="87" t="s">
+        <v>317</v>
+      </c>
+      <c r="N42" s="80">
         <v>1.6</v>
       </c>
-      <c r="O42" s="72">
+      <c r="O42" s="69">
         <f>N42*L42</f>
         <v>8</v>
       </c>
@@ -3879,48 +3882,48 @@
     </row>
     <row r="43" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A43" s="1"/>
-      <c r="B43" s="52">
+      <c r="B43" s="49">
         <f t="shared" si="0"/>
         <v>34</v>
       </c>
-      <c r="C43" s="53" t="s">
-        <v>18</v>
+      <c r="C43" s="50" t="s">
+        <v>17</v>
       </c>
       <c r="D43" s="31" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="E43" s="31" t="s">
-        <v>122</v>
+        <v>120</v>
       </c>
       <c r="F43" s="30" t="s">
-        <v>311</v>
+        <v>307</v>
       </c>
       <c r="G43" s="31" t="s">
-        <v>217</v>
+        <v>214</v>
       </c>
       <c r="H43" s="31" t="s">
-        <v>314</v>
+        <v>310</v>
       </c>
       <c r="I43" s="31" t="s">
-        <v>269</v>
+        <v>265</v>
       </c>
       <c r="J43" s="31" t="s">
-        <v>293</v>
+        <v>289</v>
       </c>
       <c r="K43" s="31">
         <v>1</v>
       </c>
-      <c r="L43" s="75">
+      <c r="L43" s="72">
         <f t="shared" ref="L43" si="25">K43*5</f>
         <v>5</v>
       </c>
-      <c r="M43" s="90" t="s">
-        <v>321</v>
-      </c>
-      <c r="N43" s="80">
+      <c r="M43" s="87" t="s">
+        <v>317</v>
+      </c>
+      <c r="N43" s="77">
         <v>1.06</v>
       </c>
-      <c r="O43" s="69">
+      <c r="O43" s="66">
         <f t="shared" ref="O43" si="26">N43*L43</f>
         <v>5.3000000000000007</v>
       </c>
@@ -3928,288 +3931,288 @@
     </row>
     <row r="44" spans="1:16" ht="30" x14ac:dyDescent="0.25">
       <c r="A44" s="1"/>
-      <c r="B44" s="49">
+      <c r="B44" s="46">
         <f>ROW(B44) - ROW($B$9)</f>
         <v>35</v>
       </c>
-      <c r="C44" s="53" t="s">
-        <v>18</v>
+      <c r="C44" s="50" t="s">
+        <v>17</v>
       </c>
       <c r="D44" s="30" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="E44" s="30" t="s">
-        <v>123</v>
+        <v>121</v>
       </c>
       <c r="F44" s="30" t="s">
-        <v>311</v>
+        <v>307</v>
       </c>
       <c r="G44" s="30" t="s">
-        <v>218</v>
+        <v>215</v>
       </c>
       <c r="H44" s="30" t="s">
-        <v>314</v>
+        <v>310</v>
       </c>
       <c r="I44" s="30" t="s">
-        <v>270</v>
+        <v>266</v>
       </c>
       <c r="J44" s="30" t="s">
-        <v>294</v>
+        <v>290</v>
       </c>
       <c r="K44" s="30">
         <v>1</v>
       </c>
-      <c r="L44" s="76">
+      <c r="L44" s="73">
         <f>K44*5</f>
         <v>5</v>
       </c>
-      <c r="M44" s="94" t="s">
-        <v>322</v>
-      </c>
-      <c r="N44" s="80" t="s">
-        <v>314</v>
-      </c>
-      <c r="O44" s="69" t="s">
-        <v>314</v>
+      <c r="M44" s="91" t="s">
+        <v>318</v>
+      </c>
+      <c r="N44" s="77" t="s">
+        <v>310</v>
+      </c>
+      <c r="O44" s="66" t="s">
+        <v>310</v>
       </c>
       <c r="P44" s="30"/>
     </row>
     <row r="45" spans="1:16" ht="30" x14ac:dyDescent="0.25">
       <c r="A45" s="1"/>
-      <c r="B45" s="52">
+      <c r="B45" s="49">
         <f t="shared" si="0"/>
         <v>36</v>
       </c>
-      <c r="C45" s="53" t="s">
-        <v>18</v>
+      <c r="C45" s="50" t="s">
+        <v>17</v>
       </c>
       <c r="D45" s="31" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="E45" s="31" t="s">
-        <v>124</v>
+        <v>122</v>
       </c>
       <c r="F45" s="31" t="s">
-        <v>173</v>
+        <v>171</v>
       </c>
       <c r="G45" s="31" t="s">
-        <v>219</v>
+        <v>216</v>
       </c>
       <c r="H45" s="31" t="s">
-        <v>314</v>
+        <v>310</v>
       </c>
       <c r="I45" s="31" t="s">
-        <v>271</v>
+        <v>267</v>
       </c>
       <c r="J45" s="31" t="s">
-        <v>295</v>
+        <v>291</v>
       </c>
       <c r="K45" s="31">
         <v>1</v>
       </c>
-      <c r="L45" s="75">
+      <c r="L45" s="72">
         <f t="shared" ref="L45" si="27">K45*5</f>
         <v>5</v>
       </c>
-      <c r="M45" s="94" t="s">
-        <v>322</v>
-      </c>
-      <c r="N45" s="80" t="s">
-        <v>314</v>
-      </c>
-      <c r="O45" s="69" t="s">
-        <v>314</v>
+      <c r="M45" s="91" t="s">
+        <v>318</v>
+      </c>
+      <c r="N45" s="77" t="s">
+        <v>310</v>
+      </c>
+      <c r="O45" s="66" t="s">
+        <v>310</v>
       </c>
       <c r="P45" s="31"/>
     </row>
     <row r="46" spans="1:16" ht="30" x14ac:dyDescent="0.25">
       <c r="A46" s="1"/>
-      <c r="B46" s="49">
+      <c r="B46" s="46">
         <f>ROW(B46) - ROW($B$9)</f>
         <v>37</v>
       </c>
-      <c r="C46" s="53" t="s">
-        <v>19</v>
+      <c r="C46" s="50" t="s">
+        <v>18</v>
       </c>
       <c r="D46" s="30" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="E46" s="30" t="s">
-        <v>125</v>
+        <v>123</v>
       </c>
       <c r="F46" s="30" t="s">
-        <v>174</v>
+        <v>172</v>
       </c>
       <c r="G46" s="30" t="s">
-        <v>220</v>
+        <v>217</v>
       </c>
       <c r="H46" s="30" t="s">
-        <v>314</v>
+        <v>310</v>
       </c>
       <c r="I46" s="30" t="s">
-        <v>272</v>
+        <v>268</v>
       </c>
       <c r="J46" s="30" t="s">
-        <v>314</v>
+        <v>310</v>
       </c>
       <c r="K46" s="30">
         <v>3</v>
       </c>
-      <c r="L46" s="76">
+      <c r="L46" s="73">
         <f>K46*5</f>
         <v>15</v>
       </c>
-      <c r="M46" s="94" t="s">
-        <v>322</v>
-      </c>
-      <c r="N46" s="80" t="s">
-        <v>314</v>
-      </c>
-      <c r="O46" s="69" t="s">
-        <v>314</v>
+      <c r="M46" s="91" t="s">
+        <v>318</v>
+      </c>
+      <c r="N46" s="77" t="s">
+        <v>310</v>
+      </c>
+      <c r="O46" s="66" t="s">
+        <v>310</v>
       </c>
       <c r="P46" s="30"/>
     </row>
     <row r="47" spans="1:16" ht="30" x14ac:dyDescent="0.25">
       <c r="A47" s="1"/>
-      <c r="B47" s="52">
+      <c r="B47" s="49">
         <f t="shared" si="0"/>
         <v>38</v>
       </c>
-      <c r="C47" s="50" t="s">
-        <v>19</v>
+      <c r="C47" s="47" t="s">
+        <v>18</v>
       </c>
       <c r="D47" s="31" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="E47" s="31" t="s">
-        <v>126</v>
+        <v>124</v>
       </c>
       <c r="F47" s="31" t="s">
-        <v>174</v>
+        <v>172</v>
       </c>
       <c r="G47" s="31" t="s">
-        <v>221</v>
+        <v>218</v>
       </c>
       <c r="H47" s="31" t="s">
-        <v>314</v>
+        <v>310</v>
       </c>
       <c r="I47" s="31" t="s">
-        <v>272</v>
+        <v>268</v>
       </c>
       <c r="J47" s="31" t="s">
-        <v>314</v>
+        <v>310</v>
       </c>
       <c r="K47" s="31">
         <v>1</v>
       </c>
-      <c r="L47" s="75">
+      <c r="L47" s="72">
         <f t="shared" ref="L47" si="28">K47*5</f>
         <v>5</v>
       </c>
-      <c r="M47" s="94" t="s">
-        <v>322</v>
-      </c>
-      <c r="N47" s="80" t="s">
-        <v>314</v>
-      </c>
-      <c r="O47" s="69" t="s">
-        <v>314</v>
+      <c r="M47" s="91" t="s">
+        <v>318</v>
+      </c>
+      <c r="N47" s="77" t="s">
+        <v>310</v>
+      </c>
+      <c r="O47" s="66" t="s">
+        <v>310</v>
       </c>
       <c r="P47" s="31"/>
     </row>
     <row r="48" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A48" s="1"/>
-      <c r="B48" s="49">
+      <c r="B48" s="46">
         <f>ROW(B48) - ROW($B$9)</f>
         <v>39</v>
       </c>
-      <c r="C48" s="53" t="s">
-        <v>312</v>
-      </c>
-      <c r="D48" s="51" t="s">
-        <v>64</v>
-      </c>
-      <c r="E48" s="51" t="s">
-        <v>127</v>
-      </c>
-      <c r="F48" s="51" t="s">
-        <v>311</v>
-      </c>
-      <c r="G48" s="51" t="s">
-        <v>175</v>
-      </c>
-      <c r="H48" s="51" t="s">
-        <v>314</v>
-      </c>
-      <c r="I48" s="51" t="s">
-        <v>314</v>
-      </c>
-      <c r="J48" s="51" t="s">
-        <v>314</v>
-      </c>
-      <c r="K48" s="51">
+      <c r="C48" s="50" t="s">
+        <v>308</v>
+      </c>
+      <c r="D48" s="48" t="s">
+        <v>63</v>
+      </c>
+      <c r="E48" s="48" t="s">
+        <v>125</v>
+      </c>
+      <c r="F48" s="48" t="s">
+        <v>307</v>
+      </c>
+      <c r="G48" s="48" t="s">
+        <v>173</v>
+      </c>
+      <c r="H48" s="48" t="s">
+        <v>310</v>
+      </c>
+      <c r="I48" s="48" t="s">
+        <v>310</v>
+      </c>
+      <c r="J48" s="48" t="s">
+        <v>310</v>
+      </c>
+      <c r="K48" s="48">
         <v>4</v>
       </c>
-      <c r="L48" s="79">
+      <c r="L48" s="76">
         <f>K48*5</f>
         <v>20</v>
       </c>
-      <c r="M48" s="91" t="s">
-        <v>314</v>
-      </c>
-      <c r="N48" s="84" t="s">
-        <v>314</v>
-      </c>
-      <c r="O48" s="66" t="s">
-        <v>314</v>
+      <c r="M48" s="88" t="s">
+        <v>310</v>
+      </c>
+      <c r="N48" s="81" t="s">
+        <v>310</v>
+      </c>
+      <c r="O48" s="63" t="s">
+        <v>310</v>
       </c>
       <c r="P48" s="30"/>
     </row>
     <row r="49" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A49" s="1"/>
-      <c r="B49" s="52">
+      <c r="B49" s="49">
         <f t="shared" si="0"/>
         <v>40</v>
       </c>
-      <c r="C49" s="50" t="s">
-        <v>20</v>
+      <c r="C49" s="47" t="s">
+        <v>19</v>
       </c>
       <c r="D49" s="31" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="E49" s="31" t="s">
-        <v>128</v>
+        <v>126</v>
       </c>
       <c r="F49" s="31" t="s">
-        <v>176</v>
+        <v>174</v>
       </c>
       <c r="G49" s="31" t="s">
-        <v>222</v>
+        <v>219</v>
       </c>
       <c r="H49" s="31" t="s">
-        <v>314</v>
+        <v>310</v>
       </c>
       <c r="I49" s="31" t="s">
-        <v>252</v>
+        <v>249</v>
       </c>
       <c r="J49" s="31" t="s">
-        <v>314</v>
+        <v>310</v>
       </c>
       <c r="K49" s="31">
         <v>6</v>
       </c>
-      <c r="L49" s="75">
+      <c r="L49" s="72">
         <f t="shared" ref="L49" si="29">K49*5</f>
         <v>30</v>
       </c>
-      <c r="M49" s="90" t="s">
-        <v>321</v>
-      </c>
-      <c r="N49" s="80">
+      <c r="M49" s="87" t="s">
+        <v>317</v>
+      </c>
+      <c r="N49" s="77">
         <v>0.125</v>
       </c>
-      <c r="O49" s="69">
+      <c r="O49" s="66">
         <f t="shared" ref="O49" si="30">N49*L49</f>
         <v>3.75</v>
       </c>
@@ -4217,96 +4220,96 @@
     </row>
     <row r="50" spans="1:16" ht="36" x14ac:dyDescent="0.25">
       <c r="A50" s="1"/>
-      <c r="B50" s="49">
+      <c r="B50" s="46">
         <f>ROW(B50) - ROW($B$9)</f>
         <v>41</v>
       </c>
-      <c r="C50" s="53" t="s">
-        <v>20</v>
+      <c r="C50" s="50" t="s">
+        <v>19</v>
       </c>
       <c r="D50" s="30" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="E50" s="30" t="s">
-        <v>129</v>
+        <v>127</v>
       </c>
       <c r="F50" s="30" t="s">
-        <v>163</v>
+        <v>161</v>
       </c>
       <c r="G50" s="30" t="s">
-        <v>223</v>
+        <v>220</v>
       </c>
       <c r="H50" s="30" t="s">
-        <v>314</v>
+        <v>310</v>
       </c>
       <c r="I50" s="30" t="s">
-        <v>256</v>
+        <v>253</v>
       </c>
       <c r="J50" s="30" t="s">
-        <v>314</v>
+        <v>310</v>
       </c>
       <c r="K50" s="30">
         <v>1</v>
       </c>
-      <c r="L50" s="76">
+      <c r="L50" s="73">
         <f>K50*5</f>
         <v>5</v>
       </c>
-      <c r="M50" s="94" t="s">
-        <v>322</v>
-      </c>
-      <c r="N50" s="80" t="s">
-        <v>314</v>
-      </c>
-      <c r="O50" s="69" t="s">
-        <v>314</v>
+      <c r="M50" s="91" t="s">
+        <v>318</v>
+      </c>
+      <c r="N50" s="77" t="s">
+        <v>310</v>
+      </c>
+      <c r="O50" s="66" t="s">
+        <v>310</v>
       </c>
       <c r="P50" s="30"/>
     </row>
     <row r="51" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A51" s="1"/>
-      <c r="B51" s="52">
+      <c r="B51" s="49">
         <f t="shared" si="0"/>
         <v>42</v>
       </c>
-      <c r="C51" s="50" t="s">
-        <v>21</v>
+      <c r="C51" s="47" t="s">
+        <v>20</v>
       </c>
       <c r="D51" s="31" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="E51" s="31" t="s">
-        <v>130</v>
+        <v>128</v>
       </c>
       <c r="F51" s="31" t="s">
-        <v>177</v>
+        <v>175</v>
       </c>
       <c r="G51" s="31" t="s">
-        <v>224</v>
+        <v>221</v>
       </c>
       <c r="H51" s="31" t="s">
-        <v>314</v>
+        <v>310</v>
       </c>
       <c r="I51" s="31" t="s">
-        <v>250</v>
+        <v>247</v>
       </c>
       <c r="J51" s="31" t="s">
-        <v>296</v>
+        <v>292</v>
       </c>
       <c r="K51" s="31">
         <v>1</v>
       </c>
-      <c r="L51" s="75">
+      <c r="L51" s="72">
         <f t="shared" ref="L51" si="31">K51*5</f>
         <v>5</v>
       </c>
-      <c r="M51" s="90" t="s">
-        <v>321</v>
-      </c>
-      <c r="N51" s="80">
+      <c r="M51" s="87" t="s">
+        <v>317</v>
+      </c>
+      <c r="N51" s="77">
         <v>0.1</v>
       </c>
-      <c r="O51" s="69">
+      <c r="O51" s="66">
         <f t="shared" ref="O51" si="32">N51*L51</f>
         <v>0.5</v>
       </c>
@@ -4314,48 +4317,48 @@
     </row>
     <row r="52" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A52" s="1"/>
-      <c r="B52" s="49">
+      <c r="B52" s="46">
         <f>ROW(B52) - ROW($B$9)</f>
         <v>43</v>
       </c>
-      <c r="C52" s="50" t="s">
-        <v>21</v>
+      <c r="C52" s="47" t="s">
+        <v>20</v>
       </c>
       <c r="D52" s="30" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="E52" s="30" t="s">
-        <v>131</v>
+        <v>129</v>
       </c>
       <c r="F52" s="30" t="s">
-        <v>178</v>
-      </c>
-      <c r="G52" s="65" t="s">
-        <v>225</v>
+        <v>176</v>
+      </c>
+      <c r="G52" s="62" t="s">
+        <v>222</v>
       </c>
       <c r="H52" s="31" t="s">
-        <v>314</v>
+        <v>310</v>
       </c>
       <c r="I52" s="31" t="s">
-        <v>250</v>
+        <v>247</v>
       </c>
       <c r="J52" s="31" t="s">
-        <v>297</v>
+        <v>293</v>
       </c>
       <c r="K52" s="30">
         <v>2</v>
       </c>
-      <c r="L52" s="76">
+      <c r="L52" s="73">
         <f>K52*5</f>
         <v>10</v>
       </c>
-      <c r="M52" s="90" t="s">
-        <v>321</v>
-      </c>
-      <c r="N52" s="80">
+      <c r="M52" s="87" t="s">
+        <v>317</v>
+      </c>
+      <c r="N52" s="77">
         <v>0.1</v>
       </c>
-      <c r="O52" s="68">
+      <c r="O52" s="65">
         <f>N52*L52</f>
         <v>1</v>
       </c>
@@ -4363,48 +4366,48 @@
     </row>
     <row r="53" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A53" s="1"/>
-      <c r="B53" s="52">
+      <c r="B53" s="49">
         <f t="shared" si="0"/>
         <v>44</v>
       </c>
-      <c r="C53" s="50" t="s">
-        <v>21</v>
+      <c r="C53" s="47" t="s">
+        <v>20</v>
       </c>
       <c r="D53" s="31" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="E53" s="31" t="s">
-        <v>132</v>
+        <v>130</v>
       </c>
       <c r="F53" s="31" t="s">
-        <v>178</v>
+        <v>176</v>
       </c>
       <c r="G53" s="31" t="s">
-        <v>226</v>
+        <v>223</v>
       </c>
       <c r="H53" s="31" t="s">
-        <v>314</v>
+        <v>310</v>
       </c>
       <c r="I53" s="31" t="s">
-        <v>250</v>
+        <v>247</v>
       </c>
       <c r="J53" s="31" t="s">
-        <v>298</v>
+        <v>294</v>
       </c>
       <c r="K53" s="31">
         <v>6</v>
       </c>
-      <c r="L53" s="75">
+      <c r="L53" s="72">
         <f t="shared" ref="L53" si="33">K53*5</f>
         <v>30</v>
       </c>
-      <c r="M53" s="90" t="s">
-        <v>321</v>
-      </c>
-      <c r="N53" s="80">
+      <c r="M53" s="87" t="s">
+        <v>317</v>
+      </c>
+      <c r="N53" s="77">
         <v>0.1</v>
       </c>
-      <c r="O53" s="69">
+      <c r="O53" s="66">
         <f t="shared" ref="O53" si="34">N53*L53</f>
         <v>3</v>
       </c>
@@ -4412,48 +4415,48 @@
     </row>
     <row r="54" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A54" s="1"/>
-      <c r="B54" s="49">
+      <c r="B54" s="46">
         <f>ROW(B54) - ROW($B$9)</f>
         <v>45</v>
       </c>
-      <c r="C54" s="50" t="s">
-        <v>21</v>
+      <c r="C54" s="47" t="s">
+        <v>20</v>
       </c>
       <c r="D54" s="30" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="E54" s="30" t="s">
-        <v>133</v>
+        <v>131</v>
       </c>
       <c r="F54" s="30" t="s">
-        <v>177</v>
+        <v>175</v>
       </c>
       <c r="G54" s="30" t="s">
-        <v>227</v>
+        <v>224</v>
       </c>
       <c r="H54" s="30" t="s">
-        <v>314</v>
+        <v>310</v>
       </c>
       <c r="I54" s="30" t="s">
-        <v>250</v>
+        <v>247</v>
       </c>
       <c r="J54" s="30" t="s">
-        <v>299</v>
+        <v>295</v>
       </c>
       <c r="K54" s="30">
         <v>1</v>
       </c>
-      <c r="L54" s="76">
+      <c r="L54" s="73">
         <f>K54*5</f>
         <v>5</v>
       </c>
-      <c r="M54" s="90" t="s">
-        <v>321</v>
-      </c>
-      <c r="N54" s="80">
+      <c r="M54" s="87" t="s">
+        <v>317</v>
+      </c>
+      <c r="N54" s="77">
         <v>0.1</v>
       </c>
-      <c r="O54" s="68">
+      <c r="O54" s="65">
         <f>N54*L54</f>
         <v>0.5</v>
       </c>
@@ -4461,48 +4464,48 @@
     </row>
     <row r="55" spans="1:16" ht="24" x14ac:dyDescent="0.25">
       <c r="A55" s="1"/>
-      <c r="B55" s="52">
+      <c r="B55" s="49">
         <f t="shared" si="0"/>
         <v>46</v>
       </c>
-      <c r="C55" s="50" t="s">
-        <v>21</v>
+      <c r="C55" s="47" t="s">
+        <v>20</v>
       </c>
       <c r="D55" s="31" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="E55" s="31" t="s">
-        <v>134</v>
+        <v>132</v>
       </c>
       <c r="F55" s="31" t="s">
-        <v>177</v>
+        <v>175</v>
       </c>
       <c r="G55" s="31" t="s">
-        <v>228</v>
+        <v>225</v>
       </c>
       <c r="H55" s="31" t="s">
-        <v>314</v>
+        <v>310</v>
       </c>
       <c r="I55" s="31" t="s">
-        <v>250</v>
+        <v>247</v>
       </c>
       <c r="J55" s="31" t="s">
-        <v>300</v>
+        <v>296</v>
       </c>
       <c r="K55" s="31">
         <v>17</v>
       </c>
-      <c r="L55" s="75">
+      <c r="L55" s="72">
         <f t="shared" ref="L55" si="35">K55*5</f>
         <v>85</v>
       </c>
-      <c r="M55" s="90" t="s">
-        <v>321</v>
-      </c>
-      <c r="N55" s="80">
+      <c r="M55" s="87" t="s">
+        <v>317</v>
+      </c>
+      <c r="N55" s="77">
         <v>0.1</v>
       </c>
-      <c r="O55" s="69">
+      <c r="O55" s="66">
         <f t="shared" ref="O55" si="36">N55*L55</f>
         <v>8.5</v>
       </c>
@@ -4510,48 +4513,48 @@
     </row>
     <row r="56" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A56" s="1"/>
-      <c r="B56" s="49">
+      <c r="B56" s="46">
         <f>ROW(B56) - ROW($B$9)</f>
         <v>47</v>
       </c>
-      <c r="C56" s="50" t="s">
-        <v>21</v>
+      <c r="C56" s="47" t="s">
+        <v>20</v>
       </c>
       <c r="D56" s="30" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="E56" s="30" t="s">
-        <v>135</v>
+        <v>133</v>
       </c>
       <c r="F56" s="30" t="s">
-        <v>177</v>
+        <v>175</v>
       </c>
       <c r="G56" s="30" t="s">
-        <v>229</v>
+        <v>226</v>
       </c>
       <c r="H56" s="30" t="s">
-        <v>314</v>
+        <v>310</v>
       </c>
       <c r="I56" s="30" t="s">
-        <v>250</v>
+        <v>247</v>
       </c>
       <c r="J56" s="30" t="s">
-        <v>301</v>
+        <v>297</v>
       </c>
       <c r="K56" s="30">
         <v>3</v>
       </c>
-      <c r="L56" s="76">
+      <c r="L56" s="73">
         <f>K56*5</f>
         <v>15</v>
       </c>
-      <c r="M56" s="90" t="s">
-        <v>321</v>
-      </c>
-      <c r="N56" s="81">
+      <c r="M56" s="87" t="s">
+        <v>317</v>
+      </c>
+      <c r="N56" s="78">
         <v>0.1</v>
       </c>
-      <c r="O56" s="68">
+      <c r="O56" s="65">
         <f>N56*L56</f>
         <v>1.5</v>
       </c>
@@ -4559,48 +4562,48 @@
     </row>
     <row r="57" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A57" s="1"/>
-      <c r="B57" s="52">
+      <c r="B57" s="49">
         <f t="shared" si="0"/>
         <v>48</v>
       </c>
-      <c r="C57" s="50" t="s">
-        <v>21</v>
+      <c r="C57" s="47" t="s">
+        <v>20</v>
       </c>
       <c r="D57" s="31" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="E57" s="31" t="s">
-        <v>136</v>
+        <v>134</v>
       </c>
       <c r="F57" s="31" t="s">
-        <v>177</v>
+        <v>175</v>
       </c>
       <c r="G57" s="31" t="s">
-        <v>230</v>
+        <v>227</v>
       </c>
       <c r="H57" s="31" t="s">
-        <v>314</v>
+        <v>310</v>
       </c>
       <c r="I57" s="31" t="s">
-        <v>250</v>
+        <v>247</v>
       </c>
       <c r="J57" s="31" t="s">
-        <v>302</v>
+        <v>298</v>
       </c>
       <c r="K57" s="31">
         <v>1</v>
       </c>
-      <c r="L57" s="75">
+      <c r="L57" s="72">
         <f t="shared" ref="L57" si="37">K57*5</f>
         <v>5</v>
       </c>
-      <c r="M57" s="90" t="s">
-        <v>321</v>
-      </c>
-      <c r="N57" s="80">
+      <c r="M57" s="87" t="s">
+        <v>317</v>
+      </c>
+      <c r="N57" s="77">
         <v>0.1</v>
       </c>
-      <c r="O57" s="69">
+      <c r="O57" s="66">
         <f t="shared" ref="O57" si="38">N57*L57</f>
         <v>0.5</v>
       </c>
@@ -4608,48 +4611,48 @@
     </row>
     <row r="58" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A58" s="1"/>
-      <c r="B58" s="49">
+      <c r="B58" s="46">
         <f>ROW(B58) - ROW($B$9)</f>
         <v>49</v>
       </c>
-      <c r="C58" s="53" t="s">
-        <v>21</v>
+      <c r="C58" s="50" t="s">
+        <v>20</v>
       </c>
       <c r="D58" s="30" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="E58" s="30" t="s">
-        <v>137</v>
+        <v>135</v>
       </c>
       <c r="F58" s="30" t="s">
-        <v>177</v>
+        <v>175</v>
       </c>
       <c r="G58" s="30" t="s">
-        <v>231</v>
+        <v>228</v>
       </c>
       <c r="H58" s="30" t="s">
-        <v>314</v>
+        <v>310</v>
       </c>
       <c r="I58" s="30" t="s">
-        <v>250</v>
+        <v>247</v>
       </c>
       <c r="J58" s="30" t="s">
-        <v>303</v>
+        <v>299</v>
       </c>
       <c r="K58" s="30">
         <v>5</v>
       </c>
-      <c r="L58" s="76">
+      <c r="L58" s="73">
         <f>K58*5</f>
         <v>25</v>
       </c>
-      <c r="M58" s="90" t="s">
-        <v>321</v>
-      </c>
-      <c r="N58" s="80">
+      <c r="M58" s="87" t="s">
+        <v>317</v>
+      </c>
+      <c r="N58" s="77">
         <v>0.1</v>
       </c>
-      <c r="O58" s="68">
+      <c r="O58" s="65">
         <f>N58*L58</f>
         <v>2.5</v>
       </c>
@@ -4657,48 +4660,48 @@
     </row>
     <row r="59" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A59" s="1"/>
-      <c r="B59" s="52">
+      <c r="B59" s="49">
         <f t="shared" si="0"/>
         <v>50</v>
       </c>
-      <c r="C59" s="53" t="s">
-        <v>21</v>
+      <c r="C59" s="50" t="s">
+        <v>20</v>
       </c>
       <c r="D59" s="31" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="E59" s="31" t="s">
-        <v>138</v>
+        <v>136</v>
       </c>
       <c r="F59" s="31" t="s">
-        <v>177</v>
-      </c>
-      <c r="G59" s="65" t="s">
-        <v>232</v>
+        <v>175</v>
+      </c>
+      <c r="G59" s="62" t="s">
+        <v>229</v>
       </c>
       <c r="H59" s="31" t="s">
-        <v>314</v>
+        <v>310</v>
       </c>
       <c r="I59" s="31" t="s">
-        <v>273</v>
+        <v>269</v>
       </c>
       <c r="J59" s="31" t="s">
-        <v>304</v>
+        <v>300</v>
       </c>
       <c r="K59" s="31">
         <v>4</v>
       </c>
-      <c r="L59" s="75">
+      <c r="L59" s="72">
         <f t="shared" ref="L59" si="39">K59*5</f>
         <v>20</v>
       </c>
-      <c r="M59" s="90" t="s">
-        <v>321</v>
-      </c>
-      <c r="N59" s="80">
+      <c r="M59" s="87" t="s">
+        <v>317</v>
+      </c>
+      <c r="N59" s="77">
         <v>0.1</v>
       </c>
-      <c r="O59" s="69">
+      <c r="O59" s="66">
         <f t="shared" ref="O59" si="40">N59*L59</f>
         <v>2</v>
       </c>
@@ -4706,48 +4709,48 @@
     </row>
     <row r="60" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A60" s="1"/>
-      <c r="B60" s="49">
+      <c r="B60" s="46">
         <f>ROW(B60) - ROW($B$9)</f>
         <v>51</v>
       </c>
-      <c r="C60" s="53" t="s">
-        <v>21</v>
+      <c r="C60" s="50" t="s">
+        <v>20</v>
       </c>
       <c r="D60" s="30" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="E60" s="30" t="s">
-        <v>139</v>
+        <v>137</v>
       </c>
       <c r="F60" s="30" t="s">
-        <v>179</v>
+        <v>177</v>
       </c>
       <c r="G60" s="30" t="s">
-        <v>233</v>
+        <v>230</v>
       </c>
       <c r="H60" s="30" t="s">
-        <v>314</v>
+        <v>310</v>
       </c>
       <c r="I60" s="30" t="s">
-        <v>250</v>
+        <v>247</v>
       </c>
       <c r="J60" s="30" t="s">
-        <v>305</v>
+        <v>301</v>
       </c>
       <c r="K60" s="30">
         <v>2</v>
       </c>
-      <c r="L60" s="76">
+      <c r="L60" s="73">
         <f>K60*5</f>
         <v>10</v>
       </c>
-      <c r="M60" s="90" t="s">
-        <v>321</v>
-      </c>
-      <c r="N60" s="80">
+      <c r="M60" s="87" t="s">
+        <v>317</v>
+      </c>
+      <c r="N60" s="77">
         <v>0.1</v>
       </c>
-      <c r="O60" s="68">
+      <c r="O60" s="65">
         <f>N60*L60</f>
         <v>1</v>
       </c>
@@ -4755,48 +4758,48 @@
     </row>
     <row r="61" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A61" s="1"/>
-      <c r="B61" s="52">
+      <c r="B61" s="49">
         <f t="shared" si="0"/>
         <v>52</v>
       </c>
-      <c r="C61" s="50" t="s">
-        <v>21</v>
+      <c r="C61" s="47" t="s">
+        <v>20</v>
       </c>
       <c r="D61" s="31" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="E61" s="31" t="s">
-        <v>140</v>
+        <v>138</v>
       </c>
       <c r="F61" s="31" t="s">
-        <v>311</v>
+        <v>307</v>
       </c>
       <c r="G61" s="31" t="s">
-        <v>234</v>
+        <v>231</v>
       </c>
       <c r="H61" s="31" t="s">
-        <v>314</v>
+        <v>310</v>
       </c>
       <c r="I61" s="31" t="s">
-        <v>250</v>
+        <v>247</v>
       </c>
       <c r="J61" s="31" t="s">
-        <v>306</v>
+        <v>302</v>
       </c>
       <c r="K61" s="31">
         <v>2</v>
       </c>
-      <c r="L61" s="75">
+      <c r="L61" s="72">
         <f t="shared" ref="L61" si="41">K61*5</f>
         <v>10</v>
       </c>
-      <c r="M61" s="90" t="s">
-        <v>321</v>
-      </c>
-      <c r="N61" s="80">
+      <c r="M61" s="87" t="s">
+        <v>317</v>
+      </c>
+      <c r="N61" s="77">
         <v>0.1</v>
       </c>
-      <c r="O61" s="69">
+      <c r="O61" s="66">
         <f t="shared" ref="O61" si="42">N61*L61</f>
         <v>1</v>
       </c>
@@ -4804,48 +4807,48 @@
     </row>
     <row r="62" spans="1:16" ht="24" x14ac:dyDescent="0.25">
       <c r="A62" s="1"/>
-      <c r="B62" s="49">
+      <c r="B62" s="46">
         <f>ROW(B62) - ROW($B$9)</f>
         <v>53</v>
       </c>
-      <c r="C62" s="53" t="s">
-        <v>22</v>
+      <c r="C62" s="50" t="s">
+        <v>21</v>
       </c>
       <c r="D62" s="30" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="E62" s="30" t="s">
-        <v>141</v>
+        <v>139</v>
       </c>
       <c r="F62" s="30" t="s">
-        <v>311</v>
+        <v>307</v>
       </c>
       <c r="G62" s="30" t="s">
-        <v>180</v>
+        <v>178</v>
       </c>
       <c r="H62" s="30" t="s">
-        <v>314</v>
+        <v>310</v>
       </c>
       <c r="I62" s="30" t="s">
-        <v>274</v>
+        <v>270</v>
       </c>
       <c r="J62" s="30" t="s">
-        <v>314</v>
+        <v>310</v>
       </c>
       <c r="K62" s="30">
         <v>1</v>
       </c>
-      <c r="L62" s="76">
+      <c r="L62" s="73">
         <f>K62*5</f>
         <v>5</v>
       </c>
-      <c r="M62" s="90" t="s">
-        <v>321</v>
-      </c>
-      <c r="N62" s="81">
+      <c r="M62" s="87" t="s">
+        <v>317</v>
+      </c>
+      <c r="N62" s="78">
         <v>0.14000000000000001</v>
       </c>
-      <c r="O62" s="68">
+      <c r="O62" s="65">
         <f>N62*L62</f>
         <v>0.70000000000000007</v>
       </c>
@@ -4853,48 +4856,48 @@
     </row>
     <row r="63" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A63" s="1"/>
-      <c r="B63" s="52">
+      <c r="B63" s="49">
         <f t="shared" si="0"/>
         <v>54</v>
       </c>
-      <c r="C63" s="50" t="s">
-        <v>23</v>
+      <c r="C63" s="47" t="s">
+        <v>22</v>
       </c>
       <c r="D63" s="31" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="E63" s="31" t="s">
-        <v>142</v>
+        <v>140</v>
       </c>
       <c r="F63" s="31" t="s">
-        <v>181</v>
+        <v>179</v>
       </c>
       <c r="G63" s="31" t="s">
-        <v>235</v>
+        <v>232</v>
       </c>
       <c r="H63" s="31" t="s">
-        <v>314</v>
+        <v>310</v>
       </c>
       <c r="I63" s="31" t="s">
-        <v>252</v>
+        <v>249</v>
       </c>
       <c r="J63" s="31" t="s">
-        <v>314</v>
+        <v>310</v>
       </c>
       <c r="K63" s="31">
         <v>1</v>
       </c>
-      <c r="L63" s="75">
+      <c r="L63" s="72">
         <f t="shared" ref="L63" si="43">K63*5</f>
         <v>5</v>
       </c>
-      <c r="M63" s="90" t="s">
-        <v>321</v>
-      </c>
-      <c r="N63" s="80">
+      <c r="M63" s="87" t="s">
+        <v>317</v>
+      </c>
+      <c r="N63" s="77">
         <v>0.87</v>
       </c>
-      <c r="O63" s="69">
+      <c r="O63" s="66">
         <f t="shared" ref="O63" si="44">N63*L63</f>
         <v>4.3499999999999996</v>
       </c>
@@ -4902,48 +4905,48 @@
     </row>
     <row r="64" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A64" s="1"/>
-      <c r="B64" s="49">
+      <c r="B64" s="46">
         <f>ROW(B64) - ROW($B$9)</f>
         <v>55</v>
       </c>
-      <c r="C64" s="53" t="s">
-        <v>23</v>
+      <c r="C64" s="50" t="s">
+        <v>22</v>
       </c>
       <c r="D64" s="30" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="E64" s="30" t="s">
-        <v>143</v>
+        <v>141</v>
       </c>
       <c r="F64" s="30" t="s">
-        <v>182</v>
+        <v>180</v>
       </c>
       <c r="G64" s="30" t="s">
-        <v>236</v>
+        <v>233</v>
       </c>
       <c r="H64" s="30" t="s">
-        <v>314</v>
+        <v>310</v>
       </c>
       <c r="I64" s="30" t="s">
-        <v>252</v>
+        <v>249</v>
       </c>
       <c r="J64" s="30" t="s">
-        <v>314</v>
+        <v>310</v>
       </c>
       <c r="K64" s="30">
         <v>1</v>
       </c>
-      <c r="L64" s="76">
+      <c r="L64" s="73">
         <f>K64*5</f>
         <v>5</v>
       </c>
-      <c r="M64" s="90" t="s">
-        <v>321</v>
-      </c>
-      <c r="N64" s="81">
+      <c r="M64" s="87" t="s">
+        <v>317</v>
+      </c>
+      <c r="N64" s="78">
         <v>0.87</v>
       </c>
-      <c r="O64" s="68">
+      <c r="O64" s="65">
         <f>N64*L64</f>
         <v>4.3499999999999996</v>
       </c>
@@ -4951,48 +4954,48 @@
     </row>
     <row r="65" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A65" s="1"/>
-      <c r="B65" s="52">
+      <c r="B65" s="49">
         <f t="shared" si="0"/>
         <v>56</v>
       </c>
-      <c r="C65" s="50" t="s">
-        <v>23</v>
+      <c r="C65" s="47" t="s">
+        <v>22</v>
       </c>
       <c r="D65" s="31" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="E65" s="31" t="s">
-        <v>144</v>
+        <v>142</v>
       </c>
       <c r="F65" s="31" t="s">
-        <v>183</v>
+        <v>181</v>
       </c>
       <c r="G65" s="31" t="s">
-        <v>237</v>
+        <v>234</v>
       </c>
       <c r="H65" s="31" t="s">
-        <v>314</v>
+        <v>310</v>
       </c>
       <c r="I65" s="31" t="s">
-        <v>275</v>
+        <v>271</v>
       </c>
       <c r="J65" s="31" t="s">
-        <v>314</v>
+        <v>310</v>
       </c>
       <c r="K65" s="31">
         <v>1</v>
       </c>
-      <c r="L65" s="75">
+      <c r="L65" s="72">
         <f t="shared" ref="L65" si="45">K65*5</f>
         <v>5</v>
       </c>
-      <c r="M65" s="90" t="s">
-        <v>321</v>
-      </c>
-      <c r="N65" s="80">
+      <c r="M65" s="87" t="s">
+        <v>317</v>
+      </c>
+      <c r="N65" s="77">
         <v>1.1499999999999999</v>
       </c>
-      <c r="O65" s="69">
+      <c r="O65" s="66">
         <f t="shared" ref="O65" si="46">N65*L65</f>
         <v>5.75</v>
       </c>
@@ -5000,48 +5003,48 @@
     </row>
     <row r="66" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A66" s="1"/>
-      <c r="B66" s="49">
+      <c r="B66" s="46">
         <f>ROW(B66) - ROW($B$9)</f>
         <v>57</v>
       </c>
-      <c r="C66" s="53" t="s">
-        <v>23</v>
+      <c r="C66" s="50" t="s">
+        <v>22</v>
       </c>
       <c r="D66" s="30" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="E66" s="30" t="s">
-        <v>145</v>
+        <v>143</v>
       </c>
       <c r="F66" s="30" t="s">
-        <v>184</v>
+        <v>182</v>
       </c>
       <c r="G66" s="30" t="s">
-        <v>238</v>
+        <v>235</v>
       </c>
       <c r="H66" s="30" t="s">
-        <v>314</v>
+        <v>310</v>
       </c>
       <c r="I66" s="30" t="s">
-        <v>276</v>
+        <v>272</v>
       </c>
       <c r="J66" s="30" t="s">
-        <v>314</v>
+        <v>310</v>
       </c>
       <c r="K66" s="30">
         <v>1</v>
       </c>
-      <c r="L66" s="76">
+      <c r="L66" s="73">
         <f>K66*5</f>
         <v>5</v>
       </c>
-      <c r="M66" s="70" t="s">
-        <v>321</v>
-      </c>
-      <c r="N66" s="81">
+      <c r="M66" s="67" t="s">
+        <v>317</v>
+      </c>
+      <c r="N66" s="78">
         <v>2.5099999999999998</v>
       </c>
-      <c r="O66" s="68">
+      <c r="O66" s="65">
         <f>N66*L66</f>
         <v>12.549999999999999</v>
       </c>
@@ -5049,46 +5052,46 @@
     </row>
     <row r="67" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A67" s="1"/>
-      <c r="B67" s="52">
+      <c r="B67" s="49">
         <f t="shared" si="0"/>
         <v>58</v>
       </c>
-      <c r="C67" s="50" t="s">
-        <v>23</v>
+      <c r="C67" s="47" t="s">
+        <v>22</v>
       </c>
       <c r="D67" s="31" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="E67" s="31" t="s">
-        <v>146</v>
+        <v>144</v>
       </c>
       <c r="F67" s="31" t="s">
-        <v>185</v>
+        <v>183</v>
       </c>
       <c r="G67" s="31" t="s">
-        <v>239</v>
+        <v>236</v>
       </c>
       <c r="H67" s="31"/>
       <c r="I67" s="31" t="s">
-        <v>277</v>
+        <v>273</v>
       </c>
       <c r="J67" s="30" t="s">
-        <v>314</v>
+        <v>310</v>
       </c>
       <c r="K67" s="31">
         <v>1</v>
       </c>
-      <c r="L67" s="75">
+      <c r="L67" s="72">
         <f t="shared" ref="L67" si="47">K67*5</f>
         <v>5</v>
       </c>
-      <c r="M67" s="90" t="s">
-        <v>321</v>
-      </c>
-      <c r="N67" s="80">
+      <c r="M67" s="87" t="s">
+        <v>317</v>
+      </c>
+      <c r="N67" s="77">
         <v>0.9</v>
       </c>
-      <c r="O67" s="69">
+      <c r="O67" s="66">
         <f t="shared" ref="O67" si="48">N67*L67</f>
         <v>4.5</v>
       </c>
@@ -5096,144 +5099,144 @@
     </row>
     <row r="68" spans="1:16" ht="30" x14ac:dyDescent="0.25">
       <c r="A68" s="1"/>
-      <c r="B68" s="49">
+      <c r="B68" s="46">
         <f>ROW(B68) - ROW($B$9)</f>
         <v>59</v>
       </c>
-      <c r="C68" s="53" t="s">
-        <v>23</v>
+      <c r="C68" s="50" t="s">
+        <v>22</v>
       </c>
       <c r="D68" s="30" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="E68" s="30" t="s">
-        <v>147</v>
+        <v>145</v>
       </c>
       <c r="F68" s="30" t="s">
-        <v>311</v>
+        <v>307</v>
       </c>
       <c r="G68" s="30" t="s">
-        <v>186</v>
+        <v>184</v>
       </c>
       <c r="H68" s="30" t="s">
-        <v>314</v>
+        <v>310</v>
       </c>
       <c r="I68" s="30" t="s">
-        <v>278</v>
+        <v>274</v>
       </c>
       <c r="J68" s="31" t="s">
-        <v>314</v>
+        <v>310</v>
       </c>
       <c r="K68" s="30">
         <v>1</v>
       </c>
-      <c r="L68" s="76">
+      <c r="L68" s="73">
         <f>K68*5</f>
         <v>5</v>
       </c>
-      <c r="M68" s="94" t="s">
-        <v>322</v>
-      </c>
-      <c r="N68" s="80" t="s">
-        <v>314</v>
-      </c>
-      <c r="O68" s="69" t="s">
-        <v>314</v>
+      <c r="M68" s="91" t="s">
+        <v>318</v>
+      </c>
+      <c r="N68" s="77" t="s">
+        <v>310</v>
+      </c>
+      <c r="O68" s="66" t="s">
+        <v>310</v>
       </c>
       <c r="P68" s="30"/>
     </row>
     <row r="69" spans="1:16" ht="30" x14ac:dyDescent="0.25">
       <c r="A69" s="1"/>
-      <c r="B69" s="52">
+      <c r="B69" s="49">
         <f t="shared" si="0"/>
         <v>60</v>
       </c>
-      <c r="C69" s="50" t="s">
+      <c r="C69" s="47" t="s">
         <v>10</v>
       </c>
       <c r="D69" s="31" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="E69" s="31" t="s">
-        <v>148</v>
+        <v>146</v>
       </c>
       <c r="F69" s="31" t="s">
-        <v>165</v>
+        <v>163</v>
       </c>
       <c r="G69" s="31" t="s">
-        <v>240</v>
+        <v>237</v>
       </c>
       <c r="H69" s="31" t="s">
-        <v>314</v>
+        <v>310</v>
       </c>
       <c r="I69" s="31" t="s">
-        <v>279</v>
+        <v>275</v>
       </c>
       <c r="J69" s="30" t="s">
-        <v>314</v>
+        <v>310</v>
       </c>
       <c r="K69" s="31">
         <v>1</v>
       </c>
-      <c r="L69" s="75">
+      <c r="L69" s="72">
         <f t="shared" ref="L69" si="49">K69*5</f>
         <v>5</v>
       </c>
-      <c r="M69" s="94" t="s">
-        <v>322</v>
-      </c>
-      <c r="N69" s="80" t="s">
-        <v>314</v>
-      </c>
-      <c r="O69" s="69" t="s">
-        <v>314</v>
+      <c r="M69" s="91" t="s">
+        <v>318</v>
+      </c>
+      <c r="N69" s="77" t="s">
+        <v>310</v>
+      </c>
+      <c r="O69" s="66" t="s">
+        <v>310</v>
       </c>
       <c r="P69" s="31"/>
     </row>
     <row r="70" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A70" s="1"/>
-      <c r="B70" s="49">
+      <c r="B70" s="46">
         <f>ROW(B70) - ROW($B$9)</f>
         <v>61</v>
       </c>
-      <c r="C70" s="53" t="s">
-        <v>23</v>
+      <c r="C70" s="50" t="s">
+        <v>22</v>
       </c>
       <c r="D70" s="30" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="E70" s="30" t="s">
-        <v>149</v>
+        <v>147</v>
       </c>
       <c r="F70" s="30" t="s">
-        <v>187</v>
+        <v>185</v>
       </c>
       <c r="G70" s="30" t="s">
-        <v>241</v>
+        <v>238</v>
       </c>
       <c r="H70" s="30" t="s">
-        <v>314</v>
+        <v>310</v>
       </c>
       <c r="I70" s="30" t="s">
-        <v>280</v>
+        <v>276</v>
       </c>
       <c r="J70" s="31" t="s">
-        <v>314</v>
+        <v>310</v>
       </c>
       <c r="K70" s="30">
         <v>1</v>
       </c>
-      <c r="L70" s="76">
+      <c r="L70" s="73">
         <f>K70*5</f>
         <v>5</v>
       </c>
-      <c r="M70" s="90" t="s">
-        <v>321</v>
-      </c>
-      <c r="N70" s="80">
+      <c r="M70" s="87" t="s">
+        <v>317</v>
+      </c>
+      <c r="N70" s="77">
         <v>1.0900000000000001</v>
       </c>
-      <c r="O70" s="68">
+      <c r="O70" s="65">
         <f>N70*L70</f>
         <v>5.45</v>
       </c>
@@ -5241,116 +5244,116 @@
     </row>
     <row r="71" spans="1:16" ht="30" x14ac:dyDescent="0.25">
       <c r="A71" s="1"/>
-      <c r="B71" s="52">
+      <c r="B71" s="49">
         <f t="shared" si="0"/>
         <v>62</v>
       </c>
-      <c r="C71" s="50" t="s">
-        <v>23</v>
+      <c r="C71" s="47" t="s">
+        <v>22</v>
       </c>
       <c r="D71" s="31" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="E71" s="31" t="s">
-        <v>150</v>
+        <v>148</v>
       </c>
       <c r="F71" s="31" t="s">
-        <v>188</v>
+        <v>186</v>
       </c>
       <c r="G71" s="31" t="s">
-        <v>242</v>
+        <v>239</v>
       </c>
       <c r="H71" s="31" t="s">
-        <v>314</v>
+        <v>310</v>
       </c>
       <c r="I71" s="31" t="s">
-        <v>280</v>
+        <v>276</v>
       </c>
       <c r="J71" s="30" t="s">
-        <v>314</v>
+        <v>310</v>
       </c>
       <c r="K71" s="31">
         <v>1</v>
       </c>
-      <c r="L71" s="75">
+      <c r="L71" s="72">
         <f t="shared" ref="L71" si="50">K71*5</f>
         <v>5</v>
       </c>
-      <c r="M71" s="94" t="s">
-        <v>322</v>
-      </c>
-      <c r="N71" s="80" t="s">
-        <v>314</v>
-      </c>
-      <c r="O71" s="69" t="s">
-        <v>314</v>
+      <c r="M71" s="91" t="s">
+        <v>318</v>
+      </c>
+      <c r="N71" s="77" t="s">
+        <v>310</v>
+      </c>
+      <c r="O71" s="66" t="s">
+        <v>310</v>
       </c>
       <c r="P71" s="31"/>
     </row>
     <row r="72" spans="1:16" ht="30.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A72" s="1"/>
-      <c r="B72" s="49">
+      <c r="B72" s="46">
         <f>ROW(B72) - ROW($B$9)</f>
         <v>63</v>
       </c>
-      <c r="C72" s="53" t="s">
-        <v>24</v>
+      <c r="C72" s="50" t="s">
+        <v>23</v>
       </c>
       <c r="D72" s="30" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="E72" s="30" t="s">
-        <v>151</v>
+        <v>149</v>
       </c>
       <c r="F72" s="30" t="s">
-        <v>311</v>
+        <v>307</v>
       </c>
       <c r="G72" s="30" t="s">
-        <v>243</v>
+        <v>240</v>
       </c>
       <c r="H72" s="30" t="s">
-        <v>314</v>
+        <v>310</v>
       </c>
       <c r="I72" s="30" t="s">
-        <v>281</v>
+        <v>277</v>
       </c>
       <c r="J72" s="30" t="s">
-        <v>307</v>
+        <v>303</v>
       </c>
       <c r="K72" s="30">
         <v>1</v>
       </c>
-      <c r="L72" s="76">
+      <c r="L72" s="73">
         <f>K72*5</f>
         <v>5</v>
       </c>
-      <c r="M72" s="94" t="s">
-        <v>322</v>
-      </c>
-      <c r="N72" s="80" t="s">
-        <v>314</v>
-      </c>
-      <c r="O72" s="69" t="s">
-        <v>314</v>
+      <c r="M72" s="91" t="s">
+        <v>318</v>
+      </c>
+      <c r="N72" s="77" t="s">
+        <v>310</v>
+      </c>
+      <c r="O72" s="66" t="s">
+        <v>310</v>
       </c>
       <c r="P72" s="30"/>
     </row>
     <row r="73" spans="1:16" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A73" s="1"/>
-      <c r="B73" s="58"/>
-      <c r="C73" s="59"/>
-      <c r="D73" s="60"/>
-      <c r="E73" s="61"/>
-      <c r="F73" s="62"/>
-      <c r="G73" s="63"/>
-      <c r="H73" s="63"/>
-      <c r="I73" s="62"/>
-      <c r="J73" s="63"/>
-      <c r="K73" s="63"/>
-      <c r="L73" s="63"/>
-      <c r="M73" s="92"/>
-      <c r="N73" s="63"/>
-      <c r="O73" s="73">
+      <c r="B73" s="55"/>
+      <c r="C73" s="56"/>
+      <c r="D73" s="57"/>
+      <c r="E73" s="58"/>
+      <c r="F73" s="59"/>
+      <c r="G73" s="60"/>
+      <c r="H73" s="60"/>
+      <c r="I73" s="59"/>
+      <c r="J73" s="60"/>
+      <c r="K73" s="60"/>
+      <c r="L73" s="60"/>
+      <c r="M73" s="89"/>
+      <c r="N73" s="60"/>
+      <c r="O73" s="70">
         <f>SUM(O10:O72)</f>
         <v>132.06449999999998</v>
       </c>
@@ -5369,9 +5372,9 @@
       <c r="J74" s="9"/>
       <c r="K74" s="9"/>
       <c r="L74" s="9"/>
-      <c r="M74" s="93"/>
+      <c r="M74" s="90"/>
       <c r="N74" s="9"/>
-      <c r="O74" s="74">
+      <c r="O74" s="71">
         <f>O73/5</f>
         <v>26.412899999999997</v>
       </c>

</xml_diff>

<commit_message>
#4 eSpark And Client BOM Peripheral Added
</commit_message>
<xml_diff>
--- a/Design Files/LightSPT-Device-v1.0/BOM/Client_BOM_Light_spt_device.xlsx
+++ b/Design Files/LightSPT-Device-v1.0/BOM/Client_BOM_Light_spt_device.xlsx
@@ -19,7 +19,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="667" uniqueCount="345">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="559" uniqueCount="342">
   <si>
     <t>Component list</t>
   </si>
@@ -942,21 +942,6 @@
     <t>Remarks</t>
   </si>
   <si>
-    <t>Links</t>
-  </si>
-  <si>
-    <t>Unit Cost (5 Boards)</t>
-  </si>
-  <si>
-    <t>Total Cost (5 Boards)</t>
-  </si>
-  <si>
-    <t>Digikey</t>
-  </si>
-  <si>
-    <t>Custom Supplier</t>
-  </si>
-  <si>
     <t>SMA Connector</t>
   </si>
   <si>
@@ -1054,16 +1039,20 @@
   </si>
   <si>
     <t>1.6nH</t>
+  </si>
+  <si>
+    <t>Refrence Link</t>
+  </si>
+  <si>
+    <t>USB Type A to A Cable</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
-  <numFmts count="3">
+  <numFmts count="1">
     <numFmt numFmtId="164" formatCode="[$-409]h:mm:ss\ AM/PM;@"/>
-    <numFmt numFmtId="165" formatCode="&quot;$&quot;#,##0.0000"/>
-    <numFmt numFmtId="166" formatCode="&quot;$&quot;#,##0.00"/>
   </numFmts>
   <fonts count="21" x14ac:knownFonts="1">
     <font>
@@ -1239,7 +1228,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="21">
+  <borders count="17">
     <border>
       <left/>
       <right/>
@@ -1423,60 +1412,12 @@
       </bottom>
       <diagonal/>
     </border>
-    <border>
-      <left/>
-      <right style="medium">
-        <color indexed="64"/>
-      </right>
-      <top/>
-      <bottom style="medium">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="medium">
-        <color indexed="64"/>
-      </left>
-      <right style="medium">
-        <color indexed="64"/>
-      </right>
-      <top/>
-      <bottom style="medium">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right style="medium">
-        <color indexed="64"/>
-      </right>
-      <top style="thin">
-        <color indexed="64"/>
-      </top>
-      <bottom style="thin">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right style="medium">
-        <color indexed="64"/>
-      </right>
-      <top/>
-      <bottom style="thin">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
   </borders>
   <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="20" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="89">
+  <cellXfs count="64">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -1553,11 +1494,6 @@
     <xf numFmtId="0" fontId="6" fillId="3" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="8" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="11" fillId="3" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="top"/>
-      <protection locked="0"/>
-    </xf>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -1639,78 +1575,11 @@
     <xf numFmtId="0" fontId="17" fillId="2" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="165" fontId="19" fillId="2" borderId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="20" fillId="2" borderId="15" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="165" fontId="17" fillId="2" borderId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="10" fillId="4" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="165" fontId="17" fillId="2" borderId="16" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="2" borderId="16" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="165" fontId="19" fillId="2" borderId="16" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="165" fontId="17" fillId="2" borderId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="166" fontId="14" fillId="3" borderId="14" xfId="0" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="166" fontId="14" fillId="3" borderId="18" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="165" fontId="17" fillId="2" borderId="19" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="165" fontId="17" fillId="2" borderId="20" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="165" fontId="19" fillId="2" borderId="19" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="165" fontId="17" fillId="2" borderId="19" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="165" fontId="19" fillId="2" borderId="20" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="4" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="3" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="0" borderId="16" xfId="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="16" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="top"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="0" borderId="16" xfId="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -1720,9 +1589,6 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="4" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -1752,13 +1618,13 @@
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
-      <xdr:col>15</xdr:col>
+      <xdr:col>12</xdr:col>
       <xdr:colOff>47625</xdr:colOff>
       <xdr:row>2</xdr:row>
       <xdr:rowOff>19942</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>15</xdr:col>
+      <xdr:col>12</xdr:col>
       <xdr:colOff>1905000</xdr:colOff>
       <xdr:row>7</xdr:row>
       <xdr:rowOff>171450</xdr:rowOff>
@@ -2066,7 +1932,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <sheetPr codeName="Sheet1"/>
-  <dimension ref="A1:P78"/>
+  <dimension ref="A1:M79"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="3.140625" style="25" customWidth="1"/>
@@ -2080,13 +1946,11 @@
     <col min="10" max="10" width="6.140625" bestFit="1" customWidth="1"/>
     <col min="11" max="11" width="8.7109375" bestFit="1" customWidth="1"/>
     <col min="12" max="12" width="18.28515625" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="8.42578125" style="25" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="18.7109375" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="19.28515625" bestFit="1" customWidth="1"/>
-    <col min="16" max="16" width="29.42578125" customWidth="1"/>
+    <col min="13" max="13" width="29.42578125" customWidth="1"/>
+    <col min="15" max="15" width="25.28515625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:16" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:13" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A1" s="1"/>
       <c r="B1" s="19"/>
       <c r="C1" s="19"/>
@@ -2096,23 +1960,20 @@
       <c r="G1" s="2"/>
       <c r="H1" s="2"/>
       <c r="I1" s="2"/>
-      <c r="J1" s="85"/>
-      <c r="K1" s="85"/>
-      <c r="L1" s="85"/>
-      <c r="M1" s="85"/>
-      <c r="N1" s="85"/>
-      <c r="O1" s="85"/>
-      <c r="P1" s="85"/>
-    </row>
-    <row r="2" spans="1:16" ht="32.25" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="J1" s="61"/>
+      <c r="K1" s="61"/>
+      <c r="L1" s="61"/>
+      <c r="M1" s="61"/>
+    </row>
+    <row r="2" spans="1:13" ht="32.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A2" s="1"/>
       <c r="B2" s="20"/>
-      <c r="C2" s="35"/>
+      <c r="C2" s="33"/>
       <c r="D2" s="10" t="s">
         <v>0</v>
       </c>
       <c r="E2" s="10"/>
-      <c r="F2" s="41" t="s">
+      <c r="F2" s="39" t="s">
         <v>298</v>
       </c>
       <c r="G2" s="11"/>
@@ -2121,20 +1982,17 @@
       <c r="J2" s="3"/>
       <c r="K2" s="3"/>
       <c r="L2" s="3"/>
-      <c r="M2" s="76"/>
-      <c r="N2" s="3"/>
-      <c r="O2" s="3"/>
-      <c r="P2" s="32"/>
-    </row>
-    <row r="3" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="M2" s="32"/>
+    </row>
+    <row r="3" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A3" s="1"/>
       <c r="B3" s="21"/>
-      <c r="C3" s="36"/>
+      <c r="C3" s="34"/>
       <c r="D3" s="12" t="s">
         <v>1</v>
       </c>
       <c r="E3" s="12"/>
-      <c r="F3" s="42" t="s">
+      <c r="F3" s="40" t="s">
         <v>299</v>
       </c>
       <c r="G3" s="12"/>
@@ -2143,20 +2001,17 @@
       <c r="J3" s="4"/>
       <c r="K3" s="4"/>
       <c r="L3" s="4"/>
-      <c r="M3" s="77"/>
-      <c r="N3" s="4"/>
-      <c r="O3" s="4"/>
-      <c r="P3" s="86"/>
-    </row>
-    <row r="4" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="M3" s="62"/>
+    </row>
+    <row r="4" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A4" s="1"/>
       <c r="B4" s="21"/>
-      <c r="C4" s="36"/>
+      <c r="C4" s="34"/>
       <c r="D4" s="12" t="s">
         <v>2</v>
       </c>
       <c r="E4" s="12"/>
-      <c r="F4" s="43" t="s">
+      <c r="F4" s="41" t="s">
         <v>299</v>
       </c>
       <c r="G4" s="13"/>
@@ -2165,20 +2020,17 @@
       <c r="J4" s="6"/>
       <c r="K4" s="6"/>
       <c r="L4" s="6"/>
-      <c r="M4" s="78"/>
-      <c r="N4" s="5"/>
-      <c r="O4" s="5"/>
-      <c r="P4" s="87"/>
-    </row>
-    <row r="5" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="M4" s="63"/>
+    </row>
+    <row r="5" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A5" s="1"/>
       <c r="B5" s="21"/>
-      <c r="C5" s="36"/>
+      <c r="C5" s="34"/>
       <c r="D5" s="12" t="s">
         <v>3</v>
       </c>
       <c r="E5" s="12"/>
-      <c r="F5" s="44" t="s">
+      <c r="F5" s="42" t="s">
         <v>5</v>
       </c>
       <c r="G5" s="14"/>
@@ -2187,15 +2039,12 @@
       <c r="J5" s="5"/>
       <c r="K5" s="5"/>
       <c r="L5" s="5"/>
-      <c r="M5" s="78"/>
-      <c r="N5" s="5"/>
-      <c r="O5" s="5"/>
-      <c r="P5" s="87"/>
-    </row>
-    <row r="6" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="M5" s="63"/>
+    </row>
+    <row r="6" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A6" s="1"/>
       <c r="B6" s="22"/>
-      <c r="C6" s="37"/>
+      <c r="C6" s="35"/>
       <c r="D6" s="15"/>
       <c r="E6" s="15"/>
       <c r="F6" s="16"/>
@@ -2205,15 +2054,12 @@
       <c r="J6" s="5"/>
       <c r="K6" s="5"/>
       <c r="L6" s="5"/>
-      <c r="M6" s="78"/>
-      <c r="N6" s="5"/>
-      <c r="O6" s="5"/>
-      <c r="P6" s="87"/>
-    </row>
-    <row r="7" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="M6" s="63"/>
+    </row>
+    <row r="7" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A7" s="1"/>
       <c r="B7" s="23"/>
-      <c r="C7" s="38"/>
+      <c r="C7" s="36"/>
       <c r="D7" s="17"/>
       <c r="E7" s="17"/>
       <c r="F7" s="18"/>
@@ -2223,15 +2069,12 @@
       <c r="J7" s="7"/>
       <c r="K7" s="7"/>
       <c r="L7" s="7"/>
-      <c r="M7" s="79"/>
-      <c r="N7" s="7"/>
-      <c r="O7" s="7"/>
-      <c r="P7" s="87"/>
-    </row>
-    <row r="8" spans="1:16" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="M7" s="63"/>
+    </row>
+    <row r="8" spans="1:13" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A8" s="1"/>
       <c r="B8" s="26"/>
-      <c r="C8" s="39"/>
+      <c r="C8" s="37"/>
       <c r="D8" s="27"/>
       <c r="E8" s="27"/>
       <c r="F8" s="28"/>
@@ -2241,12 +2084,9 @@
       <c r="J8" s="7"/>
       <c r="K8" s="7"/>
       <c r="L8" s="7"/>
-      <c r="M8" s="79"/>
-      <c r="N8" s="7"/>
-      <c r="O8" s="7"/>
-      <c r="P8" s="87"/>
-    </row>
-    <row r="9" spans="1:16" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="M8" s="63"/>
+    </row>
+    <row r="9" spans="1:13" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A9" s="1"/>
       <c r="B9" s="29" t="s">
         <v>4</v>
@@ -2282,71 +2122,53 @@
         <v>305</v>
       </c>
       <c r="M9" s="29" t="s">
-        <v>307</v>
-      </c>
-      <c r="N9" s="75" t="s">
-        <v>308</v>
-      </c>
-      <c r="O9" s="29" t="s">
-        <v>309</v>
-      </c>
-      <c r="P9" s="29" t="s">
         <v>306</v>
       </c>
     </row>
-    <row r="10" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A10" s="1"/>
-      <c r="B10" s="45">
+      <c r="B10" s="43">
         <f>ROW(B10) - ROW($B$9)</f>
         <v>1</v>
       </c>
-      <c r="C10" s="46" t="s">
+      <c r="C10" s="44" t="s">
         <v>7</v>
       </c>
-      <c r="D10" s="47" t="s">
+      <c r="D10" s="45" t="s">
         <v>25</v>
       </c>
-      <c r="E10" s="47"/>
-      <c r="F10" s="47" t="s">
+      <c r="E10" s="45"/>
+      <c r="F10" s="45" t="s">
         <v>300</v>
       </c>
-      <c r="G10" s="47" t="s">
+      <c r="G10" s="45" t="s">
         <v>147</v>
       </c>
-      <c r="H10" s="47" t="s">
-        <v>303</v>
-      </c>
-      <c r="I10" s="47" t="s">
-        <v>303</v>
-      </c>
-      <c r="J10" s="47" t="s">
-        <v>303</v>
-      </c>
-      <c r="K10" s="47">
+      <c r="H10" s="45" t="s">
+        <v>303</v>
+      </c>
+      <c r="I10" s="45" t="s">
+        <v>303</v>
+      </c>
+      <c r="J10" s="45" t="s">
+        <v>303</v>
+      </c>
+      <c r="K10" s="45">
         <v>1</v>
       </c>
-      <c r="L10" s="47">
+      <c r="L10" s="45">
         <f>K10*5</f>
         <v>5</v>
       </c>
-      <c r="M10" s="47" t="s">
-        <v>303</v>
-      </c>
-      <c r="N10" s="74" t="s">
-        <v>303</v>
-      </c>
-      <c r="O10" s="61" t="s">
-        <v>303</v>
-      </c>
-      <c r="P10" s="30"/>
-    </row>
-    <row r="11" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="M10" s="30"/>
+    </row>
+    <row r="11" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A11" s="1"/>
-      <c r="B11" s="48">
+      <c r="B11" s="46">
         <f t="shared" ref="B11:B74" si="0">ROW(B11) - ROW($B$9)</f>
         <v>2</v>
       </c>
-      <c r="C11" s="46" t="s">
+      <c r="C11" s="44" t="s">
         <v>7</v>
       </c>
       <c r="D11" s="31" t="s">
@@ -2377,25 +2199,15 @@
         <f t="shared" ref="L11" si="1">K11*5</f>
         <v>5</v>
       </c>
-      <c r="M11" s="62" t="s">
-        <v>310</v>
-      </c>
-      <c r="N11" s="71">
-        <v>1.59</v>
-      </c>
-      <c r="O11" s="64">
-        <f t="shared" ref="O11" si="2">N11*L11</f>
-        <v>7.95</v>
-      </c>
-      <c r="P11" s="31"/>
-    </row>
-    <row r="12" spans="1:16" ht="36" x14ac:dyDescent="0.25">
+      <c r="M11" s="31"/>
+    </row>
+    <row r="12" spans="1:13" ht="36" x14ac:dyDescent="0.25">
       <c r="A12" s="1"/>
-      <c r="B12" s="45">
+      <c r="B12" s="43">
         <f>ROW(B12) - ROW($B$9)</f>
         <v>3</v>
       </c>
-      <c r="C12" s="49" t="s">
+      <c r="C12" s="47" t="s">
         <v>8</v>
       </c>
       <c r="D12" s="30" t="s">
@@ -2426,29 +2238,19 @@
         <f>K12*5</f>
         <v>115</v>
       </c>
-      <c r="M12" s="65" t="s">
-        <v>310</v>
-      </c>
-      <c r="N12" s="71">
-        <v>1.03E-2</v>
-      </c>
-      <c r="O12" s="63">
-        <f>N12*L12</f>
-        <v>1.1845000000000001</v>
-      </c>
-      <c r="P12" s="30"/>
-    </row>
-    <row r="13" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="M12" s="30"/>
+    </row>
+    <row r="13" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A13" s="1"/>
-      <c r="B13" s="48">
+      <c r="B13" s="46">
         <f t="shared" si="0"/>
         <v>4</v>
       </c>
-      <c r="C13" s="46" t="s">
+      <c r="C13" s="44" t="s">
         <v>8</v>
       </c>
       <c r="D13" s="30" t="s">
-        <v>317</v>
+        <v>312</v>
       </c>
       <c r="E13" s="31" t="s">
         <v>89</v>
@@ -2472,28 +2274,18 @@
         <v>4</v>
       </c>
       <c r="L13" s="31">
-        <f t="shared" ref="L13" si="3">K13*5</f>
+        <f t="shared" ref="L13" si="2">K13*5</f>
         <v>20</v>
       </c>
-      <c r="M13" s="80" t="s">
-        <v>310</v>
-      </c>
-      <c r="N13" s="70">
-        <v>0.121</v>
-      </c>
-      <c r="O13" s="64">
-        <f t="shared" ref="O13" si="4">N13*L13</f>
-        <v>2.42</v>
-      </c>
-      <c r="P13" s="31"/>
-    </row>
-    <row r="14" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="M13" s="31"/>
+    </row>
+    <row r="14" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A14" s="1"/>
-      <c r="B14" s="45">
+      <c r="B14" s="43">
         <f>ROW(B14) - ROW($B$9)</f>
         <v>5</v>
       </c>
-      <c r="C14" s="46" t="s">
+      <c r="C14" s="44" t="s">
         <v>8</v>
       </c>
       <c r="D14" s="30" t="s">
@@ -2524,25 +2316,15 @@
         <f>K14*5</f>
         <v>5</v>
       </c>
-      <c r="M14" s="80" t="s">
-        <v>310</v>
-      </c>
-      <c r="N14" s="71">
-        <v>0.1</v>
-      </c>
-      <c r="O14" s="63">
-        <f>N14*L14</f>
-        <v>0.5</v>
-      </c>
-      <c r="P14" s="30"/>
-    </row>
-    <row r="15" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="M14" s="30"/>
+    </row>
+    <row r="15" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A15" s="1"/>
-      <c r="B15" s="48">
+      <c r="B15" s="46">
         <f t="shared" si="0"/>
         <v>6</v>
       </c>
-      <c r="C15" s="46" t="s">
+      <c r="C15" s="44" t="s">
         <v>8</v>
       </c>
       <c r="D15" s="31" t="s">
@@ -2568,28 +2350,18 @@
         <v>4</v>
       </c>
       <c r="L15" s="31">
-        <f t="shared" ref="L15" si="5">K15*5</f>
+        <f t="shared" ref="L15" si="3">K15*5</f>
         <v>20</v>
       </c>
-      <c r="M15" s="80" t="s">
-        <v>310</v>
-      </c>
-      <c r="N15" s="70">
-        <v>0.78600000000000003</v>
-      </c>
-      <c r="O15" s="64">
-        <f t="shared" ref="O15" si="6">N15*L15</f>
-        <v>15.72</v>
-      </c>
-      <c r="P15" s="31"/>
-    </row>
-    <row r="16" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="M15" s="31"/>
+    </row>
+    <row r="16" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A16" s="1"/>
-      <c r="B16" s="45">
+      <c r="B16" s="43">
         <f>ROW(B16) - ROW($B$9)</f>
         <v>7</v>
       </c>
-      <c r="C16" s="49" t="s">
+      <c r="C16" s="47" t="s">
         <v>8</v>
       </c>
       <c r="D16" s="30" t="s">
@@ -2601,11 +2373,11 @@
       <c r="F16" s="30" t="s">
         <v>149</v>
       </c>
-      <c r="G16" s="47" t="s">
+      <c r="G16" s="45" t="s">
         <v>188</v>
       </c>
       <c r="H16" s="30" t="s">
-        <v>336</v>
+        <v>331</v>
       </c>
       <c r="I16" s="30" t="s">
         <v>240</v>
@@ -2620,29 +2392,19 @@
         <f>K16*5</f>
         <v>25</v>
       </c>
-      <c r="M16" s="80" t="s">
-        <v>310</v>
-      </c>
-      <c r="N16" s="71">
-        <v>0.161</v>
-      </c>
-      <c r="O16" s="63">
-        <f>N16*L16</f>
-        <v>4.0250000000000004</v>
-      </c>
-      <c r="P16" s="30"/>
-    </row>
-    <row r="17" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="M16" s="30"/>
+    </row>
+    <row r="17" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A17" s="1"/>
-      <c r="B17" s="48">
+      <c r="B17" s="46">
         <f t="shared" si="0"/>
         <v>8</v>
       </c>
-      <c r="C17" s="46" t="s">
+      <c r="C17" s="44" t="s">
         <v>8</v>
       </c>
       <c r="D17" s="31" t="s">
-        <v>318</v>
+        <v>313</v>
       </c>
       <c r="E17" s="31" t="s">
         <v>93</v>
@@ -2666,28 +2428,18 @@
         <v>1</v>
       </c>
       <c r="L17" s="31">
-        <f t="shared" ref="L17" si="7">K17*5</f>
-        <v>5</v>
-      </c>
-      <c r="M17" s="80" t="s">
-        <v>310</v>
-      </c>
-      <c r="N17" s="70">
-        <v>1.6E-2</v>
-      </c>
-      <c r="O17" s="64">
-        <f t="shared" ref="O17" si="8">N17*L17</f>
-        <v>0.08</v>
-      </c>
-      <c r="P17" s="31"/>
-    </row>
-    <row r="18" spans="1:16" x14ac:dyDescent="0.25">
+        <f t="shared" ref="L17" si="4">K17*5</f>
+        <v>5</v>
+      </c>
+      <c r="M17" s="31"/>
+    </row>
+    <row r="18" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A18" s="1"/>
-      <c r="B18" s="45">
+      <c r="B18" s="43">
         <f>ROW(B18) - ROW($B$9)</f>
         <v>9</v>
       </c>
-      <c r="C18" s="49" t="s">
+      <c r="C18" s="47" t="s">
         <v>8</v>
       </c>
       <c r="D18" s="30" t="s">
@@ -2718,25 +2470,15 @@
         <f>K18*5</f>
         <v>25</v>
       </c>
-      <c r="M18" s="80" t="s">
-        <v>310</v>
-      </c>
-      <c r="N18" s="71">
-        <v>1.9E-2</v>
-      </c>
-      <c r="O18" s="63">
-        <f>N18*L18</f>
-        <v>0.47499999999999998</v>
-      </c>
-      <c r="P18" s="30"/>
-    </row>
-    <row r="19" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="M18" s="30"/>
+    </row>
+    <row r="19" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A19" s="1"/>
-      <c r="B19" s="48">
+      <c r="B19" s="46">
         <f t="shared" si="0"/>
         <v>10</v>
       </c>
-      <c r="C19" s="46" t="s">
+      <c r="C19" s="44" t="s">
         <v>8</v>
       </c>
       <c r="D19" s="31" t="s">
@@ -2764,28 +2506,18 @@
         <v>1</v>
       </c>
       <c r="L19" s="31">
-        <f t="shared" ref="L19" si="9">K19*5</f>
-        <v>5</v>
-      </c>
-      <c r="M19" s="80" t="s">
-        <v>310</v>
-      </c>
-      <c r="N19" s="70">
-        <v>0.1</v>
-      </c>
-      <c r="O19" s="64">
-        <f t="shared" ref="O19" si="10">N19*L19</f>
-        <v>0.5</v>
-      </c>
-      <c r="P19" s="31"/>
-    </row>
-    <row r="20" spans="1:16" x14ac:dyDescent="0.25">
+        <f t="shared" ref="L19" si="5">K19*5</f>
+        <v>5</v>
+      </c>
+      <c r="M19" s="31"/>
+    </row>
+    <row r="20" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A20" s="1"/>
-      <c r="B20" s="45">
+      <c r="B20" s="43">
         <f>ROW(B20) - ROW($B$9)</f>
         <v>11</v>
       </c>
-      <c r="C20" s="46" t="s">
+      <c r="C20" s="44" t="s">
         <v>8</v>
       </c>
       <c r="D20" s="30" t="s">
@@ -2816,25 +2548,15 @@
         <f>K20*5</f>
         <v>5</v>
       </c>
-      <c r="M20" s="80" t="s">
-        <v>310</v>
-      </c>
-      <c r="N20" s="71">
-        <v>0.1</v>
-      </c>
-      <c r="O20" s="63">
-        <f>N20*L20</f>
-        <v>0.5</v>
-      </c>
-      <c r="P20" s="30"/>
-    </row>
-    <row r="21" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="M20" s="30"/>
+    </row>
+    <row r="21" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A21" s="1"/>
-      <c r="B21" s="48">
+      <c r="B21" s="46">
         <f t="shared" si="0"/>
         <v>12</v>
       </c>
-      <c r="C21" s="46" t="s">
+      <c r="C21" s="44" t="s">
         <v>8</v>
       </c>
       <c r="D21" s="31" t="s">
@@ -2862,28 +2584,18 @@
         <v>1</v>
       </c>
       <c r="L21" s="31">
-        <f t="shared" ref="L21" si="11">K21*5</f>
-        <v>5</v>
-      </c>
-      <c r="M21" s="80" t="s">
-        <v>310</v>
-      </c>
-      <c r="N21" s="70">
-        <v>0.1</v>
-      </c>
-      <c r="O21" s="64">
-        <f t="shared" ref="O21" si="12">N21*L21</f>
-        <v>0.5</v>
-      </c>
-      <c r="P21" s="31"/>
-    </row>
-    <row r="22" spans="1:16" x14ac:dyDescent="0.25">
+        <f t="shared" ref="L21" si="6">K21*5</f>
+        <v>5</v>
+      </c>
+      <c r="M21" s="31"/>
+    </row>
+    <row r="22" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A22" s="1"/>
-      <c r="B22" s="45">
+      <c r="B22" s="43">
         <f>ROW(B22) - ROW($B$9)</f>
         <v>13</v>
       </c>
-      <c r="C22" s="49" t="s">
+      <c r="C22" s="47" t="s">
         <v>8</v>
       </c>
       <c r="D22" s="30" t="s">
@@ -2914,38 +2626,28 @@
         <f>K22*5</f>
         <v>5</v>
       </c>
-      <c r="M22" s="80" t="s">
-        <v>310</v>
-      </c>
-      <c r="N22" s="71">
-        <v>0.99</v>
-      </c>
-      <c r="O22" s="63">
-        <f>N22*L22</f>
-        <v>4.95</v>
-      </c>
-      <c r="P22" s="30"/>
-    </row>
-    <row r="23" spans="1:16" ht="30" x14ac:dyDescent="0.25">
+      <c r="M22" s="30"/>
+    </row>
+    <row r="23" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A23" s="1"/>
-      <c r="B23" s="45">
+      <c r="B23" s="43">
         <f>ROW(B23) - ROW($B$9)</f>
         <v>14</v>
       </c>
-      <c r="C23" s="49" t="s">
+      <c r="C23" s="47" t="s">
         <v>8</v>
       </c>
       <c r="D23" s="30" t="s">
-        <v>319</v>
+        <v>314</v>
       </c>
       <c r="E23" s="30" t="s">
-        <v>320</v>
+        <v>315</v>
       </c>
       <c r="F23" s="30" t="s">
-        <v>321</v>
+        <v>316</v>
       </c>
       <c r="G23" s="30" t="s">
-        <v>322</v>
+        <v>317</v>
       </c>
       <c r="H23" s="30" t="s">
         <v>303</v>
@@ -2954,7 +2656,7 @@
         <v>241</v>
       </c>
       <c r="J23" s="30" t="s">
-        <v>342</v>
+        <v>337</v>
       </c>
       <c r="K23" s="30">
         <v>1</v>
@@ -2963,37 +2665,28 @@
         <f>K23*5</f>
         <v>5</v>
       </c>
-      <c r="M23" s="84" t="s">
-        <v>311</v>
-      </c>
-      <c r="N23" s="70" t="s">
-        <v>303</v>
-      </c>
-      <c r="O23" s="64" t="s">
-        <v>303</v>
-      </c>
-      <c r="P23" s="31"/>
-    </row>
-    <row r="24" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="M23" s="31"/>
+    </row>
+    <row r="24" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A24" s="1"/>
-      <c r="B24" s="48">
-        <f t="shared" ref="B24" si="13">ROW(B24) - ROW($B$9)</f>
+      <c r="B24" s="46">
+        <f t="shared" ref="B24" si="7">ROW(B24) - ROW($B$9)</f>
         <v>15</v>
       </c>
-      <c r="C24" s="46" t="s">
+      <c r="C24" s="44" t="s">
         <v>8</v>
       </c>
       <c r="D24" s="31" t="s">
-        <v>323</v>
+        <v>318</v>
       </c>
       <c r="E24" s="31" t="s">
-        <v>324</v>
+        <v>319</v>
       </c>
       <c r="F24" s="31" t="s">
-        <v>321</v>
+        <v>316</v>
       </c>
       <c r="G24" s="31" t="s">
-        <v>325</v>
+        <v>320</v>
       </c>
       <c r="H24" s="31" t="s">
         <v>303</v>
@@ -3002,34 +2695,24 @@
         <v>241</v>
       </c>
       <c r="J24" s="31" t="s">
-        <v>343</v>
+        <v>338</v>
       </c>
       <c r="K24" s="31">
         <v>1</v>
       </c>
       <c r="L24" s="31">
-        <f t="shared" ref="L24:L25" si="14">K24*5</f>
-        <v>5</v>
-      </c>
-      <c r="M24" s="80" t="s">
-        <v>310</v>
-      </c>
-      <c r="N24" s="71">
-        <v>0.159</v>
-      </c>
-      <c r="O24" s="63">
-        <f>N24*L24</f>
-        <v>0.79500000000000004</v>
-      </c>
-      <c r="P24" s="30"/>
-    </row>
-    <row r="25" spans="1:16" ht="30" x14ac:dyDescent="0.25">
+        <f t="shared" ref="L24:L25" si="8">K24*5</f>
+        <v>5</v>
+      </c>
+      <c r="M24" s="30"/>
+    </row>
+    <row r="25" spans="1:13" ht="24" x14ac:dyDescent="0.25">
       <c r="A25" s="1"/>
-      <c r="B25" s="48">
+      <c r="B25" s="46">
         <f t="shared" si="0"/>
         <v>16</v>
       </c>
-      <c r="C25" s="46" t="s">
+      <c r="C25" s="44" t="s">
         <v>9</v>
       </c>
       <c r="D25" s="31" t="s">
@@ -3057,27 +2740,18 @@
         <v>1</v>
       </c>
       <c r="L25" s="31">
-        <f t="shared" si="14"/>
-        <v>5</v>
-      </c>
-      <c r="M25" s="84" t="s">
-        <v>311</v>
-      </c>
-      <c r="N25" s="70" t="s">
-        <v>303</v>
-      </c>
-      <c r="O25" s="64" t="s">
-        <v>303</v>
-      </c>
-      <c r="P25" s="31"/>
-    </row>
-    <row r="26" spans="1:16" x14ac:dyDescent="0.25">
+        <f t="shared" si="8"/>
+        <v>5</v>
+      </c>
+      <c r="M25" s="31"/>
+    </row>
+    <row r="26" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A26" s="1"/>
-      <c r="B26" s="45">
+      <c r="B26" s="43">
         <f>ROW(B26) - ROW($B$9)</f>
         <v>17</v>
       </c>
-      <c r="C26" s="49" t="s">
+      <c r="C26" s="47" t="s">
         <v>9</v>
       </c>
       <c r="D26" s="30" t="s">
@@ -3108,25 +2782,15 @@
         <f>K26*5</f>
         <v>10</v>
       </c>
-      <c r="M26" s="80" t="s">
-        <v>310</v>
-      </c>
-      <c r="N26" s="71">
-        <v>0.23</v>
-      </c>
-      <c r="O26" s="63">
-        <f>N26*L26</f>
-        <v>2.3000000000000003</v>
-      </c>
-      <c r="P26" s="30"/>
-    </row>
-    <row r="27" spans="1:16" ht="24" x14ac:dyDescent="0.25">
+      <c r="M26" s="30"/>
+    </row>
+    <row r="27" spans="1:13" ht="24" x14ac:dyDescent="0.25">
       <c r="A27" s="1"/>
-      <c r="B27" s="48">
+      <c r="B27" s="46">
         <f t="shared" si="0"/>
         <v>18</v>
       </c>
-      <c r="C27" s="46" t="s">
+      <c r="C27" s="44" t="s">
         <v>10</v>
       </c>
       <c r="D27" s="31" t="s">
@@ -3154,28 +2818,18 @@
         <v>1</v>
       </c>
       <c r="L27" s="31">
-        <f t="shared" ref="L27" si="15">K27*5</f>
-        <v>5</v>
-      </c>
-      <c r="M27" s="80" t="s">
-        <v>310</v>
-      </c>
-      <c r="N27" s="70">
-        <v>0.44</v>
-      </c>
-      <c r="O27" s="64">
-        <f t="shared" ref="O27" si="16">N27*L27</f>
-        <v>2.2000000000000002</v>
-      </c>
-      <c r="P27" s="31"/>
-    </row>
-    <row r="28" spans="1:16" ht="30" x14ac:dyDescent="0.25">
+        <f t="shared" ref="L27" si="9">K27*5</f>
+        <v>5</v>
+      </c>
+      <c r="M27" s="31"/>
+    </row>
+    <row r="28" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A28" s="1"/>
-      <c r="B28" s="45">
+      <c r="B28" s="43">
         <f>ROW(B28) - ROW($B$9)</f>
         <v>19</v>
       </c>
-      <c r="C28" s="49" t="s">
+      <c r="C28" s="47" t="s">
         <v>9</v>
       </c>
       <c r="D28" s="30" t="s">
@@ -3206,24 +2860,15 @@
         <f>K28*5</f>
         <v>5</v>
       </c>
-      <c r="M28" s="84" t="s">
-        <v>311</v>
-      </c>
-      <c r="N28" s="70" t="s">
-        <v>303</v>
-      </c>
-      <c r="O28" s="64" t="s">
-        <v>303</v>
-      </c>
-      <c r="P28" s="30"/>
-    </row>
-    <row r="29" spans="1:16" ht="30" x14ac:dyDescent="0.25">
+      <c r="M28" s="30"/>
+    </row>
+    <row r="29" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A29" s="1"/>
-      <c r="B29" s="48">
+      <c r="B29" s="46">
         <f t="shared" si="0"/>
         <v>20</v>
       </c>
-      <c r="C29" s="46" t="s">
+      <c r="C29" s="44" t="s">
         <v>9</v>
       </c>
       <c r="D29" s="31" t="s">
@@ -3251,27 +2896,18 @@
         <v>1</v>
       </c>
       <c r="L29" s="31">
-        <f t="shared" ref="L29" si="17">K29*5</f>
-        <v>5</v>
-      </c>
-      <c r="M29" s="84" t="s">
-        <v>311</v>
-      </c>
-      <c r="N29" s="70" t="s">
-        <v>303</v>
-      </c>
-      <c r="O29" s="64" t="s">
-        <v>303</v>
-      </c>
-      <c r="P29" s="31"/>
-    </row>
-    <row r="30" spans="1:16" ht="24" x14ac:dyDescent="0.25">
+        <f t="shared" ref="L29" si="10">K29*5</f>
+        <v>5</v>
+      </c>
+      <c r="M29" s="31"/>
+    </row>
+    <row r="30" spans="1:13" ht="24" x14ac:dyDescent="0.25">
       <c r="A30" s="1"/>
-      <c r="B30" s="45">
+      <c r="B30" s="43">
         <f>ROW(B30) - ROW($B$9)</f>
         <v>21</v>
       </c>
-      <c r="C30" s="49" t="s">
+      <c r="C30" s="47" t="s">
         <v>9</v>
       </c>
       <c r="D30" s="30" t="s">
@@ -3302,25 +2938,15 @@
         <f>K30*5</f>
         <v>5</v>
       </c>
-      <c r="M30" s="80" t="s">
-        <v>310</v>
-      </c>
-      <c r="N30" s="71">
-        <v>0.32300000000000001</v>
-      </c>
-      <c r="O30" s="63">
-        <f>N30*L30</f>
-        <v>1.615</v>
-      </c>
-      <c r="P30" s="30"/>
-    </row>
-    <row r="31" spans="1:16" ht="30" x14ac:dyDescent="0.25">
+      <c r="M30" s="30"/>
+    </row>
+    <row r="31" spans="1:13" ht="24" x14ac:dyDescent="0.25">
       <c r="A31" s="1"/>
-      <c r="B31" s="48">
+      <c r="B31" s="46">
         <f t="shared" si="0"/>
         <v>22</v>
       </c>
-      <c r="C31" s="46" t="s">
+      <c r="C31" s="44" t="s">
         <v>9</v>
       </c>
       <c r="D31" s="31" t="s">
@@ -3348,27 +2974,18 @@
         <v>2</v>
       </c>
       <c r="L31" s="31">
-        <f t="shared" ref="L31" si="18">K31*5</f>
+        <f t="shared" ref="L31" si="11">K31*5</f>
         <v>10</v>
       </c>
-      <c r="M31" s="84" t="s">
-        <v>311</v>
-      </c>
-      <c r="N31" s="70" t="s">
-        <v>303</v>
-      </c>
-      <c r="O31" s="64" t="s">
-        <v>303</v>
-      </c>
-      <c r="P31" s="31"/>
-    </row>
-    <row r="32" spans="1:16" ht="30" x14ac:dyDescent="0.25">
+      <c r="M31" s="31"/>
+    </row>
+    <row r="32" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A32" s="1"/>
-      <c r="B32" s="45">
+      <c r="B32" s="43">
         <f>ROW(B32) - ROW($B$9)</f>
         <v>23</v>
       </c>
-      <c r="C32" s="49" t="s">
+      <c r="C32" s="47" t="s">
         <v>9</v>
       </c>
       <c r="D32" s="30" t="s">
@@ -3397,24 +3014,15 @@
         <f>K32*5</f>
         <v>15</v>
       </c>
-      <c r="M32" s="84" t="s">
-        <v>311</v>
-      </c>
-      <c r="N32" s="70" t="s">
-        <v>303</v>
-      </c>
-      <c r="O32" s="64" t="s">
-        <v>303</v>
-      </c>
-      <c r="P32" s="30"/>
-    </row>
-    <row r="33" spans="1:16" ht="30" x14ac:dyDescent="0.25">
+      <c r="M32" s="30"/>
+    </row>
+    <row r="33" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A33" s="1"/>
-      <c r="B33" s="48">
+      <c r="B33" s="46">
         <f t="shared" si="0"/>
         <v>24</v>
       </c>
-      <c r="C33" s="46" t="s">
+      <c r="C33" s="44" t="s">
         <v>9</v>
       </c>
       <c r="D33" s="31" t="s">
@@ -3442,27 +3050,18 @@
         <v>2</v>
       </c>
       <c r="L33" s="31">
-        <f t="shared" ref="L33" si="19">K33*5</f>
+        <f t="shared" ref="L33" si="12">K33*5</f>
         <v>10</v>
       </c>
-      <c r="M33" s="84" t="s">
-        <v>311</v>
-      </c>
-      <c r="N33" s="70" t="s">
-        <v>303</v>
-      </c>
-      <c r="O33" s="64" t="s">
-        <v>303</v>
-      </c>
-      <c r="P33" s="31"/>
-    </row>
-    <row r="34" spans="1:16" ht="30" x14ac:dyDescent="0.25">
+      <c r="M33" s="31"/>
+    </row>
+    <row r="34" spans="1:13" ht="24" x14ac:dyDescent="0.25">
       <c r="A34" s="1"/>
-      <c r="B34" s="45">
+      <c r="B34" s="43">
         <f>ROW(B34) - ROW($B$9)</f>
         <v>25</v>
       </c>
-      <c r="C34" s="49" t="s">
+      <c r="C34" s="47" t="s">
         <v>11</v>
       </c>
       <c r="D34" s="30" t="s">
@@ -3493,24 +3092,15 @@
         <f>K34*5</f>
         <v>5</v>
       </c>
-      <c r="M34" s="84" t="s">
-        <v>311</v>
-      </c>
-      <c r="N34" s="70" t="s">
-        <v>303</v>
-      </c>
-      <c r="O34" s="64" t="s">
-        <v>303</v>
-      </c>
-      <c r="P34" s="30"/>
-    </row>
-    <row r="35" spans="1:16" ht="30" x14ac:dyDescent="0.25">
+      <c r="M34" s="30"/>
+    </row>
+    <row r="35" spans="1:13" ht="24" x14ac:dyDescent="0.25">
       <c r="A35" s="1"/>
-      <c r="B35" s="48">
+      <c r="B35" s="46">
         <f t="shared" si="0"/>
         <v>26</v>
       </c>
-      <c r="C35" s="46" t="s">
+      <c r="C35" s="44" t="s">
         <v>11</v>
       </c>
       <c r="D35" s="31" t="s">
@@ -3538,27 +3128,18 @@
         <v>1</v>
       </c>
       <c r="L35" s="31">
-        <f t="shared" ref="L35" si="20">K35*5</f>
-        <v>5</v>
-      </c>
-      <c r="M35" s="84" t="s">
-        <v>311</v>
-      </c>
-      <c r="N35" s="70" t="s">
-        <v>303</v>
-      </c>
-      <c r="O35" s="64" t="s">
-        <v>303</v>
-      </c>
-      <c r="P35" s="31"/>
-    </row>
-    <row r="36" spans="1:16" ht="30" x14ac:dyDescent="0.25">
+        <f t="shared" ref="L35" si="13">K35*5</f>
+        <v>5</v>
+      </c>
+      <c r="M35" s="31"/>
+    </row>
+    <row r="36" spans="1:13" ht="24" x14ac:dyDescent="0.25">
       <c r="A36" s="1"/>
-      <c r="B36" s="45">
+      <c r="B36" s="43">
         <f>ROW(B36) - ROW($B$9)</f>
         <v>27</v>
       </c>
-      <c r="C36" s="49" t="s">
+      <c r="C36" s="47" t="s">
         <v>11</v>
       </c>
       <c r="D36" s="30" t="s">
@@ -3589,24 +3170,15 @@
         <f>K36*5</f>
         <v>10</v>
       </c>
-      <c r="M36" s="84" t="s">
-        <v>311</v>
-      </c>
-      <c r="N36" s="70" t="s">
-        <v>303</v>
-      </c>
-      <c r="O36" s="64" t="s">
-        <v>303</v>
-      </c>
-      <c r="P36" s="30"/>
-    </row>
-    <row r="37" spans="1:16" ht="48" x14ac:dyDescent="0.25">
+      <c r="M36" s="30"/>
+    </row>
+    <row r="37" spans="1:13" ht="48" x14ac:dyDescent="0.25">
       <c r="A37" s="1"/>
-      <c r="B37" s="48">
+      <c r="B37" s="46">
         <f t="shared" si="0"/>
         <v>28</v>
       </c>
-      <c r="C37" s="46" t="s">
+      <c r="C37" s="44" t="s">
         <v>12</v>
       </c>
       <c r="D37" s="31" t="s">
@@ -3634,28 +3206,18 @@
         <v>1</v>
       </c>
       <c r="L37" s="31">
-        <f t="shared" ref="L37" si="21">K37*5</f>
-        <v>5</v>
-      </c>
-      <c r="M37" s="80" t="s">
-        <v>310</v>
-      </c>
-      <c r="N37" s="70">
-        <v>1.46</v>
-      </c>
-      <c r="O37" s="64">
-        <f t="shared" ref="O37" si="22">N37*L37</f>
-        <v>7.3</v>
-      </c>
-      <c r="P37" s="31"/>
-    </row>
-    <row r="38" spans="1:16" ht="48" x14ac:dyDescent="0.25">
+        <f t="shared" ref="L37" si="14">K37*5</f>
+        <v>5</v>
+      </c>
+      <c r="M37" s="31"/>
+    </row>
+    <row r="38" spans="1:13" ht="48" x14ac:dyDescent="0.25">
       <c r="A38" s="1"/>
-      <c r="B38" s="45">
+      <c r="B38" s="43">
         <f>ROW(B38) - ROW($B$9)</f>
         <v>29</v>
       </c>
-      <c r="C38" s="49" t="s">
+      <c r="C38" s="47" t="s">
         <v>12</v>
       </c>
       <c r="D38" s="30" t="s">
@@ -3686,43 +3248,34 @@
         <f>K38*5</f>
         <v>25</v>
       </c>
-      <c r="M38" s="84" t="s">
-        <v>311</v>
-      </c>
-      <c r="N38" s="70" t="s">
-        <v>303</v>
-      </c>
-      <c r="O38" s="64" t="s">
-        <v>303</v>
-      </c>
-      <c r="P38" s="30"/>
-    </row>
-    <row r="39" spans="1:16" ht="48" x14ac:dyDescent="0.25">
+      <c r="M38" s="30"/>
+    </row>
+    <row r="39" spans="1:13" ht="48" x14ac:dyDescent="0.25">
       <c r="A39" s="1"/>
-      <c r="B39" s="48">
+      <c r="B39" s="46">
         <f t="shared" si="0"/>
         <v>30</v>
       </c>
-      <c r="C39" s="49" t="s">
+      <c r="C39" s="47" t="s">
         <v>13</v>
       </c>
       <c r="D39" s="31" t="s">
         <v>50</v>
       </c>
       <c r="E39" s="30" t="s">
-        <v>326</v>
+        <v>321</v>
       </c>
       <c r="F39" s="30" t="s">
         <v>300</v>
       </c>
       <c r="G39" s="30" t="s">
-        <v>327</v>
+        <v>322</v>
       </c>
       <c r="H39" s="30" t="s">
         <v>303</v>
       </c>
       <c r="I39" s="30" t="s">
-        <v>339</v>
+        <v>334</v>
       </c>
       <c r="J39" s="30" t="s">
         <v>303</v>
@@ -3734,24 +3287,15 @@
         <f>K39*5</f>
         <v>5</v>
       </c>
-      <c r="M39" s="81" t="s">
-        <v>303</v>
-      </c>
-      <c r="N39" s="72" t="s">
-        <v>303</v>
-      </c>
-      <c r="O39" s="66" t="s">
-        <v>303</v>
-      </c>
-      <c r="P39" s="31"/>
-    </row>
-    <row r="40" spans="1:16" ht="36" x14ac:dyDescent="0.25">
+      <c r="M39" s="31"/>
+    </row>
+    <row r="40" spans="1:13" ht="36" x14ac:dyDescent="0.25">
       <c r="A40" s="1"/>
-      <c r="B40" s="45">
+      <c r="B40" s="43">
         <f>ROW(B40) - ROW($B$9)</f>
         <v>31</v>
       </c>
-      <c r="C40" s="49" t="s">
+      <c r="C40" s="47" t="s">
         <v>13</v>
       </c>
       <c r="D40" s="30" t="s">
@@ -3782,89 +3326,71 @@
         <f>K40*5</f>
         <v>5</v>
       </c>
-      <c r="M40" s="84" t="s">
-        <v>311</v>
-      </c>
-      <c r="N40" s="70" t="s">
-        <v>303</v>
-      </c>
-      <c r="O40" s="64" t="s">
-        <v>303</v>
-      </c>
-      <c r="P40" s="30"/>
-    </row>
-    <row r="41" spans="1:16" ht="30" x14ac:dyDescent="0.25">
+      <c r="M40" s="30"/>
+    </row>
+    <row r="41" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A41" s="1"/>
-      <c r="B41" s="48">
+      <c r="B41" s="46">
         <f t="shared" si="0"/>
         <v>32</v>
       </c>
-      <c r="C41" s="46" t="s">
+      <c r="C41" s="44" t="s">
         <v>14</v>
       </c>
-      <c r="D41" s="50" t="s">
+      <c r="D41" s="48" t="s">
         <v>52</v>
       </c>
-      <c r="E41" s="50" t="s">
+      <c r="E41" s="48" t="s">
         <v>114</v>
       </c>
-      <c r="F41" s="47" t="s">
+      <c r="F41" s="45" t="s">
         <v>300</v>
       </c>
-      <c r="G41" s="50" t="s">
+      <c r="G41" s="48" t="s">
         <v>208</v>
       </c>
-      <c r="H41" s="47" t="s">
-        <v>303</v>
-      </c>
-      <c r="I41" s="47" t="s">
-        <v>303</v>
-      </c>
-      <c r="J41" s="50" t="s">
-        <v>303</v>
-      </c>
-      <c r="K41" s="50">
+      <c r="H41" s="45" t="s">
+        <v>303</v>
+      </c>
+      <c r="I41" s="45" t="s">
+        <v>303</v>
+      </c>
+      <c r="J41" s="48" t="s">
+        <v>303</v>
+      </c>
+      <c r="K41" s="48">
         <v>2</v>
       </c>
-      <c r="L41" s="50">
-        <f t="shared" ref="L41" si="23">K41*5</f>
+      <c r="L41" s="48">
+        <f t="shared" ref="L41" si="15">K41*5</f>
         <v>10</v>
       </c>
-      <c r="M41" s="84" t="s">
-        <v>311</v>
-      </c>
-      <c r="N41" s="70" t="s">
-        <v>303</v>
-      </c>
-      <c r="O41" s="64" t="s">
-        <v>303</v>
-      </c>
-      <c r="P41" s="31"/>
-    </row>
-    <row r="42" spans="1:16" ht="24" x14ac:dyDescent="0.25">
+      <c r="M41" s="31"/>
+    </row>
+    <row r="42" spans="1:13" ht="24" x14ac:dyDescent="0.25">
       <c r="A42" s="1"/>
-      <c r="B42" s="45">
+      <c r="B42" s="43">
         <f>ROW(B42) - ROW($B$9)</f>
         <v>33</v>
       </c>
-      <c r="C42" s="49" t="s">
-        <v>312</v>
+      <c r="C42" s="47" t="s">
+        <v>307</v>
       </c>
       <c r="D42" s="30" t="s">
         <v>53</v>
       </c>
       <c r="E42" s="30" t="s">
-        <v>313</v>
+        <v>308</v>
       </c>
       <c r="F42" s="30" t="s">
-        <v>314</v>
+        <v>309</v>
       </c>
       <c r="G42" s="30" t="s">
-        <v>315</v>
+        <v>310</v>
       </c>
       <c r="H42" s="30"/>
       <c r="I42" s="30" t="s">
-        <v>316</v>
+        <v>311</v>
       </c>
       <c r="J42" s="30" t="s">
         <v>303</v>
@@ -3876,25 +3402,15 @@
         <f>K42*5</f>
         <v>5</v>
       </c>
-      <c r="M42" s="80" t="s">
-        <v>310</v>
-      </c>
-      <c r="N42" s="73">
-        <v>1.6</v>
-      </c>
-      <c r="O42" s="67">
-        <f>N42*L42</f>
-        <v>8</v>
-      </c>
-      <c r="P42" s="30"/>
-    </row>
-    <row r="43" spans="1:16" ht="48" x14ac:dyDescent="0.25">
+      <c r="M42" s="30"/>
+    </row>
+    <row r="43" spans="1:13" ht="48" x14ac:dyDescent="0.25">
       <c r="A43" s="1"/>
-      <c r="B43" s="48">
+      <c r="B43" s="46">
         <f t="shared" si="0"/>
         <v>34</v>
       </c>
-      <c r="C43" s="46" t="s">
+      <c r="C43" s="44" t="s">
         <v>15</v>
       </c>
       <c r="D43" s="31" t="s">
@@ -3922,89 +3438,70 @@
         <v>1</v>
       </c>
       <c r="L43" s="31">
-        <f t="shared" ref="L43" si="24">K43*5</f>
-        <v>5</v>
-      </c>
-      <c r="M43" s="80" t="s">
-        <v>310</v>
-      </c>
-      <c r="N43" s="70">
-        <v>1.06</v>
-      </c>
-      <c r="O43" s="64">
-        <f t="shared" ref="O43" si="25">N43*L43</f>
-        <v>5.3000000000000007</v>
-      </c>
-      <c r="P43" s="31"/>
-    </row>
-    <row r="44" spans="1:16" ht="30" x14ac:dyDescent="0.25">
+        <f t="shared" ref="L43" si="16">K43*5</f>
+        <v>5</v>
+      </c>
+      <c r="M43" s="31"/>
+    </row>
+    <row r="44" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A44" s="1"/>
-      <c r="B44" s="51">
+      <c r="B44" s="49">
         <f>ROW(B44) - ROW($B$9)</f>
         <v>35</v>
       </c>
-      <c r="C44" s="52" t="s">
+      <c r="C44" s="50" t="s">
         <v>16</v>
       </c>
-      <c r="D44" s="53" t="s">
+      <c r="D44" s="51" t="s">
         <v>55</v>
       </c>
-      <c r="E44" s="53" t="s">
+      <c r="E44" s="51" t="s">
         <v>116</v>
       </c>
-      <c r="F44" s="53" t="s">
+      <c r="F44" s="51" t="s">
         <v>300</v>
       </c>
-      <c r="G44" s="53" t="s">
+      <c r="G44" s="51" t="s">
         <v>166</v>
       </c>
-      <c r="H44" s="60" t="s">
-        <v>303</v>
-      </c>
-      <c r="I44" s="53" t="s">
+      <c r="H44" s="58" t="s">
+        <v>303</v>
+      </c>
+      <c r="I44" s="51" t="s">
         <v>257</v>
       </c>
-      <c r="J44" s="60" t="s">
-        <v>303</v>
-      </c>
-      <c r="K44" s="53">
+      <c r="J44" s="58" t="s">
+        <v>303</v>
+      </c>
+      <c r="K44" s="51">
         <v>1</v>
       </c>
-      <c r="L44" s="53">
+      <c r="L44" s="51">
         <f>K44*5</f>
         <v>5</v>
       </c>
-      <c r="M44" s="84" t="s">
-        <v>311</v>
-      </c>
-      <c r="N44" s="70" t="s">
-        <v>303</v>
-      </c>
-      <c r="O44" s="64" t="s">
-        <v>303</v>
-      </c>
-      <c r="P44" s="30"/>
-    </row>
-    <row r="45" spans="1:16" ht="30" x14ac:dyDescent="0.25">
+      <c r="M44" s="30"/>
+    </row>
+    <row r="45" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A45" s="1"/>
-      <c r="B45" s="48">
+      <c r="B45" s="46">
         <f t="shared" si="0"/>
         <v>36</v>
       </c>
-      <c r="C45" s="46" t="s">
+      <c r="C45" s="44" t="s">
         <v>17</v>
       </c>
       <c r="D45" s="31" t="s">
         <v>56</v>
       </c>
       <c r="E45" s="31" t="s">
-        <v>328</v>
+        <v>323</v>
       </c>
       <c r="F45" s="31" t="s">
-        <v>329</v>
+        <v>324</v>
       </c>
       <c r="G45" s="31" t="s">
-        <v>329</v>
+        <v>324</v>
       </c>
       <c r="H45" s="31" t="s">
         <v>303</v>
@@ -4019,27 +3516,18 @@
         <v>1</v>
       </c>
       <c r="L45" s="31">
-        <f t="shared" ref="L45" si="26">K45*5</f>
-        <v>5</v>
-      </c>
-      <c r="M45" s="84" t="s">
-        <v>311</v>
-      </c>
-      <c r="N45" s="70" t="s">
-        <v>303</v>
-      </c>
-      <c r="O45" s="64" t="s">
-        <v>303</v>
-      </c>
-      <c r="P45" s="31"/>
-    </row>
-    <row r="46" spans="1:16" ht="30" x14ac:dyDescent="0.25">
+        <f t="shared" ref="L45" si="17">K45*5</f>
+        <v>5</v>
+      </c>
+      <c r="M45" s="31"/>
+    </row>
+    <row r="46" spans="1:13" ht="24" x14ac:dyDescent="0.25">
       <c r="A46" s="1"/>
-      <c r="B46" s="45">
+      <c r="B46" s="43">
         <f>ROW(B46) - ROW($B$9)</f>
         <v>37</v>
       </c>
-      <c r="C46" s="49" t="s">
+      <c r="C46" s="47" t="s">
         <v>17</v>
       </c>
       <c r="D46" s="30" t="s">
@@ -4070,24 +3558,15 @@
         <f>K46*5</f>
         <v>5</v>
       </c>
-      <c r="M46" s="84" t="s">
-        <v>311</v>
-      </c>
-      <c r="N46" s="70" t="s">
-        <v>303</v>
-      </c>
-      <c r="O46" s="64" t="s">
-        <v>303</v>
-      </c>
-      <c r="P46" s="30"/>
-    </row>
-    <row r="47" spans="1:16" ht="30" x14ac:dyDescent="0.25">
+      <c r="M46" s="30"/>
+    </row>
+    <row r="47" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A47" s="1"/>
-      <c r="B47" s="48">
+      <c r="B47" s="46">
         <f t="shared" si="0"/>
         <v>38</v>
       </c>
-      <c r="C47" s="49" t="s">
+      <c r="C47" s="47" t="s">
         <v>17</v>
       </c>
       <c r="D47" s="31" t="s">
@@ -4115,75 +3594,57 @@
         <v>1</v>
       </c>
       <c r="L47" s="31">
-        <f t="shared" ref="L47:L48" si="27">K47*5</f>
-        <v>5</v>
-      </c>
-      <c r="M47" s="84" t="s">
-        <v>311</v>
-      </c>
-      <c r="N47" s="70" t="s">
-        <v>303</v>
-      </c>
-      <c r="O47" s="64" t="s">
-        <v>303</v>
-      </c>
-      <c r="P47" s="31"/>
-    </row>
-    <row r="48" spans="1:16" ht="24" x14ac:dyDescent="0.25">
+        <f t="shared" ref="L47:L48" si="18">K47*5</f>
+        <v>5</v>
+      </c>
+      <c r="M47" s="31"/>
+    </row>
+    <row r="48" spans="1:13" ht="24" x14ac:dyDescent="0.25">
       <c r="A48" s="1"/>
-      <c r="B48" s="48">
+      <c r="B48" s="46">
         <f t="shared" si="0"/>
         <v>39</v>
       </c>
-      <c r="C48" s="49" t="s">
+      <c r="C48" s="47" t="s">
         <v>17</v>
       </c>
       <c r="D48" s="31" t="s">
-        <v>330</v>
+        <v>325</v>
       </c>
       <c r="E48" s="31" t="s">
-        <v>331</v>
+        <v>326</v>
       </c>
       <c r="F48" s="31" t="s">
         <v>167</v>
       </c>
       <c r="G48" s="31" t="s">
-        <v>332</v>
+        <v>327</v>
       </c>
       <c r="H48" s="31" t="s">
         <v>303</v>
       </c>
       <c r="I48" s="31" t="s">
-        <v>340</v>
+        <v>335</v>
       </c>
       <c r="J48" s="31" t="s">
-        <v>344</v>
+        <v>339</v>
       </c>
       <c r="K48" s="31">
         <v>1</v>
       </c>
       <c r="L48" s="31">
-        <f t="shared" si="27"/>
-        <v>5</v>
-      </c>
-      <c r="M48" s="81" t="s">
-        <v>303</v>
-      </c>
-      <c r="N48" s="74" t="s">
-        <v>303</v>
-      </c>
-      <c r="O48" s="61" t="s">
-        <v>303</v>
-      </c>
-      <c r="P48" s="30"/>
-    </row>
-    <row r="49" spans="1:16" ht="24" x14ac:dyDescent="0.25">
+        <f t="shared" si="18"/>
+        <v>5</v>
+      </c>
+      <c r="M48" s="30"/>
+    </row>
+    <row r="49" spans="1:13" ht="24" x14ac:dyDescent="0.25">
       <c r="A49" s="1"/>
-      <c r="B49" s="45">
+      <c r="B49" s="43">
         <f>ROW(B49) - ROW($B$9)</f>
         <v>40</v>
       </c>
-      <c r="C49" s="49" t="s">
+      <c r="C49" s="47" t="s">
         <v>18</v>
       </c>
       <c r="D49" s="30" t="s">
@@ -4214,25 +3675,15 @@
         <f>K49*5</f>
         <v>15</v>
       </c>
-      <c r="M49" s="80" t="s">
-        <v>310</v>
-      </c>
-      <c r="N49" s="70">
-        <v>0.125</v>
-      </c>
-      <c r="O49" s="64">
-        <f t="shared" ref="O49" si="28">N49*L49</f>
-        <v>1.875</v>
-      </c>
-      <c r="P49" s="31"/>
-    </row>
-    <row r="50" spans="1:16" ht="30" x14ac:dyDescent="0.25">
+      <c r="M49" s="31"/>
+    </row>
+    <row r="50" spans="1:13" ht="24" x14ac:dyDescent="0.25">
       <c r="A50" s="1"/>
-      <c r="B50" s="48">
+      <c r="B50" s="46">
         <f t="shared" si="0"/>
         <v>41</v>
       </c>
-      <c r="C50" s="46" t="s">
+      <c r="C50" s="44" t="s">
         <v>18</v>
       </c>
       <c r="D50" s="31" t="s">
@@ -4260,76 +3711,57 @@
         <v>1</v>
       </c>
       <c r="L50" s="31">
-        <f t="shared" ref="L50" si="29">K50*5</f>
-        <v>5</v>
-      </c>
-      <c r="M50" s="84" t="s">
-        <v>311</v>
-      </c>
-      <c r="N50" s="70" t="s">
-        <v>303</v>
-      </c>
-      <c r="O50" s="64" t="s">
-        <v>303</v>
-      </c>
-      <c r="P50" s="30"/>
-    </row>
-    <row r="51" spans="1:16" x14ac:dyDescent="0.25">
+        <f t="shared" ref="L50" si="19">K50*5</f>
+        <v>5</v>
+      </c>
+      <c r="M50" s="30"/>
+    </row>
+    <row r="51" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A51" s="1"/>
-      <c r="B51" s="45">
+      <c r="B51" s="43">
         <f>ROW(B51) - ROW($B$9)</f>
         <v>42</v>
       </c>
-      <c r="C51" s="49" t="s">
+      <c r="C51" s="47" t="s">
         <v>301</v>
       </c>
-      <c r="D51" s="47" t="s">
+      <c r="D51" s="45" t="s">
         <v>61</v>
       </c>
-      <c r="E51" s="47" t="s">
+      <c r="E51" s="45" t="s">
         <v>121</v>
       </c>
-      <c r="F51" s="47" t="s">
+      <c r="F51" s="45" t="s">
         <v>300</v>
       </c>
-      <c r="G51" s="47" t="s">
+      <c r="G51" s="45" t="s">
         <v>169</v>
       </c>
-      <c r="H51" s="47" t="s">
-        <v>303</v>
-      </c>
-      <c r="I51" s="47" t="s">
-        <v>303</v>
-      </c>
-      <c r="J51" s="47" t="s">
-        <v>303</v>
-      </c>
-      <c r="K51" s="47">
+      <c r="H51" s="45" t="s">
+        <v>303</v>
+      </c>
+      <c r="I51" s="45" t="s">
+        <v>303</v>
+      </c>
+      <c r="J51" s="45" t="s">
+        <v>303</v>
+      </c>
+      <c r="K51" s="45">
         <v>4</v>
       </c>
-      <c r="L51" s="47">
+      <c r="L51" s="45">
         <f>K51*5</f>
         <v>20</v>
       </c>
-      <c r="M51" s="80" t="s">
-        <v>310</v>
-      </c>
-      <c r="N51" s="70">
-        <v>0.1</v>
-      </c>
-      <c r="O51" s="64">
-        <f t="shared" ref="O51" si="30">N51*L51</f>
-        <v>2</v>
-      </c>
-      <c r="P51" s="31"/>
-    </row>
-    <row r="52" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="M51" s="31"/>
+    </row>
+    <row r="52" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A52" s="1"/>
-      <c r="B52" s="48">
+      <c r="B52" s="46">
         <f t="shared" si="0"/>
         <v>43</v>
       </c>
-      <c r="C52" s="46" t="s">
+      <c r="C52" s="44" t="s">
         <v>19</v>
       </c>
       <c r="D52" s="31" t="s">
@@ -4357,28 +3789,18 @@
         <v>6</v>
       </c>
       <c r="L52" s="31">
-        <f t="shared" ref="L52" si="31">K52*5</f>
+        <f t="shared" ref="L52" si="20">K52*5</f>
         <v>30</v>
       </c>
-      <c r="M52" s="80" t="s">
-        <v>310</v>
-      </c>
-      <c r="N52" s="70">
-        <v>0.1</v>
-      </c>
-      <c r="O52" s="63">
-        <f>N52*L52</f>
-        <v>3</v>
-      </c>
-      <c r="P52" s="30"/>
-    </row>
-    <row r="53" spans="1:16" ht="36" x14ac:dyDescent="0.25">
+      <c r="M52" s="30"/>
+    </row>
+    <row r="53" spans="1:13" ht="36" x14ac:dyDescent="0.25">
       <c r="A53" s="1"/>
-      <c r="B53" s="45">
+      <c r="B53" s="43">
         <f>ROW(B53) - ROW($B$9)</f>
         <v>44</v>
       </c>
-      <c r="C53" s="49" t="s">
+      <c r="C53" s="47" t="s">
         <v>19</v>
       </c>
       <c r="D53" s="30" t="s">
@@ -4409,25 +3831,15 @@
         <f>K53*5</f>
         <v>5</v>
       </c>
-      <c r="M53" s="80" t="s">
-        <v>310</v>
-      </c>
-      <c r="N53" s="70">
-        <v>0.1</v>
-      </c>
-      <c r="O53" s="64">
-        <f t="shared" ref="O53" si="32">N53*L53</f>
-        <v>0.5</v>
-      </c>
-      <c r="P53" s="31"/>
-    </row>
-    <row r="54" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="M53" s="31"/>
+    </row>
+    <row r="54" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A54" s="1"/>
-      <c r="B54" s="48">
+      <c r="B54" s="46">
         <f t="shared" si="0"/>
         <v>45</v>
       </c>
-      <c r="C54" s="46" t="s">
+      <c r="C54" s="44" t="s">
         <v>20</v>
       </c>
       <c r="D54" s="31" t="s">
@@ -4455,28 +3867,18 @@
         <v>1</v>
       </c>
       <c r="L54" s="31">
-        <f t="shared" ref="L54" si="33">K54*5</f>
-        <v>5</v>
-      </c>
-      <c r="M54" s="80" t="s">
-        <v>310</v>
-      </c>
-      <c r="N54" s="70">
-        <v>0.1</v>
-      </c>
-      <c r="O54" s="63">
-        <f>N54*L54</f>
-        <v>0.5</v>
-      </c>
-      <c r="P54" s="30"/>
-    </row>
-    <row r="55" spans="1:16" x14ac:dyDescent="0.25">
+        <f t="shared" ref="L54" si="21">K54*5</f>
+        <v>5</v>
+      </c>
+      <c r="M54" s="30"/>
+    </row>
+    <row r="55" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A55" s="1"/>
-      <c r="B55" s="45">
+      <c r="B55" s="43">
         <f>ROW(B55) - ROW($B$9)</f>
         <v>46</v>
       </c>
-      <c r="C55" s="46" t="s">
+      <c r="C55" s="44" t="s">
         <v>20</v>
       </c>
       <c r="D55" s="30" t="s">
@@ -4488,11 +3890,11 @@
       <c r="F55" s="30" t="s">
         <v>172</v>
       </c>
-      <c r="G55" s="47" t="s">
+      <c r="G55" s="45" t="s">
         <v>216</v>
       </c>
       <c r="H55" s="31" t="s">
-        <v>337</v>
+        <v>332</v>
       </c>
       <c r="I55" s="31" t="s">
         <v>241</v>
@@ -4507,25 +3909,15 @@
         <f>K55*5</f>
         <v>10</v>
       </c>
-      <c r="M55" s="80" t="s">
-        <v>310</v>
-      </c>
-      <c r="N55" s="70">
-        <v>0.1</v>
-      </c>
-      <c r="O55" s="64">
-        <f t="shared" ref="O55" si="34">N55*L55</f>
-        <v>1</v>
-      </c>
-      <c r="P55" s="31"/>
-    </row>
-    <row r="56" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="M55" s="31"/>
+    </row>
+    <row r="56" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A56" s="1"/>
-      <c r="B56" s="48">
+      <c r="B56" s="46">
         <f t="shared" si="0"/>
         <v>47</v>
       </c>
-      <c r="C56" s="46" t="s">
+      <c r="C56" s="44" t="s">
         <v>20</v>
       </c>
       <c r="D56" s="31" t="s">
@@ -4553,28 +3945,18 @@
         <v>6</v>
       </c>
       <c r="L56" s="31">
-        <f t="shared" ref="L56" si="35">K56*5</f>
+        <f t="shared" ref="L56" si="22">K56*5</f>
         <v>30</v>
       </c>
-      <c r="M56" s="80" t="s">
-        <v>310</v>
-      </c>
-      <c r="N56" s="71">
-        <v>0.1</v>
-      </c>
-      <c r="O56" s="63">
-        <f>N56*L56</f>
-        <v>3</v>
-      </c>
-      <c r="P56" s="30"/>
-    </row>
-    <row r="57" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="M56" s="30"/>
+    </row>
+    <row r="57" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A57" s="1"/>
-      <c r="B57" s="45">
+      <c r="B57" s="43">
         <f>ROW(B57) - ROW($B$9)</f>
         <v>48</v>
       </c>
-      <c r="C57" s="46" t="s">
+      <c r="C57" s="44" t="s">
         <v>20</v>
       </c>
       <c r="D57" s="30" t="s">
@@ -4605,25 +3987,15 @@
         <f>K57*5</f>
         <v>5</v>
       </c>
-      <c r="M57" s="80" t="s">
-        <v>310</v>
-      </c>
-      <c r="N57" s="70">
-        <v>0.1</v>
-      </c>
-      <c r="O57" s="64">
-        <f t="shared" ref="O57" si="36">N57*L57</f>
-        <v>0.5</v>
-      </c>
-      <c r="P57" s="31"/>
-    </row>
-    <row r="58" spans="1:16" ht="24" x14ac:dyDescent="0.25">
+      <c r="M57" s="31"/>
+    </row>
+    <row r="58" spans="1:13" ht="24" x14ac:dyDescent="0.25">
       <c r="A58" s="1"/>
-      <c r="B58" s="48">
+      <c r="B58" s="46">
         <f t="shared" si="0"/>
         <v>49</v>
       </c>
-      <c r="C58" s="46" t="s">
+      <c r="C58" s="44" t="s">
         <v>20</v>
       </c>
       <c r="D58" s="31" t="s">
@@ -4651,28 +4023,18 @@
         <v>17</v>
       </c>
       <c r="L58" s="31">
-        <f t="shared" ref="L58" si="37">K58*5</f>
+        <f t="shared" ref="L58" si="23">K58*5</f>
         <v>85</v>
       </c>
-      <c r="M58" s="80" t="s">
-        <v>310</v>
-      </c>
-      <c r="N58" s="70">
-        <v>0.1</v>
-      </c>
-      <c r="O58" s="63">
-        <f>N58*L58</f>
-        <v>8.5</v>
-      </c>
-      <c r="P58" s="30"/>
-    </row>
-    <row r="59" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="M58" s="30"/>
+    </row>
+    <row r="59" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A59" s="1"/>
-      <c r="B59" s="45">
+      <c r="B59" s="43">
         <f>ROW(B59) - ROW($B$9)</f>
         <v>50</v>
       </c>
-      <c r="C59" s="46" t="s">
+      <c r="C59" s="44" t="s">
         <v>20</v>
       </c>
       <c r="D59" s="30" t="s">
@@ -4703,25 +4065,15 @@
         <f>K59*5</f>
         <v>15</v>
       </c>
-      <c r="M59" s="80" t="s">
-        <v>310</v>
-      </c>
-      <c r="N59" s="70">
-        <v>0.1</v>
-      </c>
-      <c r="O59" s="64">
-        <f t="shared" ref="O59" si="38">N59*L59</f>
-        <v>1.5</v>
-      </c>
-      <c r="P59" s="31"/>
-    </row>
-    <row r="60" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="M59" s="31"/>
+    </row>
+    <row r="60" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A60" s="1"/>
-      <c r="B60" s="48">
+      <c r="B60" s="46">
         <f t="shared" si="0"/>
         <v>51</v>
       </c>
-      <c r="C60" s="46" t="s">
+      <c r="C60" s="44" t="s">
         <v>20</v>
       </c>
       <c r="D60" s="31" t="s">
@@ -4749,28 +4101,18 @@
         <v>1</v>
       </c>
       <c r="L60" s="31">
-        <f t="shared" ref="L60" si="39">K60*5</f>
-        <v>5</v>
-      </c>
-      <c r="M60" s="80" t="s">
-        <v>310</v>
-      </c>
-      <c r="N60" s="70">
-        <v>0.1</v>
-      </c>
-      <c r="O60" s="63">
-        <f>N60*L60</f>
-        <v>0.5</v>
-      </c>
-      <c r="P60" s="30"/>
-    </row>
-    <row r="61" spans="1:16" x14ac:dyDescent="0.25">
+        <f t="shared" ref="L60" si="24">K60*5</f>
+        <v>5</v>
+      </c>
+      <c r="M60" s="30"/>
+    </row>
+    <row r="61" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A61" s="1"/>
-      <c r="B61" s="45">
+      <c r="B61" s="43">
         <f>ROW(B61) - ROW($B$9)</f>
         <v>52</v>
       </c>
-      <c r="C61" s="49" t="s">
+      <c r="C61" s="47" t="s">
         <v>20</v>
       </c>
       <c r="D61" s="30" t="s">
@@ -4801,25 +4143,15 @@
         <f>K61*5</f>
         <v>25</v>
       </c>
-      <c r="M61" s="80" t="s">
-        <v>310</v>
-      </c>
-      <c r="N61" s="70">
-        <v>0.1</v>
-      </c>
-      <c r="O61" s="64">
-        <f t="shared" ref="O61" si="40">N61*L61</f>
-        <v>2.5</v>
-      </c>
-      <c r="P61" s="31"/>
-    </row>
-    <row r="62" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="M61" s="31"/>
+    </row>
+    <row r="62" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A62" s="1"/>
-      <c r="B62" s="48">
+      <c r="B62" s="46">
         <f t="shared" si="0"/>
         <v>53</v>
       </c>
-      <c r="C62" s="49" t="s">
+      <c r="C62" s="47" t="s">
         <v>20</v>
       </c>
       <c r="D62" s="31" t="s">
@@ -4831,11 +4163,11 @@
       <c r="F62" s="31" t="s">
         <v>171</v>
       </c>
-      <c r="G62" s="47" t="s">
+      <c r="G62" s="45" t="s">
         <v>223</v>
       </c>
       <c r="H62" s="31" t="s">
-        <v>338</v>
+        <v>333</v>
       </c>
       <c r="I62" s="31" t="s">
         <v>262</v>
@@ -4847,28 +4179,18 @@
         <v>4</v>
       </c>
       <c r="L62" s="31">
-        <f t="shared" ref="L62" si="41">K62*5</f>
+        <f t="shared" ref="L62" si="25">K62*5</f>
         <v>20</v>
       </c>
-      <c r="M62" s="80" t="s">
-        <v>310</v>
-      </c>
-      <c r="N62" s="71">
-        <v>0.14000000000000001</v>
-      </c>
-      <c r="O62" s="63">
-        <f>N62*L62</f>
-        <v>2.8000000000000003</v>
-      </c>
-      <c r="P62" s="30"/>
-    </row>
-    <row r="63" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="M62" s="30"/>
+    </row>
+    <row r="63" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A63" s="1"/>
-      <c r="B63" s="45">
+      <c r="B63" s="43">
         <f>ROW(B63) - ROW($B$9)</f>
         <v>54</v>
       </c>
-      <c r="C63" s="49" t="s">
+      <c r="C63" s="47" t="s">
         <v>20</v>
       </c>
       <c r="D63" s="30" t="s">
@@ -4899,25 +4221,15 @@
         <f>K63*5</f>
         <v>10</v>
       </c>
-      <c r="M63" s="80" t="s">
-        <v>310</v>
-      </c>
-      <c r="N63" s="70">
-        <v>0.87</v>
-      </c>
-      <c r="O63" s="64">
-        <f t="shared" ref="O63" si="42">N63*L63</f>
-        <v>8.6999999999999993</v>
-      </c>
-      <c r="P63" s="31"/>
-    </row>
-    <row r="64" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="M63" s="31"/>
+    </row>
+    <row r="64" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A64" s="1"/>
-      <c r="B64" s="48">
+      <c r="B64" s="46">
         <f t="shared" si="0"/>
         <v>55</v>
       </c>
-      <c r="C64" s="46" t="s">
+      <c r="C64" s="44" t="s">
         <v>20</v>
       </c>
       <c r="D64" s="31" t="s">
@@ -4945,28 +4257,18 @@
         <v>2</v>
       </c>
       <c r="L64" s="31">
-        <f t="shared" ref="L64" si="43">K64*5</f>
+        <f t="shared" ref="L64" si="26">K64*5</f>
         <v>10</v>
       </c>
-      <c r="M64" s="80" t="s">
-        <v>310</v>
-      </c>
-      <c r="N64" s="71">
-        <v>0.87</v>
-      </c>
-      <c r="O64" s="63">
-        <f>N64*L64</f>
-        <v>8.6999999999999993</v>
-      </c>
-      <c r="P64" s="30"/>
-    </row>
-    <row r="65" spans="1:16" ht="24" x14ac:dyDescent="0.25">
+      <c r="M64" s="30"/>
+    </row>
+    <row r="65" spans="1:13" ht="24" x14ac:dyDescent="0.25">
       <c r="A65" s="1"/>
-      <c r="B65" s="45">
+      <c r="B65" s="43">
         <f>ROW(B65) - ROW($B$9)</f>
         <v>56</v>
       </c>
-      <c r="C65" s="49" t="s">
+      <c r="C65" s="47" t="s">
         <v>21</v>
       </c>
       <c r="D65" s="30" t="s">
@@ -4997,25 +4299,15 @@
         <f>K65*5</f>
         <v>5</v>
       </c>
-      <c r="M65" s="80" t="s">
-        <v>310</v>
-      </c>
-      <c r="N65" s="70">
-        <v>1.1499999999999999</v>
-      </c>
-      <c r="O65" s="64">
-        <f t="shared" ref="O65" si="44">N65*L65</f>
-        <v>5.75</v>
-      </c>
-      <c r="P65" s="31"/>
-    </row>
-    <row r="66" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="M65" s="31"/>
+    </row>
+    <row r="66" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A66" s="1"/>
-      <c r="B66" s="48">
+      <c r="B66" s="46">
         <f t="shared" si="0"/>
         <v>57</v>
       </c>
-      <c r="C66" s="46" t="s">
+      <c r="C66" s="44" t="s">
         <v>22</v>
       </c>
       <c r="D66" s="31" t="s">
@@ -5043,28 +4335,18 @@
         <v>1</v>
       </c>
       <c r="L66" s="31">
-        <f t="shared" ref="L66" si="45">K66*5</f>
-        <v>5</v>
-      </c>
-      <c r="M66" s="65" t="s">
-        <v>310</v>
-      </c>
-      <c r="N66" s="71">
-        <v>2.5099999999999998</v>
-      </c>
-      <c r="O66" s="63">
-        <f>N66*L66</f>
-        <v>12.549999999999999</v>
-      </c>
-      <c r="P66" s="30"/>
-    </row>
-    <row r="67" spans="1:16" x14ac:dyDescent="0.25">
+        <f t="shared" ref="L66" si="27">K66*5</f>
+        <v>5</v>
+      </c>
+      <c r="M66" s="30"/>
+    </row>
+    <row r="67" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A67" s="1"/>
-      <c r="B67" s="45">
+      <c r="B67" s="43">
         <f>ROW(B67) - ROW($B$9)</f>
         <v>58</v>
       </c>
-      <c r="C67" s="49" t="s">
+      <c r="C67" s="47" t="s">
         <v>22</v>
       </c>
       <c r="D67" s="30" t="s">
@@ -5095,25 +4377,15 @@
         <f>K67*5</f>
         <v>5</v>
       </c>
-      <c r="M67" s="80" t="s">
-        <v>310</v>
-      </c>
-      <c r="N67" s="70">
-        <v>0.9</v>
-      </c>
-      <c r="O67" s="64">
-        <f t="shared" ref="O67" si="46">N67*L67</f>
-        <v>4.5</v>
-      </c>
-      <c r="P67" s="31"/>
-    </row>
-    <row r="68" spans="1:16" ht="30" x14ac:dyDescent="0.25">
+      <c r="M67" s="31"/>
+    </row>
+    <row r="68" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A68" s="1"/>
-      <c r="B68" s="48">
+      <c r="B68" s="46">
         <f t="shared" si="0"/>
         <v>59</v>
       </c>
-      <c r="C68" s="46" t="s">
+      <c r="C68" s="44" t="s">
         <v>22</v>
       </c>
       <c r="D68" s="31" t="s">
@@ -5141,27 +4413,18 @@
         <v>1</v>
       </c>
       <c r="L68" s="31">
-        <f t="shared" ref="L68" si="47">K68*5</f>
-        <v>5</v>
-      </c>
-      <c r="M68" s="84" t="s">
-        <v>311</v>
-      </c>
-      <c r="N68" s="70" t="s">
-        <v>303</v>
-      </c>
-      <c r="O68" s="64" t="s">
-        <v>303</v>
-      </c>
-      <c r="P68" s="30"/>
-    </row>
-    <row r="69" spans="1:16" ht="30" x14ac:dyDescent="0.25">
+        <f t="shared" ref="L68" si="28">K68*5</f>
+        <v>5</v>
+      </c>
+      <c r="M68" s="30"/>
+    </row>
+    <row r="69" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A69" s="1"/>
-      <c r="B69" s="45">
+      <c r="B69" s="43">
         <f>ROW(B69) - ROW($B$9)</f>
         <v>60</v>
       </c>
-      <c r="C69" s="49" t="s">
+      <c r="C69" s="47" t="s">
         <v>22</v>
       </c>
       <c r="D69" s="30" t="s">
@@ -5192,24 +4455,15 @@
         <f>K69*5</f>
         <v>5</v>
       </c>
-      <c r="M69" s="84" t="s">
-        <v>311</v>
-      </c>
-      <c r="N69" s="70" t="s">
-        <v>303</v>
-      </c>
-      <c r="O69" s="64" t="s">
-        <v>303</v>
-      </c>
-      <c r="P69" s="31"/>
-    </row>
-    <row r="70" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="M69" s="31"/>
+    </row>
+    <row r="70" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A70" s="1"/>
-      <c r="B70" s="48">
+      <c r="B70" s="46">
         <f t="shared" si="0"/>
         <v>61</v>
       </c>
-      <c r="C70" s="46" t="s">
+      <c r="C70" s="44" t="s">
         <v>22</v>
       </c>
       <c r="D70" s="31" t="s">
@@ -5235,28 +4489,18 @@
         <v>1</v>
       </c>
       <c r="L70" s="31">
-        <f t="shared" ref="L70" si="48">K70*5</f>
-        <v>5</v>
-      </c>
-      <c r="M70" s="80" t="s">
-        <v>310</v>
-      </c>
-      <c r="N70" s="70">
-        <v>1.0900000000000001</v>
-      </c>
-      <c r="O70" s="63">
-        <f>N70*L70</f>
-        <v>5.45</v>
-      </c>
-      <c r="P70" s="30"/>
-    </row>
-    <row r="71" spans="1:16" ht="30" x14ac:dyDescent="0.25">
+        <f t="shared" ref="L70" si="29">K70*5</f>
+        <v>5</v>
+      </c>
+      <c r="M70" s="30"/>
+    </row>
+    <row r="71" spans="1:13" ht="24" x14ac:dyDescent="0.25">
       <c r="A71" s="1"/>
-      <c r="B71" s="45">
+      <c r="B71" s="43">
         <f>ROW(B71) - ROW($B$9)</f>
         <v>62</v>
       </c>
-      <c r="C71" s="49" t="s">
+      <c r="C71" s="47" t="s">
         <v>22</v>
       </c>
       <c r="D71" s="30" t="s">
@@ -5287,24 +4531,15 @@
         <f>K71*5</f>
         <v>5</v>
       </c>
-      <c r="M71" s="84" t="s">
-        <v>311</v>
-      </c>
-      <c r="N71" s="70" t="s">
-        <v>303</v>
-      </c>
-      <c r="O71" s="64" t="s">
-        <v>303</v>
-      </c>
-      <c r="P71" s="31"/>
-    </row>
-    <row r="72" spans="1:16" ht="30.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="M71" s="31"/>
+    </row>
+    <row r="72" spans="1:13" ht="24" x14ac:dyDescent="0.25">
       <c r="A72" s="1"/>
-      <c r="B72" s="48">
+      <c r="B72" s="46">
         <f t="shared" si="0"/>
         <v>63</v>
       </c>
-      <c r="C72" s="46" t="s">
+      <c r="C72" s="44" t="s">
         <v>10</v>
       </c>
       <c r="D72" s="31" t="s">
@@ -5332,27 +4567,18 @@
         <v>1</v>
       </c>
       <c r="L72" s="31">
-        <f t="shared" ref="L72" si="49">K72*5</f>
-        <v>5</v>
-      </c>
-      <c r="M72" s="84" t="s">
-        <v>311</v>
-      </c>
-      <c r="N72" s="70" t="s">
-        <v>303</v>
-      </c>
-      <c r="O72" s="64" t="s">
-        <v>303</v>
-      </c>
-      <c r="P72" s="30"/>
-    </row>
-    <row r="73" spans="1:16" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
+        <f t="shared" ref="L72" si="30">K72*5</f>
+        <v>5</v>
+      </c>
+      <c r="M72" s="30"/>
+    </row>
+    <row r="73" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A73" s="1"/>
-      <c r="B73" s="45">
+      <c r="B73" s="43">
         <f>ROW(B73) - ROW($B$9)</f>
         <v>64</v>
       </c>
-      <c r="C73" s="49" t="s">
+      <c r="C73" s="47" t="s">
         <v>22</v>
       </c>
       <c r="D73" s="30" t="s">
@@ -5383,21 +4609,15 @@
         <f>K73*5</f>
         <v>5</v>
       </c>
-      <c r="M73" s="82"/>
-      <c r="N73" s="59"/>
-      <c r="O73" s="68">
-        <f>SUM(O10:O72)</f>
-        <v>140.1395</v>
-      </c>
-      <c r="P73" s="33"/>
-    </row>
-    <row r="74" spans="1:16" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="M73" s="30"/>
+    </row>
+    <row r="74" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A74" s="1"/>
-      <c r="B74" s="48">
+      <c r="B74" s="46">
         <f t="shared" si="0"/>
         <v>65</v>
       </c>
-      <c r="C74" s="46" t="s">
+      <c r="C74" s="44" t="s">
         <v>22</v>
       </c>
       <c r="D74" s="31" t="s">
@@ -5425,23 +4645,17 @@
         <v>1</v>
       </c>
       <c r="L74" s="31">
-        <f t="shared" ref="L74" si="50">K74*5</f>
-        <v>5</v>
-      </c>
-      <c r="M74" s="83"/>
-      <c r="N74" s="9"/>
-      <c r="O74" s="69">
-        <f>O73/5</f>
-        <v>28.027899999999999</v>
-      </c>
-      <c r="P74" s="34"/>
-    </row>
-    <row r="75" spans="1:16" ht="24" x14ac:dyDescent="0.25">
-      <c r="B75" s="45">
+        <f t="shared" ref="L74" si="31">K74*5</f>
+        <v>5</v>
+      </c>
+      <c r="M74" s="30"/>
+    </row>
+    <row r="75" spans="1:13" ht="24" x14ac:dyDescent="0.25">
+      <c r="B75" s="43">
         <f>ROW(B75) - ROW($B$9)</f>
         <v>66</v>
       </c>
-      <c r="C75" s="49" t="s">
+      <c r="C75" s="47" t="s">
         <v>23</v>
       </c>
       <c r="D75" s="30" t="s">
@@ -5472,31 +4686,32 @@
         <f>K75*5</f>
         <v>5</v>
       </c>
-    </row>
-    <row r="76" spans="1:16" ht="24" x14ac:dyDescent="0.25">
-      <c r="B76" s="88">
+      <c r="M75" s="30"/>
+    </row>
+    <row r="76" spans="1:13" ht="24" x14ac:dyDescent="0.25">
+      <c r="B76" s="60">
         <v>67</v>
       </c>
-      <c r="C76" s="46" t="s">
-        <v>333</v>
+      <c r="C76" s="44" t="s">
+        <v>328</v>
       </c>
       <c r="D76" s="31" t="s">
         <v>303</v>
       </c>
       <c r="E76" s="31" t="s">
-        <v>334</v>
+        <v>329</v>
       </c>
       <c r="F76" s="31" t="s">
         <v>303</v>
       </c>
       <c r="G76" s="31" t="s">
-        <v>335</v>
+        <v>330</v>
       </c>
       <c r="H76" s="31" t="s">
         <v>303</v>
       </c>
       <c r="I76" s="31" t="s">
-        <v>341</v>
+        <v>336</v>
       </c>
       <c r="J76" s="30" t="s">
         <v>303</v>
@@ -5508,80 +4723,83 @@
         <f>K76*5</f>
         <v>5</v>
       </c>
-    </row>
-    <row r="77" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="B77" s="54"/>
-      <c r="C77" s="55"/>
-      <c r="D77" s="56"/>
-      <c r="E77" s="57"/>
-      <c r="F77" s="58"/>
-      <c r="G77" s="59"/>
-      <c r="H77" s="59"/>
-      <c r="I77" s="58"/>
-      <c r="J77" s="59"/>
-      <c r="K77" s="59"/>
-      <c r="L77" s="59"/>
-    </row>
-    <row r="78" spans="1:16" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B78" s="24"/>
-      <c r="C78" s="40"/>
-      <c r="D78" s="8"/>
-      <c r="E78" s="9"/>
-      <c r="F78" s="9"/>
-      <c r="G78" s="9"/>
-      <c r="H78" s="9"/>
-      <c r="I78" s="9"/>
-      <c r="J78" s="9"/>
-      <c r="K78" s="9"/>
-      <c r="L78" s="9"/>
+      <c r="M76" s="30"/>
+    </row>
+    <row r="77" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="B77" s="60">
+        <v>68</v>
+      </c>
+      <c r="C77" s="44" t="s">
+        <v>328</v>
+      </c>
+      <c r="D77" s="31" t="s">
+        <v>303</v>
+      </c>
+      <c r="E77" s="31"/>
+      <c r="F77" s="31" t="s">
+        <v>303</v>
+      </c>
+      <c r="G77" s="31" t="s">
+        <v>341</v>
+      </c>
+      <c r="H77" s="31" t="s">
+        <v>303</v>
+      </c>
+      <c r="I77" s="31" t="s">
+        <v>303</v>
+      </c>
+      <c r="J77" s="30" t="s">
+        <v>303</v>
+      </c>
+      <c r="K77" s="31">
+        <v>1</v>
+      </c>
+      <c r="L77" s="31">
+        <f>K77*5</f>
+        <v>5</v>
+      </c>
+      <c r="M77" s="59" t="s">
+        <v>340</v>
+      </c>
+    </row>
+    <row r="78" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="B78" s="52"/>
+      <c r="C78" s="53"/>
+      <c r="D78" s="54"/>
+      <c r="E78" s="55"/>
+      <c r="F78" s="56"/>
+      <c r="G78" s="57"/>
+      <c r="H78" s="57"/>
+      <c r="I78" s="56"/>
+      <c r="J78" s="57"/>
+      <c r="K78" s="57"/>
+      <c r="L78" s="57"/>
+      <c r="M78" s="57"/>
+    </row>
+    <row r="79" spans="1:13" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B79" s="24"/>
+      <c r="C79" s="38"/>
+      <c r="D79" s="8"/>
+      <c r="E79" s="9"/>
+      <c r="F79" s="9"/>
+      <c r="G79" s="9"/>
+      <c r="H79" s="9"/>
+      <c r="I79" s="9"/>
+      <c r="J79" s="9"/>
+      <c r="K79" s="9"/>
+      <c r="L79" s="9"/>
+      <c r="M79" s="9"/>
     </row>
   </sheetData>
   <mergeCells count="2">
-    <mergeCell ref="J1:P1"/>
-    <mergeCell ref="P3:P8"/>
+    <mergeCell ref="J1:M1"/>
+    <mergeCell ref="M3:M8"/>
   </mergeCells>
   <hyperlinks>
-    <hyperlink ref="M70" r:id="rId1"/>
-    <hyperlink ref="M67" r:id="rId2"/>
-    <hyperlink ref="M65" r:id="rId3"/>
-    <hyperlink ref="M64" r:id="rId4"/>
-    <hyperlink ref="M63" r:id="rId5"/>
-    <hyperlink ref="M62" r:id="rId6"/>
-    <hyperlink ref="M61" r:id="rId7"/>
-    <hyperlink ref="M60" r:id="rId8"/>
-    <hyperlink ref="M59" r:id="rId9"/>
-    <hyperlink ref="M58" r:id="rId10"/>
-    <hyperlink ref="M57" r:id="rId11"/>
-    <hyperlink ref="M56" r:id="rId12"/>
-    <hyperlink ref="M55" r:id="rId13"/>
-    <hyperlink ref="M54" r:id="rId14"/>
-    <hyperlink ref="M53" r:id="rId15"/>
-    <hyperlink ref="M52" r:id="rId16"/>
-    <hyperlink ref="M51" r:id="rId17"/>
-    <hyperlink ref="M49" r:id="rId18"/>
-    <hyperlink ref="M43" r:id="rId19"/>
-    <hyperlink ref="M42" r:id="rId20"/>
-    <hyperlink ref="M37" r:id="rId21"/>
-    <hyperlink ref="M30" r:id="rId22"/>
-    <hyperlink ref="M27" r:id="rId23"/>
-    <hyperlink ref="M26" r:id="rId24"/>
-    <hyperlink ref="M24" r:id="rId25"/>
-    <hyperlink ref="M22" r:id="rId26"/>
-    <hyperlink ref="M21" r:id="rId27"/>
-    <hyperlink ref="M20" r:id="rId28"/>
-    <hyperlink ref="M19" r:id="rId29"/>
-    <hyperlink ref="M18" r:id="rId30"/>
-    <hyperlink ref="M17" r:id="rId31"/>
-    <hyperlink ref="M16" r:id="rId32"/>
-    <hyperlink ref="M15" r:id="rId33"/>
-    <hyperlink ref="M14" r:id="rId34"/>
-    <hyperlink ref="M13" r:id="rId35"/>
-    <hyperlink ref="M12" r:id="rId36"/>
-    <hyperlink ref="M11" r:id="rId37"/>
-    <hyperlink ref="M66" r:id="rId38"/>
+    <hyperlink ref="M77" r:id="rId1"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" orientation="portrait" r:id="rId39"/>
-  <drawing r:id="rId40"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId2"/>
+  <drawing r:id="rId3"/>
 </worksheet>
 </file>
</xml_diff>